<commit_message>
feat: generate 9:16 720p keyframe images for all 245 segments categorized into track directories
</commit_message>
<xml_diff>
--- a/docs/Album1_Dance_Production_Spec.xlsx
+++ b/docs/Album1_Dance_Production_Spec.xlsx
@@ -29,7 +29,7 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <numFmts count="0"/>
-  <fonts count="9">
+  <fonts count="12">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
@@ -83,8 +83,25 @@
       <color rgb="00334155"/>
       <sz val="10"/>
     </font>
+    <font>
+      <name val="Microsoft JhengHei"/>
+      <b val="1"/>
+      <color rgb="000F766E"/>
+      <sz val="9"/>
+    </font>
+    <font>
+      <name val="Microsoft JhengHei"/>
+      <b val="1"/>
+      <color rgb="001E293B"/>
+      <sz val="9"/>
+    </font>
+    <font>
+      <name val="Microsoft JhengHei"/>
+      <color rgb="00334155"/>
+      <sz val="9"/>
+    </font>
   </fonts>
-  <fills count="7">
+  <fills count="8">
     <fill>
       <patternFill/>
     </fill>
@@ -119,6 +136,12 @@
       <patternFill patternType="solid">
         <fgColor rgb="004F46E5"/>
         <bgColor rgb="004F46E5"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="000D9488"/>
+        <bgColor rgb="000D9488"/>
       </patternFill>
     </fill>
   </fills>
@@ -162,7 +185,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="19">
+  <cellXfs count="26">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
@@ -217,6 +240,27 @@
     </xf>
     <xf numFmtId="0" fontId="8" fillId="0" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="7" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="9" fillId="0" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="6" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="10" fillId="0" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="11" fillId="0" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="11" fillId="0" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="10" fillId="0" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -1023,7 +1067,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J28"/>
+  <dimension ref="A1:K28"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="18" customWidth="1" min="1" max="1"/>
@@ -1036,6 +1080,7 @@
     <col width="30" customWidth="1" min="8" max="8"/>
     <col width="12" customWidth="1" min="9" max="9"/>
     <col width="55" customWidth="1" min="10" max="10"/>
+    <col width="34" customWidth="1" min="11" max="11"/>
   </cols>
   <sheetData>
     <row r="1" ht="32" customHeight="1">
@@ -1096,6 +1141,11 @@
           <t>AI 影片動畫生成提示詞 (Prompt)</t>
         </is>
       </c>
+      <c r="K2" s="19" t="inlineStr">
+        <is>
+          <t>首張圖片路徑 (9:16 720p)</t>
+        </is>
+      </c>
     </row>
     <row r="3" ht="30" customHeight="1">
       <c r="A3" s="10" t="inlineStr">
@@ -1144,6 +1194,11 @@
           <t>3D Pixar Disney style preschool animation video keyframe, vertical 9:16 aspect ratio 720p HD. Full body standing shot of the cheerful 5-year-old girl dance coach with brown curly pigtails tied with yellow ribbons, pink dance tee with smiling yellow star, yellow shorts, pink sneakers. In colorful kindergarten dance studio. Starter keyframe for action "[前奏] 蒸汽火車汽笛響起" (🚂 嗚嗚！拉響火車汽笛，ABC 字母列車準備開動！). The character is in lively dance starter pose, joyful radiant beaming smile, sparkling expressive eyes. 4k 3D Pixar render, clean frame without text overlay, starter keyframe for image-to-video generation (a1_s07_seg01_girl.jpg).</t>
         </is>
       </c>
+      <c r="K3" s="20" t="inlineStr">
+        <is>
+          <t>images/track_07/a1_s07_seg01_girl.jpg</t>
+        </is>
+      </c>
     </row>
     <row r="4" ht="30" customHeight="1">
       <c r="A4" s="8" t="inlineStr">
@@ -1192,6 +1247,11 @@
           <t>3D Pixar Disney style cheerful toddler dance coach, smooth playful animation, vibrant kindergarten studio, soft bright volumetric lighting, clean studio background, highly expressive face, full body dynamic camera shot: Song 'The Magic ABC Train', Action '第 01 節: ABC 列車全員上車'. 🎫 揮手招呼大家快上車，踩著節拍小碎步！. The character is waving both hands overhead in friendly wide arcs, swaying gently from side to side, sparkling excited eyes. 4k resolution, 60fps, Disney Pixar render, joyful preschool music video style.</t>
         </is>
       </c>
+      <c r="K4" s="20" t="inlineStr">
+        <is>
+          <t>images/track_07/a1_s07_seg02_girl.jpg</t>
+        </is>
+      </c>
     </row>
     <row r="5" ht="30" customHeight="1">
       <c r="A5" s="10" t="inlineStr">
@@ -1240,6 +1300,11 @@
           <t>3D Pixar Disney style cheerful toddler dance coach, smooth playful animation, vibrant kindergarten studio, soft bright volumetric lighting, clean studio background, highly expressive face, full body dynamic camera shot: Song 'The Magic ABC Train', Action '第 02 節: A 是蘋果 B 是皮球'. 🍎 右手比圓圓大蘋果，左手拍拍小皮球！. The character is stretching arms up high to reach floating elements, standing on tiptoes, joyful posture, looking up with wonder. 4k resolution, 60fps, Disney Pixar render, joyful preschool music video style.</t>
         </is>
       </c>
+      <c r="K5" s="20" t="inlineStr">
+        <is>
+          <t>images/track_07/a1_s07_seg03_girl.jpg</t>
+        </is>
+      </c>
     </row>
     <row r="6" ht="30" customHeight="1">
       <c r="A6" s="8" t="inlineStr">
@@ -1288,6 +1353,11 @@
           <t>3D Pixar Disney style cheerful toddler dance coach, smooth playful animation, vibrant kindergarten studio, soft bright volumetric lighting, clean studio background, highly expressive face, full body dynamic camera shot: Song 'The Magic ABC Train', Action '第 03 節: C 是小貓爬上牆'. 🐱 雙手像貓咪爪爪，交替向上抓抓爬牆！. The character is stretching arms up high to reach floating elements, standing on tiptoes, joyful posture, looking up with wonder. 4k resolution, 60fps, Disney Pixar render, joyful preschool music video style.</t>
         </is>
       </c>
+      <c r="K6" s="20" t="inlineStr">
+        <is>
+          <t>images/track_07/a1_s07_seg04_girl.jpg</t>
+        </is>
+      </c>
     </row>
     <row r="7" ht="30" customHeight="1">
       <c r="A7" s="10" t="inlineStr">
@@ -1336,6 +1406,11 @@
           <t>3D Pixar Disney style cheerful toddler dance coach, smooth playful animation, vibrant kindergarten studio, soft bright volumetric lighting, clean studio background, highly expressive face, full body dynamic camera shot: Song 'The Magic ABC Train', Action '第 04 節: D 是小狗 E 是大象'. 🐘 雙手放耳朵搖搖，雙手做長長大象鼻！. The character is swaying hips and arms like a breeze, smooth fluid body roll, playful rhythmic dancing, friendly warm smile. 4k resolution, 60fps, Disney Pixar render, joyful preschool music video style.</t>
         </is>
       </c>
+      <c r="K7" s="20" t="inlineStr">
+        <is>
+          <t>images/track_07/a1_s07_seg05_girl.jpg</t>
+        </is>
+      </c>
     </row>
     <row r="8" ht="30" customHeight="1">
       <c r="A8" s="8" t="inlineStr">
@@ -1384,6 +1459,11 @@
           <t>3D Pixar Disney style cheerful toddler dance coach, smooth playful animation, vibrant kindergarten studio, soft bright volumetric lighting, clean studio background, highly expressive face, full body dynamic camera shot: Song 'The Magic ABC Train', Action '第 05 節: F 是小魚游向前'. 🐟 雙手合十左右擺動，像小魚游水！. The character is waving both hands overhead in friendly wide arcs, swaying gently from side to side, sparkling excited eyes. 4k resolution, 60fps, Disney Pixar render, joyful preschool music video style.</t>
         </is>
       </c>
+      <c r="K8" s="20" t="inlineStr">
+        <is>
+          <t>images/track_07/a1_s07_seg06_girl.jpg</t>
+        </is>
+      </c>
     </row>
     <row r="9" ht="30" customHeight="1">
       <c r="A9" s="10" t="inlineStr">
@@ -1432,6 +1512,11 @@
           <t>3D Pixar Disney style cheerful toddler dance coach, smooth playful animation, vibrant kindergarten studio, soft bright volumetric lighting, clean studio background, highly expressive face, full body dynamic camera shot: Song 'The Magic ABC Train', Action '第 06 節: G H I J K L 六字母'. 🔢 伸出手指跟著節拍有節奏地點一點！. The character is marching in place energetically, hands on hips, knees lifting high in rhythmic bounce, enthusiastic happy smile. 4k resolution, 60fps, Disney Pixar render, joyful preschool music video style.</t>
         </is>
       </c>
+      <c r="K9" s="20" t="inlineStr">
+        <is>
+          <t>images/track_07/a1_s07_seg07_girl.jpg</t>
+        </is>
+      </c>
     </row>
     <row r="10" ht="30" customHeight="1">
       <c r="A10" s="8" t="inlineStr">
@@ -1480,6 +1565,11 @@
           <t>3D Pixar Disney style cheerful toddler dance coach, smooth playful animation, vibrant kindergarten studio, soft bright volumetric lighting, clean studio background, highly expressive face, full body dynamic camera shot: Song 'The Magic ABC Train', Action '第 07 節: 聽火車汽笛鈴聲'. 🔔 單手拉響汽笛：嗚嗚！聽車鈴叮噹響！. The character is stretching arms up high to reach floating elements, standing on tiptoes, joyful posture, looking up with wonder. 4k resolution, 60fps, Disney Pixar render, joyful preschool music video style.</t>
         </is>
       </c>
+      <c r="K10" s="20" t="inlineStr">
+        <is>
+          <t>images/track_07/a1_s07_seg08_girl.jpg</t>
+        </is>
+      </c>
     </row>
     <row r="11" ht="30" customHeight="1">
       <c r="A11" s="10" t="inlineStr">
@@ -1528,6 +1618,11 @@
           <t>3D Pixar Disney style cheerful toddler dance coach, smooth playful animation, vibrant kindergarten studio, soft bright volumetric lighting, clean studio background, highly expressive face, full body dynamic camera shot: Song 'The Magic ABC Train', Action '第 08 節: 字母 M 露出微笑'. 😊 雙手在嘴角畫出最甜的微笑波浪！. The character is bringing hands together at the chest forming an adorable glowing heart shape, leaning slightly forward, loving gentle smile. 4k resolution, 60fps, Disney Pixar render, joyful preschool music video style.</t>
         </is>
       </c>
+      <c r="K11" s="20" t="inlineStr">
+        <is>
+          <t>images/track_07/a1_s07_seg09_girl.jpg</t>
+        </is>
+      </c>
     </row>
     <row r="12" ht="30" customHeight="1">
       <c r="A12" s="8" t="inlineStr">
@@ -1576,6 +1671,11 @@
           <t>3D Pixar Disney style cheerful toddler dance coach, smooth playful animation, vibrant kindergarten studio, soft bright volumetric lighting, clean studio background, highly expressive face, full body dynamic camera shot: Song 'The Magic ABC Train', Action '第 09 節: 指引列車迎向光明'. ✨ 雙臂向前上方伸出，指引光明方向！. The character is lifting arms from heart to sky creating a big golden sun circle, chest open, radiant beaming joyful smile. 4k resolution, 60fps, Disney Pixar render, joyful preschool music video style.</t>
         </is>
       </c>
+      <c r="K12" s="20" t="inlineStr">
+        <is>
+          <t>images/track_07/a1_s07_seg10_girl.jpg</t>
+        </is>
+      </c>
     </row>
     <row r="13" ht="30" customHeight="1">
       <c r="A13" s="10" t="inlineStr">
@@ -1624,6 +1724,11 @@
           <t>3D Pixar Disney style cheerful toddler dance coach, smooth playful animation, vibrant kindergarten studio, soft bright volumetric lighting, clean studio background, highly expressive face, full body dynamic camera shot: Song 'The Magic ABC Train', Action '第 10 節: 咔嚓咔嚓車輪滾'. 🚂 雙手在腰側做車輪旋轉動作向前滾！. The character is marching in place energetically, hands on hips, knees lifting high in rhythmic bounce, enthusiastic happy smile. 4k resolution, 60fps, Disney Pixar render, joyful preschool music video style.</t>
         </is>
       </c>
+      <c r="K13" s="20" t="inlineStr">
+        <is>
+          <t>images/track_07/a1_s07_seg11_girl.jpg</t>
+        </is>
+      </c>
     </row>
     <row r="14" ht="30" customHeight="1">
       <c r="A14" s="8" t="inlineStr">
@@ -1672,6 +1777,11 @@
           <t>3D Pixar Disney style cheerful toddler dance coach, smooth playful animation, vibrant kindergarten studio, soft bright volumetric lighting, clean studio background, highly expressive face, full body dynamic camera shot: Song 'The Magic ABC Train', Action '第 11 節: 字母歌聲唱呀唱'. 🎶 張開雙臂放聲歌唱，身體輕快彈動！. The character is waving both hands overhead in friendly wide arcs, swaying gently from side to side, sparkling excited eyes. 4k resolution, 60fps, Disney Pixar render, joyful preschool music video style.</t>
         </is>
       </c>
+      <c r="K14" s="20" t="inlineStr">
+        <is>
+          <t>images/track_07/a1_s07_seg12_girl.jpg</t>
+        </is>
+      </c>
     </row>
     <row r="15" ht="30" customHeight="1">
       <c r="A15" s="10" t="inlineStr">
@@ -1720,6 +1830,11 @@
           <t>3D Pixar Disney style cheerful toddler dance coach, smooth playful animation, vibrant kindergarten studio, soft bright volumetric lighting, clean studio background, highly expressive face, full body dynamic camera shot: Song 'The Magic ABC Train', Action '第 12 節: 鐵軌從 A 開到 Z'. 🛤️ 雙手臂向兩側平展，像長長鐵軌！. The character is stretching arms up high to reach floating elements, standing on tiptoes, joyful posture, looking up with wonder. 4k resolution, 60fps, Disney Pixar render, joyful preschool music video style.</t>
         </is>
       </c>
+      <c r="K15" s="20" t="inlineStr">
+        <is>
+          <t>images/track_07/a1_s07_seg13_girl.jpg</t>
+        </is>
+      </c>
     </row>
     <row r="16" ht="30" customHeight="1">
       <c r="A16" s="8" t="inlineStr">
@@ -1768,6 +1883,11 @@
           <t>3D Pixar Disney style cheerful toddler dance coach, smooth playful animation, vibrant kindergarten studio, soft bright volumetric lighting, clean studio background, highly expressive face, full body dynamic camera shot: Song 'The Magic ABC Train', Action '第 13 節: 快快樂樂學字母'. 🎉 歡快原地踏步拍拍手，學習好快樂！. The character is squatting down and bursting into a high happy jump, feet kicking joyfully in mid-air, both fists punching the sky in victory. 4k resolution, 60fps, Disney Pixar render, joyful preschool music video style.</t>
         </is>
       </c>
+      <c r="K16" s="20" t="inlineStr">
+        <is>
+          <t>images/track_07/a1_s07_seg14_girl.jpg</t>
+        </is>
+      </c>
     </row>
     <row r="17" ht="30" customHeight="1">
       <c r="A17" s="10" t="inlineStr">
@@ -1816,6 +1936,11 @@
           <t>3D Pixar Disney style cheerful toddler dance coach, smooth playful animation, vibrant kindergarten studio, soft bright volumetric lighting, clean studio background, highly expressive face, full body dynamic camera shot: Song 'The Magic ABC Train', Action '第 14 節: N 是鳥巢 O 是貓頭鷹'. 🦉 雙手捧起溫暖鳥巢，雙手圈眼睛當大眼！. The character is bringing hands together at the chest forming an adorable glowing heart shape, leaning slightly forward, loving gentle smile. 4k resolution, 60fps, Disney Pixar render, joyful preschool music video style.</t>
         </is>
       </c>
+      <c r="K17" s="20" t="inlineStr">
+        <is>
+          <t>images/track_07/a1_s07_seg15_girl.jpg</t>
+        </is>
+      </c>
     </row>
     <row r="18" ht="30" customHeight="1">
       <c r="A18" s="8" t="inlineStr">
@@ -1864,6 +1989,11 @@
           <t>3D Pixar Disney style cheerful toddler dance coach, smooth playful animation, vibrant kindergarten studio, soft bright volumetric lighting, clean studio background, highly expressive face, full body dynamic camera shot: Song 'The Magic ABC Train', Action '第 15 節: P 是圓圓黑眼大熊貓'. 🐼 雙手揉揉黑眼圈，學小熊貓吃竹子！. The character is swaying hips and arms like a breeze, smooth fluid body roll, playful rhythmic dancing, friendly warm smile. 4k resolution, 60fps, Disney Pixar render, joyful preschool music video style.</t>
         </is>
       </c>
+      <c r="K18" s="20" t="inlineStr">
+        <is>
+          <t>images/track_07/a1_s07_seg16_girl.jpg</t>
+        </is>
+      </c>
     </row>
     <row r="19" ht="30" customHeight="1">
       <c r="A19" s="10" t="inlineStr">
@@ -1912,6 +2042,11 @@
           <t>3D Pixar Disney style cheerful toddler dance coach, smooth playful animation, vibrant kindergarten studio, soft bright volumetric lighting, clean studio background, highly expressive face, full body dynamic camera shot: Song 'The Magic ABC Train', Action '第 16 節: Q R S T 快快衝'. ⚡ 雙腳加速踩踏步，列車飛速奔馳！. The character is marching in place energetically, hands on hips, knees lifting high in rhythmic bounce, enthusiastic happy smile. 4k resolution, 60fps, Disney Pixar render, joyful preschool music video style.</t>
         </is>
       </c>
+      <c r="K19" s="20" t="inlineStr">
+        <is>
+          <t>images/track_07/a1_s07_seg17_girl.jpg</t>
+        </is>
+      </c>
     </row>
     <row r="20" ht="30" customHeight="1">
       <c r="A20" s="8" t="inlineStr">
@@ -1960,6 +2095,11 @@
           <t>3D Pixar Disney style cheerful toddler dance coach, smooth playful animation, vibrant kindergarten studio, soft bright volumetric lighting, clean studio background, highly expressive face, full body dynamic camera shot: Song 'The Magic ABC Train', Action '第 17 節: 看美麗字母飛過'. 👀 伸手指向窗外，欣賞美麗字母飄過！. The character is stretching arms up high to reach floating elements, standing on tiptoes, joyful posture, looking up with wonder. 4k resolution, 60fps, Disney Pixar render, joyful preschool music video style.</t>
         </is>
       </c>
+      <c r="K20" s="20" t="inlineStr">
+        <is>
+          <t>images/track_07/a1_s07_seg18_girl.jpg</t>
+        </is>
+      </c>
     </row>
     <row r="21" ht="30" customHeight="1">
       <c r="A21" s="10" t="inlineStr">
@@ -2008,6 +2148,11 @@
           <t>3D Pixar Disney style cheerful toddler dance coach, smooth playful animation, vibrant kindergarten studio, soft bright volumetric lighting, clean studio background, highly expressive face, full body dynamic camera shot: Song 'The Magic ABC Train', Action '第 18 節: U V W X Y Z 全學會'. 🌟 雙手高舉揮舞，26 個字母全認識啦！. The character is lifting arms from heart to sky creating a big golden sun circle, chest open, radiant beaming joyful smile. 4k resolution, 60fps, Disney Pixar render, joyful preschool music video style.</t>
         </is>
       </c>
+      <c r="K21" s="20" t="inlineStr">
+        <is>
+          <t>images/track_07/a1_s07_seg19_girl.jpg</t>
+        </is>
+      </c>
     </row>
     <row r="22" ht="30" customHeight="1">
       <c r="A22" s="8" t="inlineStr">
@@ -2056,6 +2201,11 @@
           <t>3D Pixar Disney style cheerful toddler dance coach, smooth playful animation, vibrant kindergarten studio, soft bright volumetric lighting, clean studio background, highly expressive face, full body dynamic camera shot: Song 'The Magic ABC Train', Action '第 19 節: 每個字母都有聲音'. 👂 小手貼耳仔細聽，每個發音都動聽！. The character is swaying hips and arms like a breeze, smooth fluid body roll, playful rhythmic dancing, friendly warm smile. 4k resolution, 60fps, Disney Pixar render, joyful preschool music video style.</t>
         </is>
       </c>
+      <c r="K22" s="20" t="inlineStr">
+        <is>
+          <t>images/track_07/a1_s07_seg20_girl.jpg</t>
+        </is>
+      </c>
     </row>
     <row r="23" ht="30" customHeight="1">
       <c r="A23" s="10" t="inlineStr">
@@ -2104,6 +2254,11 @@
           <t>3D Pixar Disney style cheerful toddler dance coach, smooth playful animation, vibrant kindergarten studio, soft bright volumetric lighting, clean studio background, highly expressive face, full body dynamic camera shot: Song 'The Magic ABC Train', Action '第 20 節: 拼出魔法奇妙單字'. ✨ 雙手像施魔法在前方抓一抓灑一灑！. The character is stretching arms up high to reach floating elements, standing on tiptoes, joyful posture, looking up with wonder. 4k resolution, 60fps, Disney Pixar render, joyful preschool music video style.</t>
         </is>
       </c>
+      <c r="K23" s="20" t="inlineStr">
+        <is>
+          <t>images/track_07/a1_s07_seg21_girl.jpg</t>
+        </is>
+      </c>
     </row>
     <row r="24" ht="30" customHeight="1">
       <c r="A24" s="8" t="inlineStr">
@@ -2152,6 +2307,11 @@
           <t>3D Pixar Disney style cheerful toddler dance coach, smooth playful animation, vibrant kindergarten studio, soft bright volumetric lighting, clean studio background, highly expressive face, full body dynamic camera shot: Song 'The Magic ABC Train', Action '第 21 節: 咔嚓咔嚓鈴兒響'. 🔔 再次轉動火車小輪子，聽鈴鐺叮叮！. The character is marching in place energetically, hands on hips, knees lifting high in rhythmic bounce, enthusiastic happy smile. 4k resolution, 60fps, Disney Pixar render, joyful preschool music video style.</t>
         </is>
       </c>
+      <c r="K24" s="20" t="inlineStr">
+        <is>
+          <t>images/track_07/a1_s07_seg22_girl.jpg</t>
+        </is>
+      </c>
     </row>
     <row r="25" ht="30" customHeight="1">
       <c r="A25" s="10" t="inlineStr">
@@ -2200,6 +2360,11 @@
           <t>3D Pixar Disney style cheerful toddler dance coach, smooth playful animation, vibrant kindergarten studio, soft bright volumetric lighting, clean studio background, highly expressive face, full body dynamic camera shot: Song 'The Magic ABC Train', Action '第 22 節: 字母歌聲唱呀唱'. 🎶 大聲齊聲合唱：Sing! Sing! Sing!. The character is waving both hands overhead in friendly wide arcs, swaying gently from side to side, sparkling excited eyes. 4k resolution, 60fps, Disney Pixar render, joyful preschool music video style.</t>
         </is>
       </c>
+      <c r="K25" s="20" t="inlineStr">
+        <is>
+          <t>images/track_07/a1_s07_seg23_girl.jpg</t>
+        </is>
+      </c>
     </row>
     <row r="26" ht="30" customHeight="1">
       <c r="A26" s="8" t="inlineStr">
@@ -2248,6 +2413,11 @@
           <t>3D Pixar Disney style cheerful toddler dance coach, smooth playful animation, vibrant kindergarten studio, soft bright volumetric lighting, clean studio background, highly expressive face, full body dynamic camera shot: Song 'The Magic ABC Train', Action '第 23 節: 沿著軌道 A 到 Z'. 🛤️ 雙臂大幅度擺動，列車一路暢通！. The character is stretching arms up high to reach floating elements, standing on tiptoes, joyful posture, looking up with wonder. 4k resolution, 60fps, Disney Pixar render, joyful preschool music video style.</t>
         </is>
       </c>
+      <c r="K26" s="20" t="inlineStr">
+        <is>
+          <t>images/track_07/a1_s07_seg24_girl.jpg</t>
+        </is>
+      </c>
     </row>
     <row r="27" ht="30" customHeight="1">
       <c r="A27" s="10" t="inlineStr">
@@ -2296,6 +2466,11 @@
           <t>3D Pixar Disney style cheerful toddler dance coach, smooth playful animation, vibrant kindergarten studio, soft bright volumetric lighting, clean studio background, highly expressive face, full body dynamic camera shot: Song 'The Magic ABC Train', Action '第 24 節: 字母列車真好玩'. ⭐ 雙手胸前比心，身體快樂搖晃！. The character is bringing hands together at the chest forming an adorable glowing heart shape, leaning slightly forward, loving gentle smile. 4k resolution, 60fps, Disney Pixar render, joyful preschool music video style.</t>
         </is>
       </c>
+      <c r="K27" s="20" t="inlineStr">
+        <is>
+          <t>images/track_07/a1_s07_seg25_girl.jpg</t>
+        </is>
+      </c>
     </row>
     <row r="28" ht="30" customHeight="1">
       <c r="A28" s="8" t="inlineStr">
@@ -2342,6 +2517,11 @@
       <c r="J28" s="9" t="inlineStr">
         <is>
           <t>3D Pixar Disney style cheerful toddler dance coach, smooth playful animation, vibrant kindergarten studio, soft bright volumetric lighting, clean studio background, highly expressive face, full body dynamic camera shot: Song 'The Magic ABC Train', Action '第 25 節: 閱讀車站到站啦定格'. 🚉 敬禮拉汽笛：叮叮！全劇歡樂定格！. The character is lifting arms from heart to sky creating a big golden sun circle, chest open, radiant beaming joyful smile. 4k resolution, 60fps, Disney Pixar render, joyful preschool music video style.</t>
+        </is>
+      </c>
+      <c r="K28" s="20" t="inlineStr">
+        <is>
+          <t>images/track_07/a1_s07_seg26_girl.jpg</t>
         </is>
       </c>
     </row>
@@ -2359,7 +2539,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J29"/>
+  <dimension ref="A1:K29"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="18" customWidth="1" min="1" max="1"/>
@@ -2372,6 +2552,7 @@
     <col width="30" customWidth="1" min="8" max="8"/>
     <col width="12" customWidth="1" min="9" max="9"/>
     <col width="55" customWidth="1" min="10" max="10"/>
+    <col width="34" customWidth="1" min="11" max="11"/>
   </cols>
   <sheetData>
     <row r="1" ht="32" customHeight="1">
@@ -2432,6 +2613,11 @@
           <t>AI 影片動畫生成提示詞 (Prompt)</t>
         </is>
       </c>
+      <c r="K2" s="19" t="inlineStr">
+        <is>
+          <t>首張圖片路徑 (9:16 720p)</t>
+        </is>
+      </c>
     </row>
     <row r="3" ht="30" customHeight="1">
       <c r="A3" s="10" t="inlineStr">
@@ -2480,6 +2666,11 @@
           <t>3D Pixar Disney style preschool animation video keyframe, vertical 9:16 aspect ratio 720p HD. Full body standing shot of the cheerful 5-year-old boy dance coach in bright blue athletic t-shirt with orange center and KIDS DANCE logo, blue shorts, orange running sneakers. In colorful kindergarten dance studio. Starter keyframe for action "第 01 節: 節奏鼓點咚咚咚" (🥁 腳尖踩拍子，雙手輕快拍拍大腿！). The character is in lively dance starter pose, joyful radiant beaming smile, sparkling expressive eyes. 4k 3D Pixar render, clean frame without text overlay, starter keyframe for image-to-video generation (a1_s08_seg01_boy.jpg).</t>
         </is>
       </c>
+      <c r="K3" s="20" t="inlineStr">
+        <is>
+          <t>images/track_08/a1_s08_seg01_boy.jpg</t>
+        </is>
+      </c>
     </row>
     <row r="4" ht="30" customHeight="1">
       <c r="A4" s="8" t="inlineStr">
@@ -2528,6 +2719,11 @@
           <t>3D Pixar Disney style cheerful toddler dance coach, smooth playful animation, vibrant kindergarten studio, soft bright volumetric lighting, clean studio background, highly expressive face, full body dynamic camera shot: Song 'Wiggle &amp; Freeze!', Action '第 02 節: 口哨響起準備扭'. 🎶 雙手插腰，肩膀跟著旋律左右擺動！. The character is swaying hips and arms like a breeze, smooth fluid body roll, playful rhythmic dancing, friendly warm smile. 4k resolution, 60fps, Disney Pixar render, joyful preschool music video style.</t>
         </is>
       </c>
+      <c r="K4" s="20" t="inlineStr">
+        <is>
+          <t>images/track_08/a1_s08_seg02_boy.jpg</t>
+        </is>
+      </c>
     </row>
     <row r="5" ht="30" customHeight="1">
       <c r="A5" s="10" t="inlineStr">
@@ -2576,6 +2772,11 @@
           <t>3D Pixar Disney style cheerful toddler dance coach, smooth playful animation, vibrant kindergarten studio, soft bright volumetric lighting, clean studio background, highly expressive face, full body dynamic camera shot: Song 'Wiggle &amp; Freeze!', Action '第 03 節: 全身扭動別忘定格'. 💃 全身快樂扭動，耳朵豎起聽指令！. The character is swaying hips and arms like a breeze, smooth fluid body roll, playful rhythmic dancing, friendly warm smile. 4k resolution, 60fps, Disney Pixar render, joyful preschool music video style.</t>
         </is>
       </c>
+      <c r="K5" s="20" t="inlineStr">
+        <is>
+          <t>images/track_08/a1_s08_seg03_boy.jpg</t>
+        </is>
+      </c>
     </row>
     <row r="6" ht="30" customHeight="1">
       <c r="A6" s="8" t="inlineStr">
@@ -2624,6 +2825,11 @@
           <t>3D Pixar Disney style cheerful toddler dance coach, smooth playful animation, vibrant kindergarten studio, soft bright volumetric lighting, clean studio background, highly expressive face, full body dynamic camera shot: Song 'Wiggle &amp; Freeze!', Action '第 04 節: 搖搖肩膀搖搖膝蓋'. 🦵 左右肩膀抖一抖，膝蓋跟著彈一彈！. The character is marching in place energetically, hands on hips, knees lifting high in rhythmic bounce, enthusiastic happy smile. 4k resolution, 60fps, Disney Pixar render, joyful preschool music video style.</t>
         </is>
       </c>
+      <c r="K6" s="20" t="inlineStr">
+        <is>
+          <t>images/track_08/a1_s08_seg04_boy.jpg</t>
+        </is>
+      </c>
     </row>
     <row r="7" ht="30" customHeight="1">
       <c r="A7" s="10" t="inlineStr">
@@ -2672,6 +2878,11 @@
           <t>3D Pixar Disney style cheerful toddler dance coach, smooth playful animation, vibrant kindergarten studio, soft bright volumetric lighting, clean studio background, highly expressive face, full body dynamic camera shot: Song 'Wiggle &amp; Freeze!', Action '第 05 節: 像秋天落葉隨風飄'. 🍂 雙手像樹葉在微風中輕輕飄落！. The character is waving both hands overhead in friendly wide arcs, swaying gently from side to side, sparkling excited eyes. 4k resolution, 60fps, Disney Pixar render, joyful preschool music video style.</t>
         </is>
       </c>
+      <c r="K7" s="20" t="inlineStr">
+        <is>
+          <t>images/track_08/a1_s08_seg05_boy.jpg</t>
+        </is>
+      </c>
     </row>
     <row r="8" ht="30" customHeight="1">
       <c r="A8" s="8" t="inlineStr">
@@ -2720,6 +2931,11 @@
           <t>3D Pixar Disney style cheerful toddler dance coach, smooth playful animation, vibrant kindergarten studio, soft bright volumetric lighting, clean studio background, highly expressive face, full body dynamic camera shot: Song 'Wiggle &amp; Freeze!', Action '第 06 節: 高高跳起摸摸天地'. ⭐ 向上跳摸天花板，下蹲摸摸小地板！. The character is squatting down and bursting into a high happy jump, feet kicking joyfully in mid-air, both fists punching the sky in victory. 4k resolution, 60fps, Disney Pixar render, joyful preschool music video style.</t>
         </is>
       </c>
+      <c r="K8" s="20" t="inlineStr">
+        <is>
+          <t>images/track_08/a1_s08_seg06_boy.jpg</t>
+        </is>
+      </c>
     </row>
     <row r="9" ht="30" customHeight="1">
       <c r="A9" s="10" t="inlineStr">
@@ -2768,6 +2984,11 @@
           <t>3D Pixar Disney style cheerful toddler dance coach, smooth playful animation, vibrant kindergarten studio, soft bright volumetric lighting, clean studio background, highly expressive face, full body dynamic camera shot: Song 'Wiggle &amp; Freeze!', Action '第 07 節: 原地小跑步跑起來'. 🏃 原地快速小碎步跑步，越跑越快！. The character is marching in place energetically, hands on hips, knees lifting high in rhythmic bounce, enthusiastic happy smile. 4k resolution, 60fps, Disney Pixar render, joyful preschool music video style.</t>
         </is>
       </c>
+      <c r="K9" s="20" t="inlineStr">
+        <is>
+          <t>images/track_08/a1_s08_seg07_boy.jpg</t>
+        </is>
+      </c>
     </row>
     <row r="10" ht="30" customHeight="1">
       <c r="A10" s="8" t="inlineStr">
@@ -2816,6 +3037,11 @@
           <t>3D Pixar Disney style cheerful toddler dance coach, smooth playful animation, vibrant kindergarten studio, soft bright volumetric lighting, clean studio background, highly expressive face, full body dynamic camera shot: Song 'Wiggle &amp; Freeze!', Action '第 08 節: 仔細聽停下腳步'. 👂 停下腳步站穩，準備倒數！. The character is stretching arms up high to reach floating elements, standing on tiptoes, joyful posture, looking up with wonder. 4k resolution, 60fps, Disney Pixar render, joyful preschool music video style.</t>
         </is>
       </c>
+      <c r="K10" s="20" t="inlineStr">
+        <is>
+          <t>images/track_08/a1_s08_seg08_boy.jpg</t>
+        </is>
+      </c>
     </row>
     <row r="11" ht="30" customHeight="1">
       <c r="A11" s="10" t="inlineStr">
@@ -2864,6 +3090,11 @@
           <t>3D Pixar Disney style cheerful toddler dance coach, smooth playful animation, vibrant kindergarten studio, soft bright volumetric lighting, clean studio background, highly expressive face, full body dynamic camera shot: Song 'Wiggle &amp; Freeze!', Action '第 09 節: 三二一定格成雕像'. 🗿 3 2 1... 定格！像雕像一樣一動不動！. The character is stretching arms up high to reach floating elements, standing on tiptoes, joyful posture, looking up with wonder. 4k resolution, 60fps, Disney Pixar render, joyful preschool music video style.</t>
         </is>
       </c>
+      <c r="K11" s="20" t="inlineStr">
+        <is>
+          <t>images/track_08/a1_s08_seg09_boy.jpg</t>
+        </is>
+      </c>
     </row>
     <row r="12" ht="30" customHeight="1">
       <c r="A12" s="8" t="inlineStr">
@@ -2912,6 +3143,11 @@
           <t>3D Pixar Disney style cheerful toddler dance coach, smooth playful animation, vibrant kindergarten studio, soft bright volumetric lighting, clean studio background, highly expressive face, full body dynamic camera shot: Song 'Wiggle &amp; Freeze!', Action '第 10 節: 安靜定格不許動'. 🤫 憋住笑不許動，維持雕像姿勢！. The character is stretching arms up high to reach floating elements, standing on tiptoes, joyful posture, looking up with wonder. 4k resolution, 60fps, Disney Pixar render, joyful preschool music video style.</t>
         </is>
       </c>
+      <c r="K12" s="20" t="inlineStr">
+        <is>
+          <t>images/track_08/a1_s08_seg10_boy.jpg</t>
+        </is>
+      </c>
     </row>
     <row r="13" ht="30" customHeight="1">
       <c r="A13" s="10" t="inlineStr">
@@ -2960,6 +3196,11 @@
           <t>3D Pixar Disney style cheerful toddler dance coach, smooth playful animation, vibrant kindergarten studio, soft bright volumetric lighting, clean studio background, highly expressive face, full body dynamic camera shot: Song 'Wiggle &amp; Freeze!', Action '第 11 節: 扭扭扭動跳舞囉'. 🎉 解凍啦！扭動全身，滿場飛舞！. The character is squatting down and bursting into a high happy jump, feet kicking joyfully in mid-air, both fists punching the sky in victory. 4k resolution, 60fps, Disney Pixar render, joyful preschool music video style.</t>
         </is>
       </c>
+      <c r="K13" s="20" t="inlineStr">
+        <is>
+          <t>images/track_08/a1_s08_seg11_boy.jpg</t>
+        </is>
+      </c>
     </row>
     <row r="14" ht="30" customHeight="1">
       <c r="A14" s="8" t="inlineStr">
@@ -3008,6 +3249,11 @@
           <t>3D Pixar Disney style cheerful toddler dance coach, smooth playful animation, vibrant kindergarten studio, soft bright volumetric lighting, clean studio background, highly expressive face, full body dynamic camera shot: Song 'Wiggle &amp; Freeze!', Action '第 12 節: 大腳重重踏地上'. 👣 雙腳大踏步：咚！咚！咚！踏在地上！. The character is marching in place energetically, hands on hips, knees lifting high in rhythmic bounce, enthusiastic happy smile. 4k resolution, 60fps, Disney Pixar render, joyful preschool music video style.</t>
         </is>
       </c>
+      <c r="K14" s="20" t="inlineStr">
+        <is>
+          <t>images/track_08/a1_s08_seg12_boy.jpg</t>
+        </is>
+      </c>
     </row>
     <row r="15" ht="30" customHeight="1">
       <c r="A15" s="10" t="inlineStr">
@@ -3056,6 +3302,11 @@
           <t>3D Pixar Disney style cheerful toddler dance coach, smooth playful animation, vibrant kindergarten studio, soft bright volumetric lighting, clean studio background, highly expressive face, full body dynamic camera shot: Song 'Wiggle &amp; Freeze!', Action '第 13 節: 往左扭扭往右扭扭'. ↔️ 身體向左扭一扭，向右扭一扭！. The character is swaying hips and arms like a breeze, smooth fluid body roll, playful rhythmic dancing, friendly warm smile. 4k resolution, 60fps, Disney Pixar render, joyful preschool music video style.</t>
         </is>
       </c>
+      <c r="K15" s="20" t="inlineStr">
+        <is>
+          <t>images/track_08/a1_s08_seg13_boy.jpg</t>
+        </is>
+      </c>
     </row>
     <row r="16" ht="30" customHeight="1">
       <c r="A16" s="8" t="inlineStr">
@@ -3104,6 +3355,11 @@
           <t>3D Pixar Disney style cheerful toddler dance coach, smooth playful animation, vibrant kindergarten studio, soft bright volumetric lighting, clean studio background, highly expressive face, full body dynamic camera shot: Song 'Wiggle &amp; Freeze!', Action '第 14 節: 使出全力快樂跳'. 🔥 使出全身力氣，跳出最帥舞蹈！. The character is squatting down and bursting into a high happy jump, feet kicking joyfully in mid-air, both fists punching the sky in victory. 4k resolution, 60fps, Disney Pixar render, joyful preschool music video style.</t>
         </is>
       </c>
+      <c r="K16" s="20" t="inlineStr">
+        <is>
+          <t>images/track_08/a1_s08_seg14_boy.jpg</t>
+        </is>
+      </c>
     </row>
     <row r="17" ht="30" customHeight="1">
       <c r="A17" s="10" t="inlineStr">
@@ -3152,6 +3408,11 @@
           <t>3D Pixar Disney style cheerful toddler dance coach, smooth playful animation, vibrant kindergarten studio, soft bright volumetric lighting, clean studio background, highly expressive face, full body dynamic camera shot: Song 'Wiggle &amp; Freeze!', Action '第 15 節: 像陀螺旋轉轉圈'. 🔄 雙手平展像小陀螺，旋轉轉個圈！. The character is swaying hips and arms like a breeze, smooth fluid body roll, playful rhythmic dancing, friendly warm smile. 4k resolution, 60fps, Disney Pixar render, joyful preschool music video style.</t>
         </is>
       </c>
+      <c r="K17" s="20" t="inlineStr">
+        <is>
+          <t>images/track_08/a1_s08_seg15_boy.jpg</t>
+        </is>
+      </c>
     </row>
     <row r="18" ht="30" customHeight="1">
       <c r="A18" s="8" t="inlineStr">
@@ -3200,6 +3461,11 @@
           <t>3D Pixar Disney style cheerful toddler dance coach, smooth playful animation, vibrant kindergarten studio, soft bright volumetric lighting, clean studio background, highly expressive face, full body dynamic camera shot: Song 'Wiggle &amp; Freeze!', Action '第 16 節: 墊起腳尖悄悄走'. 🐾 墊起腳尖輕輕走，一點聲音都沒有！. The character is marching in place energetically, hands on hips, knees lifting high in rhythmic bounce, enthusiastic happy smile. 4k resolution, 60fps, Disney Pixar render, joyful preschool music video style.</t>
         </is>
       </c>
+      <c r="K18" s="20" t="inlineStr">
+        <is>
+          <t>images/track_08/a1_s08_seg16_boy.jpg</t>
+        </is>
+      </c>
     </row>
     <row r="19" ht="30" customHeight="1">
       <c r="A19" s="10" t="inlineStr">
@@ -3248,6 +3514,11 @@
           <t>3D Pixar Disney style cheerful toddler dance coach, smooth playful animation, vibrant kindergarten studio, soft bright volumetric lighting, clean studio background, highly expressive face, full body dynamic camera shot: Song 'Wiggle &amp; Freeze!', Action '第 17 節: 雄鷹展翅翱翔天'. 🦅 雙臂像雄鷹拍打翅膀，飛上天空！. The character is waving both hands overhead in friendly wide arcs, swaying gently from side to side, sparkling excited eyes. 4k resolution, 60fps, Disney Pixar render, joyful preschool music video style.</t>
         </is>
       </c>
+      <c r="K19" s="20" t="inlineStr">
+        <is>
+          <t>images/track_08/a1_s08_seg17_boy.jpg</t>
+        </is>
+      </c>
     </row>
     <row r="20" ht="30" customHeight="1">
       <c r="A20" s="8" t="inlineStr">
@@ -3296,6 +3567,11 @@
           <t>3D Pixar Disney style cheerful toddler dance coach, smooth playful animation, vibrant kindergarten studio, soft bright volumetric lighting, clean studio background, highly expressive face, full body dynamic camera shot: Song 'Wiggle &amp; Freeze!', Action '第 18 節: 雙手舉高高大招手'. 👋 雙手舉過頭頂，熱情大幅度招手！. The character is lifting arms from heart to sky creating a big golden sun circle, chest open, radiant beaming joyful smile. 4k resolution, 60fps, Disney Pixar render, joyful preschool music video style.</t>
         </is>
       </c>
+      <c r="K20" s="20" t="inlineStr">
+        <is>
+          <t>images/track_08/a1_s08_seg18_boy.jpg</t>
+        </is>
+      </c>
     </row>
     <row r="21" ht="30" customHeight="1">
       <c r="A21" s="10" t="inlineStr">
@@ -3344,6 +3620,11 @@
           <t>3D Pixar Disney style cheerful toddler dance coach, smooth playful animation, vibrant kindergarten studio, soft bright volumetric lighting, clean studio background, highly expressive face, full body dynamic camera shot: Song 'Wiggle &amp; Freeze!', Action '第 19 節: 準備好擺好姿勢'. 🎯 保持好平衡姿勢，馬上要定格啦！. The character is stretching arms up high to reach floating elements, standing on tiptoes, joyful posture, looking up with wonder. 4k resolution, 60fps, Disney Pixar render, joyful preschool music video style.</t>
         </is>
       </c>
+      <c r="K21" s="20" t="inlineStr">
+        <is>
+          <t>images/track_08/a1_s08_seg19_boy.jpg</t>
+        </is>
+      </c>
     </row>
     <row r="22" ht="30" customHeight="1">
       <c r="A22" s="8" t="inlineStr">
@@ -3392,6 +3673,11 @@
           <t>3D Pixar Disney style cheerful toddler dance coach, smooth playful animation, vibrant kindergarten studio, soft bright volumetric lighting, clean studio background, highly expressive face, full body dynamic camera shot: Song 'Wiggle &amp; Freeze!', Action '第 20 節: 三二一定格摸鼻子'. 👃 3 2 1... 定格！食指摸著小鼻子！. The character is stretching arms up high to reach floating elements, standing on tiptoes, joyful posture, looking up with wonder. 4k resolution, 60fps, Disney Pixar render, joyful preschool music video style.</t>
         </is>
       </c>
+      <c r="K22" s="20" t="inlineStr">
+        <is>
+          <t>images/track_08/a1_s08_seg20_boy.jpg</t>
+        </is>
+      </c>
     </row>
     <row r="23" ht="30" customHeight="1">
       <c r="A23" s="10" t="inlineStr">
@@ -3440,6 +3726,11 @@
           <t>3D Pixar Disney style cheerful toddler dance coach, smooth playful animation, vibrant kindergarten studio, soft bright volumetric lighting, clean studio background, highly expressive face, full body dynamic camera shot: Song 'Wiggle &amp; Freeze!', Action '第 21 節: 安靜定格摸鼻子'. 🤫 保持摸鼻子的造型，一動也不動！. The character is stretching arms up high to reach floating elements, standing on tiptoes, joyful posture, looking up with wonder. 4k resolution, 60fps, Disney Pixar render, joyful preschool music video style.</t>
         </is>
       </c>
+      <c r="K23" s="20" t="inlineStr">
+        <is>
+          <t>images/track_08/a1_s08_seg21_boy.jpg</t>
+        </is>
+      </c>
     </row>
     <row r="24" ht="30" customHeight="1">
       <c r="A24" s="8" t="inlineStr">
@@ -3488,6 +3779,11 @@
           <t>3D Pixar Disney style cheerful toddler dance coach, smooth playful animation, vibrant kindergarten studio, soft bright volumetric lighting, clean studio background, highly expressive face, full body dynamic camera shot: Song 'Wiggle &amp; Freeze!', Action '第 22 節: 解凍繼續扭扭跳'. 🎉 解凍！滿場歡跳，跟著節奏搖擺！. The character is squatting down and bursting into a high happy jump, feet kicking joyfully in mid-air, both fists punching the sky in victory. 4k resolution, 60fps, Disney Pixar render, joyful preschool music video style.</t>
         </is>
       </c>
+      <c r="K24" s="20" t="inlineStr">
+        <is>
+          <t>images/track_08/a1_s08_seg22_boy.jpg</t>
+        </is>
+      </c>
     </row>
     <row r="25" ht="30" customHeight="1">
       <c r="A25" s="10" t="inlineStr">
@@ -3536,6 +3832,11 @@
           <t>3D Pixar Disney style cheerful toddler dance coach, smooth playful animation, vibrant kindergarten studio, soft bright volumetric lighting, clean studio background, highly expressive face, full body dynamic camera shot: Song 'Wiggle &amp; Freeze!', Action '第 23 節: 大腳踏地震天響'. 👣 跟著大鼓重重踩踩腳，地面咚咚響！. The character is marching in place energetically, hands on hips, knees lifting high in rhythmic bounce, enthusiastic happy smile. 4k resolution, 60fps, Disney Pixar render, joyful preschool music video style.</t>
         </is>
       </c>
+      <c r="K25" s="20" t="inlineStr">
+        <is>
+          <t>images/track_08/a1_s08_seg23_boy.jpg</t>
+        </is>
+      </c>
     </row>
     <row r="26" ht="30" customHeight="1">
       <c r="A26" s="8" t="inlineStr">
@@ -3584,6 +3885,11 @@
           <t>3D Pixar Disney style cheerful toddler dance coach, smooth playful animation, vibrant kindergarten studio, soft bright volumetric lighting, clean studio background, highly expressive face, full body dynamic camera shot: Song 'Wiggle &amp; Freeze!', Action '第 24 節: 向左向右齊搖擺'. ↔️ 雙手左右擺動，身體快樂起伏！. The character is swaying hips and arms like a breeze, smooth fluid body roll, playful rhythmic dancing, friendly warm smile. 4k resolution, 60fps, Disney Pixar render, joyful preschool music video style.</t>
         </is>
       </c>
+      <c r="K26" s="20" t="inlineStr">
+        <is>
+          <t>images/track_08/a1_s08_seg24_boy.jpg</t>
+        </is>
+      </c>
     </row>
     <row r="27" ht="30" customHeight="1">
       <c r="A27" s="10" t="inlineStr">
@@ -3632,6 +3938,11 @@
           <t>3D Pixar Disney style cheerful toddler dance coach, smooth playful animation, vibrant kindergarten studio, soft bright volumetric lighting, clean studio background, highly expressive face, full body dynamic camera shot: Song 'Wiggle &amp; Freeze!', Action '第 25 節: 盡情釋放活力跳'. ⚡ 雙臂高舉甩動，活力拉滿！. The character is squatting down and bursting into a high happy jump, feet kicking joyfully in mid-air, both fists punching the sky in victory. 4k resolution, 60fps, Disney Pixar render, joyful preschool music video style.</t>
         </is>
       </c>
+      <c r="K27" s="20" t="inlineStr">
+        <is>
+          <t>images/track_08/a1_s08_seg25_boy.jpg</t>
+        </is>
+      </c>
     </row>
     <row r="28" ht="30" customHeight="1">
       <c r="A28" s="8" t="inlineStr">
@@ -3680,6 +3991,11 @@
           <t>3D Pixar Disney style cheerful toddler dance coach, smooth playful animation, vibrant kindergarten studio, soft bright volumetric lighting, clean studio background, highly expressive face, full body dynamic camera shot: Song 'Wiggle &amp; Freeze!', Action '第 26 節: 你完全沒動！你贏了'. 🏆 太厲害啦！你一動都沒動，大獲全勝！. The character is bringing hands together at the chest forming an adorable glowing heart shape, leaning slightly forward, loving gentle smile. 4k resolution, 60fps, Disney Pixar render, joyful preschool music video style.</t>
         </is>
       </c>
+      <c r="K28" s="20" t="inlineStr">
+        <is>
+          <t>images/track_08/a1_s08_seg26_boy.jpg</t>
+        </is>
+      </c>
     </row>
     <row r="29" ht="30" customHeight="1">
       <c r="A29" s="10" t="inlineStr">
@@ -3726,6 +4042,11 @@
       <c r="J29" s="11" t="inlineStr">
         <is>
           <t>3D Pixar Disney style cheerful toddler dance coach, smooth playful animation, vibrant kindergarten studio, soft bright volumetric lighting, clean studio background, highly expressive face, full body dynamic camera shot: Song 'Wiggle &amp; Freeze!', Action '第 27 節: 坐下深呼吸大定格'. 🧘 雙手慢慢撫胸，做個深呼吸，微笑定格！. The character is lifting arms from heart to sky creating a big golden sun circle, chest open, radiant beaming joyful smile. 4k resolution, 60fps, Disney Pixar render, joyful preschool music video style.</t>
+        </is>
+      </c>
+      <c r="K29" s="20" t="inlineStr">
+        <is>
+          <t>images/track_08/a1_s08_seg27_boy.jpg</t>
         </is>
       </c>
     </row>
@@ -3743,7 +4064,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J26"/>
+  <dimension ref="A1:K26"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="18" customWidth="1" min="1" max="1"/>
@@ -3756,6 +4077,7 @@
     <col width="30" customWidth="1" min="8" max="8"/>
     <col width="12" customWidth="1" min="9" max="9"/>
     <col width="55" customWidth="1" min="10" max="10"/>
+    <col width="34" customWidth="1" min="11" max="11"/>
   </cols>
   <sheetData>
     <row r="1" ht="32" customHeight="1">
@@ -3816,6 +4138,11 @@
           <t>AI 影片動畫生成提示詞 (Prompt)</t>
         </is>
       </c>
+      <c r="K2" s="19" t="inlineStr">
+        <is>
+          <t>首張圖片路徑 (9:16 720p)</t>
+        </is>
+      </c>
     </row>
     <row r="3" ht="30" customHeight="1">
       <c r="A3" s="10" t="inlineStr">
@@ -3864,6 +4191,11 @@
           <t>3D Pixar Disney style preschool animation video keyframe, vertical 9:16 aspect ratio 720p HD. Full body standing shot of the cheerful 5-year-old boy dance coach in bright blue athletic t-shirt with orange center and KIDS DANCE logo, blue shorts, orange running sneakers. In colorful kindergarten dance studio. Starter keyframe for action "[前奏] 肚子咕嚕嚕美食預備" (🥣 肚子咕嚕嚕！戴上小廚師帽，健康點心開動囉！). The character is in lively dance starter pose, joyful radiant beaming smile, sparkling expressive eyes. 4k 3D Pixar render, clean frame without text overlay, starter keyframe for image-to-video generation (a1_s09_seg01_boy.jpg).</t>
         </is>
       </c>
+      <c r="K3" s="20" t="inlineStr">
+        <is>
+          <t>images/track_09/a1_s09_seg01_boy.jpg</t>
+        </is>
+      </c>
     </row>
     <row r="4" ht="30" customHeight="1">
       <c r="A4" s="8" t="inlineStr">
@@ -3912,6 +4244,11 @@
           <t>3D Pixar Disney style cheerful toddler dance coach, smooth playful animation, vibrant kindergarten studio, soft bright volumetric lighting, clean studio background, highly expressive face, full body dynamic camera shot: Song 'Yummy Healthy Snack', Action '第 01 節: 脆脆橘色甜胡蘿蔔'. 🥕 雙手拿著胡蘿蔔，喀嚓喀嚓大口咬！. The character is stretching arms up high to reach floating elements, standing on tiptoes, joyful posture, looking up with wonder. 4k resolution, 60fps, Disney Pixar render, joyful preschool music video style.</t>
         </is>
       </c>
+      <c r="K4" s="20" t="inlineStr">
+        <is>
+          <t>images/track_09/a1_s09_seg02_boy.jpg</t>
+        </is>
+      </c>
     </row>
     <row r="5" ht="30" customHeight="1">
       <c r="A5" s="10" t="inlineStr">
@@ -3960,6 +4297,11 @@
           <t>3D Pixar Disney style cheerful toddler dance coach, smooth playful animation, vibrant kindergarten studio, soft bright volumetric lighting, clean studio background, highly expressive face, full body dynamic camera shot: Song 'Yummy Healthy Snack', Action '第 02 節: 綠色花椰菜好好吃'. 🥦 雙手像綠色小樹，嚼一嚼真美味！. The character is swaying hips and arms like a breeze, smooth fluid body roll, playful rhythmic dancing, friendly warm smile. 4k resolution, 60fps, Disney Pixar render, joyful preschool music video style.</t>
         </is>
       </c>
+      <c r="K5" s="20" t="inlineStr">
+        <is>
+          <t>images/track_09/a1_s09_seg03_boy.jpg</t>
+        </is>
+      </c>
     </row>
     <row r="6" ht="30" customHeight="1">
       <c r="A6" s="8" t="inlineStr">
@@ -4008,6 +4350,11 @@
           <t>3D Pixar Disney style cheerful toddler dance coach, smooth playful animation, vibrant kindergarten studio, soft bright volumetric lighting, clean studio background, highly expressive face, full body dynamic camera shot: Song 'Yummy Healthy Snack', Action '第 03 節: 肥皂清水把手洗淨'. 🧼 雙手手心搓搓手背搓搓，洗乾淨！. The character is waving both hands overhead in friendly wide arcs, swaying gently from side to side, sparkling excited eyes. 4k resolution, 60fps, Disney Pixar render, joyful preschool music video style.</t>
         </is>
       </c>
+      <c r="K6" s="20" t="inlineStr">
+        <is>
+          <t>images/track_09/a1_s09_seg04_boy.jpg</t>
+        </is>
+      </c>
     </row>
     <row r="7" ht="30" customHeight="1">
       <c r="A7" s="10" t="inlineStr">
@@ -4056,6 +4403,11 @@
           <t>3D Pixar Disney style cheerful toddler dance coach, smooth playful animation, vibrant kindergarten studio, soft bright volumetric lighting, clean studio background, highly expressive face, full body dynamic camera shot: Song 'Yummy Healthy Snack', Action '第 04 節: 最棒的小廚師登場'. 👨‍🍳 摸摸高高廚師帽，豎起大拇指！. The character is marching in place energetically, hands on hips, knees lifting high in rhythmic bounce, enthusiastic happy smile. 4k resolution, 60fps, Disney Pixar render, joyful preschool music video style.</t>
         </is>
       </c>
+      <c r="K7" s="20" t="inlineStr">
+        <is>
+          <t>images/track_09/a1_s09_seg05_boy.jpg</t>
+        </is>
+      </c>
     </row>
     <row r="8" ht="30" customHeight="1">
       <c r="A8" s="8" t="inlineStr">
@@ -4104,6 +4456,11 @@
           <t>3D Pixar Disney style cheerful toddler dance coach, smooth playful animation, vibrant kindergarten studio, soft bright volumetric lighting, clean studio background, highly expressive face, full body dynamic camera shot: Song 'Yummy Healthy Snack', Action '第 05 節: 咬一小口慢慢嚼'. 🍎 一口一口慢慢咬，細嚼慢嚥最健康！. The character is bringing hands together at the chest forming an adorable glowing heart shape, leaning slightly forward, loving gentle smile. 4k resolution, 60fps, Disney Pixar render, joyful preschool music video style.</t>
         </is>
       </c>
+      <c r="K8" s="20" t="inlineStr">
+        <is>
+          <t>images/track_09/a1_s09_seg06_boy.jpg</t>
+        </is>
+      </c>
     </row>
     <row r="9" ht="30" customHeight="1">
       <c r="A9" s="10" t="inlineStr">
@@ -4152,6 +4509,11 @@
           <t>3D Pixar Disney style cheerful toddler dance coach, smooth playful animation, vibrant kindergarten studio, soft bright volumetric lighting, clean studio background, highly expressive face, full body dynamic camera shot: Song 'Yummy Healthy Snack', Action '第 06 節: 健康食物幫忙長高'. 🌱 雙腳踩直向上拔高，天天長高長壯！. The character is lifting arms from heart to sky creating a big golden sun circle, chest open, radiant beaming joyful smile. 4k resolution, 60fps, Disney Pixar render, joyful preschool music video style.</t>
         </is>
       </c>
+      <c r="K9" s="20" t="inlineStr">
+        <is>
+          <t>images/track_09/a1_s09_seg07_boy.jpg</t>
+        </is>
+      </c>
     </row>
     <row r="10" ht="30" customHeight="1">
       <c r="A10" s="8" t="inlineStr">
@@ -4200,6 +4562,11 @@
           <t>3D Pixar Disney style cheerful toddler dance coach, smooth playful animation, vibrant kindergarten studio, soft bright volumetric lighting, clean studio background, highly expressive face, full body dynamic camera shot: Song 'Yummy Healthy Snack', Action '第 07 節: 阿姆阿姆大口嚼'. 😋 雙手摸肚肚，嘴巴嚼呀嚼真香！. The character is marching in place energetically, hands on hips, knees lifting high in rhythmic bounce, enthusiastic happy smile. 4k resolution, 60fps, Disney Pixar render, joyful preschool music video style.</t>
         </is>
       </c>
+      <c r="K10" s="20" t="inlineStr">
+        <is>
+          <t>images/track_09/a1_s09_seg08_boy.jpg</t>
+        </is>
+      </c>
     </row>
     <row r="11" ht="30" customHeight="1">
       <c r="A11" s="10" t="inlineStr">
@@ -4248,6 +4615,11 @@
           <t>3D Pixar Disney style cheerful toddler dance coach, smooth playful animation, vibrant kindergarten studio, soft bright volumetric lighting, clean studio background, highly expressive face, full body dynamic camera shot: Song 'Yummy Healthy Snack', Action '第 08 節: 營養食物身體棒'. 💪 雙臂展示小肌肉，身體強壯壯！. The character is squatting down and bursting into a high happy jump, feet kicking joyfully in mid-air, both fists punching the sky in victory. 4k resolution, 60fps, Disney Pixar render, joyful preschool music video style.</t>
         </is>
       </c>
+      <c r="K11" s="20" t="inlineStr">
+        <is>
+          <t>images/track_09/a1_s09_seg09_boy.jpg</t>
+        </is>
+      </c>
     </row>
     <row r="12" ht="30" customHeight="1">
       <c r="A12" s="8" t="inlineStr">
@@ -4296,6 +4668,11 @@
           <t>3D Pixar Disney style cheerful toddler dance coach, smooth playful animation, vibrant kindergarten studio, soft bright volumetric lighting, clean studio background, highly expressive face, full body dynamic camera shot: Song 'Yummy Healthy Snack', Action '第 09 節: 盤子盛滿蔬果盤'. 🥗 雙手在胸前端起五彩繽紛蔬果盤！. The character is stretching arms up high to reach floating elements, standing on tiptoes, joyful posture, looking up with wonder. 4k resolution, 60fps, Disney Pixar render, joyful preschool music video style.</t>
         </is>
       </c>
+      <c r="K12" s="20" t="inlineStr">
+        <is>
+          <t>images/track_09/a1_s09_seg10_boy.jpg</t>
+        </is>
+      </c>
     </row>
     <row r="13" ht="30" customHeight="1">
       <c r="A13" s="10" t="inlineStr">
@@ -4344,6 +4721,11 @@
           <t>3D Pixar Disney style cheerful toddler dance coach, smooth playful animation, vibrant kindergarten studio, soft bright volumetric lighting, clean studio background, highly expressive face, full body dynamic camera shot: Song 'Yummy Healthy Snack', Action '第 10 節: 吃下彩虹身體好棒'. 🌈 雙臂在空中畫出大彩虹，精神好！. The character is lifting arms from heart to sky creating a big golden sun circle, chest open, radiant beaming joyful smile. 4k resolution, 60fps, Disney Pixar render, joyful preschool music video style.</t>
         </is>
       </c>
+      <c r="K13" s="20" t="inlineStr">
+        <is>
+          <t>images/track_09/a1_s09_seg11_boy.jpg</t>
+        </is>
+      </c>
     </row>
     <row r="14" ht="30" customHeight="1">
       <c r="A14" s="8" t="inlineStr">
@@ -4392,6 +4774,11 @@
           <t>3D Pixar Disney style cheerful toddler dance coach, smooth playful animation, vibrant kindergarten studio, soft bright volumetric lighting, clean studio background, highly expressive face, full body dynamic camera shot: Song 'Yummy Healthy Snack', Action '[旋律間奏] 動作接續歡樂跳'. 🔄 雙手插腰踩小碎步，轉個歡樂大圓圈，保持微笑！. The character is swaying hips and arms like a breeze, smooth fluid body roll, playful rhythmic dancing, friendly warm smile. 4k resolution, 60fps, Disney Pixar render, joyful preschool music video style.</t>
         </is>
       </c>
+      <c r="K14" s="20" t="inlineStr">
+        <is>
+          <t>images/track_09/a1_s09_seg12_boy.jpg</t>
+        </is>
+      </c>
     </row>
     <row r="15" ht="30" customHeight="1">
       <c r="A15" s="10" t="inlineStr">
@@ -4440,6 +4827,11 @@
           <t>3D Pixar Disney style cheerful toddler dance coach, smooth playful animation, vibrant kindergarten studio, soft bright volumetric lighting, clean studio background, highly expressive face, full body dynamic camera shot: Song 'Yummy Healthy Snack', Action '第 11 節: 紅紅蘋果香蕉笑臉'. 🍌 雙手托起紅蘋果，嘴角揚起香蕉大笑！. The character is bringing hands together at the chest forming an adorable glowing heart shape, leaning slightly forward, loving gentle smile. 4k resolution, 60fps, Disney Pixar render, joyful preschool music video style.</t>
         </is>
       </c>
+      <c r="K15" s="20" t="inlineStr">
+        <is>
+          <t>images/track_09/a1_s09_seg13_boy.jpg</t>
+        </is>
+      </c>
     </row>
     <row r="16" ht="30" customHeight="1">
       <c r="A16" s="8" t="inlineStr">
@@ -4488,6 +4880,11 @@
           <t>3D Pixar Disney style cheerful toddler dance coach, smooth playful animation, vibrant kindergarten studio, soft bright volumetric lighting, clean studio background, highly expressive face, full body dynamic camera shot: Song 'Yummy Healthy Snack', Action '第 12 節: 喝杯牛奶歇一歇'. 🥛 雙手捧杯咕嚕咕嚕喝牛奶，休息一下！. The character is marching in place energetically, hands on hips, knees lifting high in rhythmic bounce, enthusiastic happy smile. 4k resolution, 60fps, Disney Pixar render, joyful preschool music video style.</t>
         </is>
       </c>
+      <c r="K16" s="20" t="inlineStr">
+        <is>
+          <t>images/track_09/a1_s09_seg14_boy.jpg</t>
+        </is>
+      </c>
     </row>
     <row r="17" ht="30" customHeight="1">
       <c r="A17" s="10" t="inlineStr">
@@ -4536,6 +4933,11 @@
           <t>3D Pixar Disney style cheerful toddler dance coach, smooth playful animation, vibrant kindergarten studio, soft bright volumetric lighting, clean studio background, highly expressive face, full body dynamic camera shot: Song 'Yummy Healthy Snack', Action '第 13 節: 碗裡草莓閃亮亮'. 🍓 伸手進碗裡抓一把小草莓放嘴裡！. The character is stretching arms up high to reach floating elements, standing on tiptoes, joyful posture, looking up with wonder. 4k resolution, 60fps, Disney Pixar render, joyful preschool music video style.</t>
         </is>
       </c>
+      <c r="K17" s="20" t="inlineStr">
+        <is>
+          <t>images/track_09/a1_s09_seg15_boy.jpg</t>
+        </is>
+      </c>
     </row>
     <row r="18" ht="30" customHeight="1">
       <c r="A18" s="8" t="inlineStr">
@@ -4584,6 +4986,11 @@
           <t>3D Pixar Disney style cheerful toddler dance coach, smooth playful animation, vibrant kindergarten studio, soft bright volumetric lighting, clean studio background, highly expressive face, full body dynamic camera shot: Song 'Yummy Healthy Snack', Action '第 14 節: 健康點心營養滿分'. ⭐ 拍拍雙手，全身元氣滿滿！. The character is waving both hands overhead in friendly wide arcs, swaying gently from side to side, sparkling excited eyes. 4k resolution, 60fps, Disney Pixar render, joyful preschool music video style.</t>
         </is>
       </c>
+      <c r="K18" s="20" t="inlineStr">
+        <is>
+          <t>images/track_09/a1_s09_seg16_boy.jpg</t>
+        </is>
+      </c>
     </row>
     <row r="19" ht="30" customHeight="1">
       <c r="A19" s="10" t="inlineStr">
@@ -4632,6 +5039,11 @@
           <t>3D Pixar Disney style cheerful toddler dance coach, smooth playful animation, vibrant kindergarten studio, soft bright volumetric lighting, clean studio background, highly expressive face, full body dynamic camera shot: Song 'Yummy Healthy Snack', Action '第 15 節: 揉揉肚肚說好好吃'. 😋 雙手揉揉圓滾滾肚肚，說聲好好吃！. The character is swaying hips and arms like a breeze, smooth fluid body roll, playful rhythmic dancing, friendly warm smile. 4k resolution, 60fps, Disney Pixar render, joyful preschool music video style.</t>
         </is>
       </c>
+      <c r="K19" s="20" t="inlineStr">
+        <is>
+          <t>images/track_09/a1_s09_seg17_boy.jpg</t>
+        </is>
+      </c>
     </row>
     <row r="20" ht="30" customHeight="1">
       <c r="A20" s="8" t="inlineStr">
@@ -4680,6 +5092,11 @@
           <t>3D Pixar Disney style cheerful toddler dance coach, smooth playful animation, vibrant kindergarten studio, soft bright volumetric lighting, clean studio background, highly expressive face, full body dynamic camera shot: Song 'Yummy Healthy Snack', Action '第 16 節: 滿滿活力玩遊戲'. 🏃 雙腳原地快速跑動，隨時去玩耍！. The character is marching in place energetically, hands on hips, knees lifting high in rhythmic bounce, enthusiastic happy smile. 4k resolution, 60fps, Disney Pixar render, joyful preschool music video style.</t>
         </is>
       </c>
+      <c r="K20" s="20" t="inlineStr">
+        <is>
+          <t>images/track_09/a1_s09_seg18_boy.jpg</t>
+        </is>
+      </c>
     </row>
     <row r="21" ht="30" customHeight="1">
       <c r="A21" s="10" t="inlineStr">
@@ -4728,6 +5145,11 @@
           <t>3D Pixar Disney style cheerful toddler dance coach, smooth playful animation, vibrant kindergarten studio, soft bright volumetric lighting, clean studio background, highly expressive face, full body dynamic camera shot: Song 'Yummy Healthy Snack', Action '第 17 節: 阿姆阿姆大口嚼'. 🍽️ 跟著節奏大口大口吃點心！. The character is marching in place energetically, hands on hips, knees lifting high in rhythmic bounce, enthusiastic happy smile. 4k resolution, 60fps, Disney Pixar render, joyful preschool music video style.</t>
         </is>
       </c>
+      <c r="K21" s="20" t="inlineStr">
+        <is>
+          <t>images/track_09/a1_s09_seg19_boy.jpg</t>
+        </is>
+      </c>
     </row>
     <row r="22" ht="30" customHeight="1">
       <c r="A22" s="8" t="inlineStr">
@@ -4776,6 +5198,11 @@
           <t>3D Pixar Disney style cheerful toddler dance coach, smooth playful animation, vibrant kindergarten studio, soft bright volumetric lighting, clean studio background, highly expressive face, full body dynamic camera shot: Song 'Yummy Healthy Snack', Action '第 18 節: 健康食物最美味'. 💪 雙臂再次展現健康活力！. The character is squatting down and bursting into a high happy jump, feet kicking joyfully in mid-air, both fists punching the sky in victory. 4k resolution, 60fps, Disney Pixar render, joyful preschool music video style.</t>
         </is>
       </c>
+      <c r="K22" s="20" t="inlineStr">
+        <is>
+          <t>images/track_09/a1_s09_seg20_boy.jpg</t>
+        </is>
+      </c>
     </row>
     <row r="23" ht="30" customHeight="1">
       <c r="A23" s="10" t="inlineStr">
@@ -4824,6 +5251,11 @@
           <t>3D Pixar Disney style cheerful toddler dance coach, smooth playful animation, vibrant kindergarten studio, soft bright volumetric lighting, clean studio background, highly expressive face, full body dynamic camera shot: Song 'Yummy Healthy Snack', Action '第 19 節: 蔬果吃光盤子空'. 🥗 把蔬菜水果吃光光，營養好寶寶！. The character is stretching arms up high to reach floating elements, standing on tiptoes, joyful posture, looking up with wonder. 4k resolution, 60fps, Disney Pixar render, joyful preschool music video style.</t>
         </is>
       </c>
+      <c r="K23" s="20" t="inlineStr">
+        <is>
+          <t>images/track_09/a1_s09_seg21_boy.jpg</t>
+        </is>
+      </c>
     </row>
     <row r="24" ht="30" customHeight="1">
       <c r="A24" s="8" t="inlineStr">
@@ -4872,6 +5304,11 @@
           <t>3D Pixar Disney style cheerful toddler dance coach, smooth playful animation, vibrant kindergarten studio, soft bright volumetric lighting, clean studio background, highly expressive face, full body dynamic camera shot: Song 'Yummy Healthy Snack', Action '第 20 節: 彩色營養能量足'. ✨ 雙手向上綻放金色光芒！. The character is lifting arms from heart to sky creating a big golden sun circle, chest open, radiant beaming joyful smile. 4k resolution, 60fps, Disney Pixar render, joyful preschool music video style.</t>
         </is>
       </c>
+      <c r="K24" s="20" t="inlineStr">
+        <is>
+          <t>images/track_09/a1_s09_seg22_boy.jpg</t>
+        </is>
+      </c>
     </row>
     <row r="25" ht="30" customHeight="1">
       <c r="A25" s="10" t="inlineStr">
@@ -4920,6 +5357,11 @@
           <t>3D Pixar Disney style cheerful toddler dance coach, smooth playful animation, vibrant kindergarten studio, soft bright volumetric lighting, clean studio background, highly expressive face, full body dynamic camera shot: Song 'Yummy Healthy Snack', Action '第 21 節: 全吃完啦太美味'. 👏 拍拍小手舔舔嘴唇，美味滿分！. The character is bringing hands together at the chest forming an adorable glowing heart shape, leaning slightly forward, loving gentle smile. 4k resolution, 60fps, Disney Pixar render, joyful preschool music video style.</t>
         </is>
       </c>
+      <c r="K25" s="20" t="inlineStr">
+        <is>
+          <t>images/track_09/a1_s09_seg23_boy.jpg</t>
+        </is>
+      </c>
     </row>
     <row r="26" ht="30" customHeight="1">
       <c r="A26" s="8" t="inlineStr">
@@ -4966,6 +5408,11 @@
       <c r="J26" s="9" t="inlineStr">
         <is>
           <t>3D Pixar Disney style cheerful toddler dance coach, smooth playful animation, vibrant kindergarten studio, soft bright volumetric lighting, clean studio background, highly expressive face, full body dynamic camera shot: Song 'Yummy Healthy Snack', Action '第 22 節: 謝謝美味健康點心'. 🙏 雙手合十胸前鞠躬，定格感恩大微笑！. The character is lifting arms from heart to sky creating a big golden sun circle, chest open, radiant beaming joyful smile. 4k resolution, 60fps, Disney Pixar render, joyful preschool music video style.</t>
+        </is>
+      </c>
+      <c r="K26" s="20" t="inlineStr">
+        <is>
+          <t>images/track_09/a1_s09_seg24_boy.jpg</t>
         </is>
       </c>
     </row>
@@ -4983,7 +5430,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J23"/>
+  <dimension ref="A1:K23"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="18" customWidth="1" min="1" max="1"/>
@@ -4996,6 +5443,7 @@
     <col width="30" customWidth="1" min="8" max="8"/>
     <col width="12" customWidth="1" min="9" max="9"/>
     <col width="55" customWidth="1" min="10" max="10"/>
+    <col width="34" customWidth="1" min="11" max="11"/>
   </cols>
   <sheetData>
     <row r="1" ht="32" customHeight="1">
@@ -5056,6 +5504,11 @@
           <t>AI 影片動畫生成提示詞 (Prompt)</t>
         </is>
       </c>
+      <c r="K2" s="19" t="inlineStr">
+        <is>
+          <t>首張圖片路徑 (9:16 720p)</t>
+        </is>
+      </c>
     </row>
     <row r="3" ht="30" customHeight="1">
       <c r="A3" s="10" t="inlineStr">
@@ -5104,6 +5557,11 @@
           <t>3D Pixar Disney style preschool animation video keyframe, vertical 9:16 aspect ratio 720p HD. Full body standing shot of the cheerful 5-year-old girl dance coach with brown curly pigtails tied with yellow ribbons, pink dance tee with smiling yellow star, yellow shorts, pink sneakers. In colorful kindergarten dance studio. Starter keyframe for action "[前奏] 夜幕低垂搖籃曲" (🌙 月亮升起，微風吹拂，輕輕左右搖擺放鬆身體！). The character is in lively dance starter pose, joyful radiant beaming smile, sparkling expressive eyes. 4k 3D Pixar render, clean frame without text overlay, starter keyframe for image-to-video generation (a1_s10_seg01_girl.jpg).</t>
         </is>
       </c>
+      <c r="K3" s="20" t="inlineStr">
+        <is>
+          <t>images/track_10/a1_s10_seg01_girl.jpg</t>
+        </is>
+      </c>
     </row>
     <row r="4" ht="30" customHeight="1">
       <c r="A4" s="8" t="inlineStr">
@@ -5152,6 +5610,11 @@
           <t>3D Pixar Disney style cheerful toddler dance coach, smooth playful animation, vibrant kindergarten studio, soft bright volumetric lighting, clean studio background, highly expressive face, full body dynamic camera shot: Song 'Soft Pillow Goodnight', Action '第 01 節: 閉上雙眼日光落'. 🌅 雙手在眼前輕輕抹過，溫柔閉上雙眼！. The character is stretching arms up high to reach floating elements, standing on tiptoes, joyful posture, looking up with wonder. 4k resolution, 60fps, Disney Pixar render, joyful preschool music video style.</t>
         </is>
       </c>
+      <c r="K4" s="20" t="inlineStr">
+        <is>
+          <t>images/track_10/a1_s10_seg02_girl.jpg</t>
+        </is>
+      </c>
     </row>
     <row r="5" ht="30" customHeight="1">
       <c r="A5" s="10" t="inlineStr">
@@ -5200,6 +5663,11 @@
           <t>3D Pixar Disney style cheerful toddler dance coach, smooth playful animation, vibrant kindergarten studio, soft bright volumetric lighting, clean studio background, highly expressive face, full body dynamic camera shot: Song 'Soft Pillow Goodnight', Action '第 02 節: 太陽身後靜靜歇'. ☀️ 雙手慢慢下落，像夕陽落到山後！. The character is swaying hips and arms like a breeze, smooth fluid body roll, playful rhythmic dancing, friendly warm smile. 4k resolution, 60fps, Disney Pixar render, joyful preschool music video style.</t>
         </is>
       </c>
+      <c r="K5" s="20" t="inlineStr">
+        <is>
+          <t>images/track_10/a1_s10_seg03_girl.jpg</t>
+        </is>
+      </c>
     </row>
     <row r="6" ht="30" customHeight="1">
       <c r="A6" s="8" t="inlineStr">
@@ -5248,6 +5716,11 @@
           <t>3D Pixar Disney style cheerful toddler dance coach, smooth playful animation, vibrant kindergarten studio, soft bright volumetric lighting, clean studio background, highly expressive face, full body dynamic camera shot: Song 'Soft Pillow Goodnight', Action '第 03 節: 紫夜繁星眨眼睛'. ⭐ 雙手抬至夜空，小手指如星星眨眼！. The character is lifting arms from heart to sky creating a big golden sun circle, chest open, radiant beaming joyful smile. 4k resolution, 60fps, Disney Pixar render, joyful preschool music video style.</t>
         </is>
       </c>
+      <c r="K6" s="20" t="inlineStr">
+        <is>
+          <t>images/track_10/a1_s10_seg04_girl.jpg</t>
+        </is>
+      </c>
     </row>
     <row r="7" ht="30" customHeight="1">
       <c r="A7" s="10" t="inlineStr">
@@ -5296,6 +5769,11 @@
           <t>3D Pixar Disney style cheerful toddler dance coach, smooth playful animation, vibrant kindergarten studio, soft bright volumetric lighting, clean studio background, highly expressive face, full body dynamic camera shot: Song 'Soft Pillow Goodnight', Action '第 05 節: 小熊緊抱在胸前'. 🧸 雙臂胸前緊緊抱住心愛的小熊玩偶！. The character is bringing hands together at the chest forming an adorable glowing heart shape, leaning slightly forward, loving gentle smile. 4k resolution, 60fps, Disney Pixar render, joyful preschool music video style.</t>
         </is>
       </c>
+      <c r="K7" s="20" t="inlineStr">
+        <is>
+          <t>images/track_10/a1_s10_seg05_girl.jpg</t>
+        </is>
+      </c>
     </row>
     <row r="8" ht="30" customHeight="1">
       <c r="A8" s="8" t="inlineStr">
@@ -5344,6 +5822,11 @@
           <t>3D Pixar Disney style cheerful toddler dance coach, smooth playful animation, vibrant kindergarten studio, soft bright volumetric lighting, clean studio background, highly expressive face, full body dynamic camera shot: Song 'Soft Pillow Goodnight', Action '第 06 節: 疲憊雙眼歇一歇'. 😴 雙手合十貼在右臉頰，輕輕閉目！. The character is stretching arms up high to reach floating elements, standing on tiptoes, joyful posture, looking up with wonder. 4k resolution, 60fps, Disney Pixar render, joyful preschool music video style.</t>
         </is>
       </c>
+      <c r="K8" s="20" t="inlineStr">
+        <is>
+          <t>images/track_10/a1_s10_seg06_girl.jpg</t>
+        </is>
+      </c>
     </row>
     <row r="9" ht="30" customHeight="1">
       <c r="A9" s="10" t="inlineStr">
@@ -5392,6 +5875,11 @@
           <t>3D Pixar Disney style cheerful toddler dance coach, smooth playful animation, vibrant kindergarten studio, soft bright volumetric lighting, clean studio background, highly expressive face, full body dynamic camera shot: Song 'Soft Pillow Goodnight', Action '第 07 節: 安睡吧小腦袋'. 🛏️ 頭部輕靠在左側枕頭，身體放鬆！. The character is swaying hips and arms like a breeze, smooth fluid body roll, playful rhythmic dancing, friendly warm smile. 4k resolution, 60fps, Disney Pixar render, joyful preschool music video style.</t>
         </is>
       </c>
+      <c r="K9" s="20" t="inlineStr">
+        <is>
+          <t>images/track_10/a1_s10_seg07_girl.jpg</t>
+        </is>
+      </c>
     </row>
     <row r="10" ht="30" customHeight="1">
       <c r="A10" s="8" t="inlineStr">
@@ -5440,6 +5928,11 @@
           <t>3D Pixar Disney style cheerful toddler dance coach, smooth playful animation, vibrant kindergarten studio, soft bright volumetric lighting, clean studio background, highly expressive face, full body dynamic camera shot: Song 'Soft Pillow Goodnight', Action '第 08 節: 柔軟被窩好溫暖'. 🛌 雙手向上拉起被角，縮進溫暖被窩！. The character is bringing hands together at the chest forming an adorable glowing heart shape, leaning slightly forward, loving gentle smile. 4k resolution, 60fps, Disney Pixar render, joyful preschool music video style.</t>
         </is>
       </c>
+      <c r="K10" s="20" t="inlineStr">
+        <is>
+          <t>images/track_10/a1_s10_seg08_girl.jpg</t>
+        </is>
+      </c>
     </row>
     <row r="11" ht="30" customHeight="1">
       <c r="A11" s="10" t="inlineStr">
@@ -5488,6 +5981,11 @@
           <t>3D Pixar Disney style cheerful toddler dance coach, smooth playful animation, vibrant kindergarten studio, soft bright volumetric lighting, clean studio background, highly expressive face, full body dynamic camera shot: Song 'Soft Pillow Goodnight', Action '第 09 節: 雲朵之上輕漂浮'. ☁️ 雙臂平展，身體像在雲朵上漂浮！. The character is swaying hips and arms like a breeze, smooth fluid body roll, playful rhythmic dancing, friendly warm smile. 4k resolution, 60fps, Disney Pixar render, joyful preschool music video style.</t>
         </is>
       </c>
+      <c r="K11" s="20" t="inlineStr">
+        <is>
+          <t>images/track_10/a1_s10_seg09_girl.jpg</t>
+        </is>
+      </c>
     </row>
     <row r="12" ht="30" customHeight="1">
       <c r="A12" s="8" t="inlineStr">
@@ -5536,6 +6034,11 @@
           <t>3D Pixar Disney style cheerful toddler dance coach, smooth playful animation, vibrant kindergarten studio, soft bright volumetric lighting, clean studio background, highly expressive face, full body dynamic camera shot: Song 'Soft Pillow Goodnight', Action '第 10 節: 小天使晚安好夢'. 👼 雙手在胸口化作小翅膀輕拍，晚安！. The character is bringing hands together at the chest forming an adorable glowing heart shape, leaning slightly forward, loving gentle smile. 4k resolution, 60fps, Disney Pixar render, joyful preschool music video style.</t>
         </is>
       </c>
+      <c r="K12" s="20" t="inlineStr">
+        <is>
+          <t>images/track_10/a1_s10_seg10_girl.jpg</t>
+        </is>
+      </c>
     </row>
     <row r="13" ht="30" customHeight="1">
       <c r="A13" s="10" t="inlineStr">
@@ -5584,6 +6087,11 @@
           <t>3D Pixar Disney style cheerful toddler dance coach, smooth playful animation, vibrant kindergarten studio, soft bright volumetric lighting, clean studio background, highly expressive face, full body dynamic camera shot: Song 'Soft Pillow Goodnight', Action '第 11 節: 月光透過窗櫺照'. 🌕 抬頭望向窗外銀色月光，手撫窗櫺！. The character is stretching arms up high to reach floating elements, standing on tiptoes, joyful posture, looking up with wonder. 4k resolution, 60fps, Disney Pixar render, joyful preschool music video style.</t>
         </is>
       </c>
+      <c r="K13" s="20" t="inlineStr">
+        <is>
+          <t>images/track_10/a1_s10_seg11_girl.jpg</t>
+        </is>
+      </c>
     </row>
     <row r="14" ht="30" customHeight="1">
       <c r="A14" s="8" t="inlineStr">
@@ -5632,6 +6140,11 @@
           <t>3D Pixar Disney style cheerful toddler dance coach, smooth playful animation, vibrant kindergarten studio, soft bright volumetric lighting, clean studio background, highly expressive face, full body dynamic camera shot: Song 'Soft Pillow Goodnight', Action '第 12 節: 銀色雨滴小巷跳'. 💧 手指輕柔如細雨從空中緩緩落下！. The character is waving both hands overhead in friendly wide arcs, swaying gently from side to side, sparkling excited eyes. 4k resolution, 60fps, Disney Pixar render, joyful preschool music video style.</t>
         </is>
       </c>
+      <c r="K14" s="20" t="inlineStr">
+        <is>
+          <t>images/track_10/a1_s10_seg12_girl.jpg</t>
+        </is>
+      </c>
     </row>
     <row r="15" ht="30" customHeight="1">
       <c r="A15" s="10" t="inlineStr">
@@ -5680,6 +6193,11 @@
           <t>3D Pixar Disney style cheerful toddler dance coach, smooth playful animation, vibrant kindergarten studio, soft bright volumetric lighting, clean studio background, highly expressive face, full body dynamic camera shot: Song 'Soft Pillow Goodnight', Action '第 13 節: 快樂思緒飄入夢'. 💭 雙手由胸前向外輕撫，放飛好夢！. The character is stretching arms up high to reach floating elements, standing on tiptoes, joyful posture, looking up with wonder. 4k resolution, 60fps, Disney Pixar render, joyful preschool music video style.</t>
         </is>
       </c>
+      <c r="K15" s="20" t="inlineStr">
+        <is>
+          <t>images/track_10/a1_s10_seg13_girl.jpg</t>
+        </is>
+      </c>
     </row>
     <row r="16" ht="30" customHeight="1">
       <c r="A16" s="8" t="inlineStr">
@@ -5728,6 +6246,11 @@
           <t>3D Pixar Disney style cheerful toddler dance coach, smooth playful animation, vibrant kindergarten studio, soft bright volumetric lighting, clean studio background, highly expressive face, full body dynamic camera shot: Song 'Soft Pillow Goodnight', Action '第 14 節: 數數跳跳毛毛羊'. 🐑 食指輕輕點數：一隻羊、兩隻羊.... The character is stretching arms up high to reach floating elements, standing on tiptoes, joyful posture, looking up with wonder. 4k resolution, 60fps, Disney Pixar render, joyful preschool music video style.</t>
         </is>
       </c>
+      <c r="K16" s="20" t="inlineStr">
+        <is>
+          <t>images/track_10/a1_s10_seg14_girl.jpg</t>
+        </is>
+      </c>
     </row>
     <row r="17" ht="30" customHeight="1">
       <c r="A17" s="10" t="inlineStr">
@@ -5776,6 +6299,11 @@
           <t>3D Pixar Disney style cheerful toddler dance coach, smooth playful animation, vibrant kindergarten studio, soft bright volumetric lighting, clean studio background, highly expressive face, full body dynamic camera shot: Song 'Soft Pillow Goodnight', Action '第 15 節: 明天晴天再來玩'. ☀️ 嘴角泛起微笑，期待明天的晴朗！. The character is lifting arms from heart to sky creating a big golden sun circle, chest open, radiant beaming joyful smile. 4k resolution, 60fps, Disney Pixar render, joyful preschool music video style.</t>
         </is>
       </c>
+      <c r="K17" s="20" t="inlineStr">
+        <is>
+          <t>images/track_10/a1_s10_seg15_girl.jpg</t>
+        </is>
+      </c>
     </row>
     <row r="18" ht="30" customHeight="1">
       <c r="A18" s="8" t="inlineStr">
@@ -5824,6 +6352,11 @@
           <t>3D Pixar Disney style cheerful toddler dance coach, smooth playful animation, vibrant kindergarten studio, soft bright volumetric lighting, clean studio background, highly expressive face, full body dynamic camera shot: Song 'Soft Pillow Goodnight', Action '第 16 節: 夢幻泡泡飛向遠'. 🎈 雙手輕輕吹出夢想泡泡，隨風飛走！. The character is waving both hands overhead in friendly wide arcs, swaying gently from side to side, sparkling excited eyes. 4k resolution, 60fps, Disney Pixar render, joyful preschool music video style.</t>
         </is>
       </c>
+      <c r="K18" s="20" t="inlineStr">
+        <is>
+          <t>images/track_10/a1_s10_seg16_girl.jpg</t>
+        </is>
+      </c>
     </row>
     <row r="19" ht="30" customHeight="1">
       <c r="A19" s="10" t="inlineStr">
@@ -5872,6 +6405,11 @@
           <t>3D Pixar Disney style cheerful toddler dance coach, smooth playful animation, vibrant kindergarten studio, soft bright volumetric lighting, clean studio background, highly expressive face, full body dynamic camera shot: Song 'Soft Pillow Goodnight', Action '第 17 節: 安睡吧小腦袋'. 😴 雙手再次合十貼在臉頰，輕輕搖曳！. The character is swaying hips and arms like a breeze, smooth fluid body roll, playful rhythmic dancing, friendly warm smile. 4k resolution, 60fps, Disney Pixar render, joyful preschool music video style.</t>
         </is>
       </c>
+      <c r="K19" s="20" t="inlineStr">
+        <is>
+          <t>images/track_10/a1_s10_seg17_girl.jpg</t>
+        </is>
+      </c>
     </row>
     <row r="20" ht="30" customHeight="1">
       <c r="A20" s="8" t="inlineStr">
@@ -5920,6 +6458,11 @@
           <t>3D Pixar Disney style cheerful toddler dance coach, smooth playful animation, vibrant kindergarten studio, soft bright volumetric lighting, clean studio background, highly expressive face, full body dynamic camera shot: Song 'Soft Pillow Goodnight', Action '第 18 節: 柔軟被窩好安全'. 🛌 雙手收於胸前，感受平靜與安穩！. The character is bringing hands together at the chest forming an adorable glowing heart shape, leaning slightly forward, loving gentle smile. 4k resolution, 60fps, Disney Pixar render, joyful preschool music video style.</t>
         </is>
       </c>
+      <c r="K20" s="20" t="inlineStr">
+        <is>
+          <t>images/track_10/a1_s10_seg18_girl.jpg</t>
+        </is>
+      </c>
     </row>
     <row r="21" ht="30" customHeight="1">
       <c r="A21" s="10" t="inlineStr">
@@ -5968,6 +6511,11 @@
           <t>3D Pixar Disney style cheerful toddler dance coach, smooth playful animation, vibrant kindergarten studio, soft bright volumetric lighting, clean studio background, highly expressive face, full body dynamic camera shot: Song 'Soft Pillow Goodnight', Action '第 19 節: 雲朵之上軟綿綿'. ☁️ 身體緩緩微晃，像睡在羽毛雲朵上！. The character is swaying hips and arms like a breeze, smooth fluid body roll, playful rhythmic dancing, friendly warm smile. 4k resolution, 60fps, Disney Pixar render, joyful preschool music video style.</t>
         </is>
       </c>
+      <c r="K21" s="20" t="inlineStr">
+        <is>
+          <t>images/track_10/a1_s10_seg19_girl.jpg</t>
+        </is>
+      </c>
     </row>
     <row r="22" ht="30" customHeight="1">
       <c r="A22" s="8" t="inlineStr">
@@ -6016,6 +6564,11 @@
           <t>3D Pixar Disney style cheerful toddler dance coach, smooth playful animation, vibrant kindergarten studio, soft bright volumetric lighting, clean studio background, highly expressive face, full body dynamic camera shot: Song 'Soft Pillow Goodnight', Action '第 20 節: 甜美夢鄉祝晚安'. 🌟 雙手合十胸前，輕輕定格，祝大家晚安！. The character is bringing hands together at the chest forming an adorable glowing heart shape, leaning slightly forward, loving gentle smile. 4k resolution, 60fps, Disney Pixar render, joyful preschool music video style.</t>
         </is>
       </c>
+      <c r="K22" s="20" t="inlineStr">
+        <is>
+          <t>images/track_10/a1_s10_seg20_girl.jpg</t>
+        </is>
+      </c>
     </row>
     <row r="23" ht="30" customHeight="1">
       <c r="A23" s="10" t="inlineStr">
@@ -6062,6 +6615,11 @@
       <c r="J23" s="11" t="inlineStr">
         <is>
           <t>3D Pixar Disney style cheerful toddler dance coach, smooth playful animation, vibrant kindergarten studio, soft bright volumetric lighting, clean studio background, highly expressive face, full body dynamic camera shot: Song 'Soft Pillow Goodnight', Action '第 21 節: 甜美夢鄉祝晚安'. 🌟 雙手合十胸前，輕輕定格，祝大家晚安！. The character is bringing hands together at the chest forming an adorable glowing heart shape, leaning slightly forward, loving gentle smile. 4k resolution, 60fps, Disney Pixar render, joyful preschool music video style.</t>
+        </is>
+      </c>
+      <c r="K23" s="20" t="inlineStr">
+        <is>
+          <t>images/track_10/a1_s10_seg21_girl.jpg</t>
         </is>
       </c>
     </row>
@@ -6079,613 +6637,716 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J12"/>
+  <dimension ref="A1:L12"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="8" customWidth="1" min="1" max="1"/>
     <col width="24" customWidth="1" min="2" max="2"/>
     <col width="18" customWidth="1" min="3" max="3"/>
     <col width="16" customWidth="1" min="4" max="4"/>
-    <col width="22" customWidth="1" min="5" max="5"/>
-    <col width="24" customWidth="1" min="6" max="6"/>
-    <col width="16" customWidth="1" min="7" max="7"/>
-    <col width="28" customWidth="1" min="8" max="8"/>
-    <col width="12" customWidth="1" min="9" max="9"/>
-    <col width="45" customWidth="1" min="10" max="10"/>
+    <col width="12" customWidth="1" min="5" max="5"/>
+    <col width="20" customWidth="1" min="6" max="6"/>
+    <col width="24" customWidth="1" min="7" max="7"/>
+    <col width="32" customWidth="1" min="8" max="8"/>
+    <col width="38" customWidth="1" min="9" max="9"/>
+    <col width="16" customWidth="1" min="10" max="10"/>
+    <col width="12" customWidth="1" min="11" max="11"/>
+    <col width="45" customWidth="1" min="12" max="12"/>
   </cols>
   <sheetData>
     <row r="1" ht="36" customHeight="1">
       <c r="A1" s="14" t="inlineStr">
         <is>
-          <t>🎬 KaiDance 第一輯《小小腳步 大大世界》各曲目動畫第一張圖片 (9:16 720p 圖生影片起始幀) 規格表</t>
+          <t>🎬 KaiDance 第一輯《小小腳步 大大世界》各曲目動畫首張圖片規格表 (9:16 720p 分目錄儲存架構)</t>
         </is>
       </c>
     </row>
     <row r="2" ht="28" customHeight="1">
-      <c r="A2" s="15" t="inlineStr">
+      <c r="A2" s="21" t="inlineStr">
         <is>
           <t>曲目</t>
         </is>
       </c>
-      <c r="B2" s="15" t="inlineStr">
+      <c r="B2" s="21" t="inlineStr">
         <is>
           <t>英文歌名</t>
         </is>
       </c>
-      <c r="C2" s="15" t="inlineStr">
+      <c r="C2" s="21" t="inlineStr">
         <is>
           <t>中文主題</t>
         </is>
       </c>
-      <c r="D2" s="15" t="inlineStr">
+      <c r="D2" s="21" t="inlineStr">
         <is>
           <t>角色指派</t>
         </is>
       </c>
-      <c r="E2" s="15" t="inlineStr">
-        <is>
-          <t>選用依據與動作風格</t>
-        </is>
-      </c>
-      <c r="F2" s="15" t="inlineStr">
-        <is>
-          <t>第一張圖片檔名 (9:16)</t>
-        </is>
-      </c>
-      <c r="G2" s="15" t="inlineStr">
+      <c r="E2" s="21" t="inlineStr">
+        <is>
+          <t>全曲段落數</t>
+        </is>
+      </c>
+      <c r="F2" s="21" t="inlineStr">
+        <is>
+          <t>目錄名稱</t>
+        </is>
+      </c>
+      <c r="G2" s="21" t="inlineStr">
+        <is>
+          <t>首張圖片檔名 (Seg #01)</t>
+        </is>
+      </c>
+      <c r="H2" s="21" t="inlineStr">
+        <is>
+          <t>首張圖片完整路徑</t>
+        </is>
+      </c>
+      <c r="I2" s="21" t="inlineStr">
+        <is>
+          <t>全曲圖片範圍</t>
+        </is>
+      </c>
+      <c r="J2" s="21" t="inlineStr">
         <is>
           <t>解析度規格</t>
         </is>
       </c>
-      <c r="H2" s="15" t="inlineStr">
-        <is>
-          <t>對應動作口令/主題</t>
-        </is>
-      </c>
-      <c r="I2" s="15" t="inlineStr">
-        <is>
-          <t>姿態標籤</t>
-        </is>
-      </c>
-      <c r="J2" s="15" t="inlineStr">
+      <c r="K2" s="21" t="inlineStr">
+        <is>
+          <t>姿態類型</t>
+        </is>
+      </c>
+      <c r="L2" s="21" t="inlineStr">
         <is>
           <t>圖生影片提示詞 (Image-to-Video Prompt)</t>
         </is>
       </c>
     </row>
     <row r="3" ht="54" customHeight="1">
-      <c r="A3" s="16" t="inlineStr">
+      <c r="A3" s="22" t="inlineStr">
         <is>
           <t>#01</t>
         </is>
       </c>
-      <c r="B3" s="17" t="inlineStr">
+      <c r="B3" s="23" t="inlineStr">
         <is>
           <t>Morning Sunshine Hello</t>
         </is>
       </c>
-      <c r="C3" s="17" t="inlineStr">
+      <c r="C3" s="23" t="inlineStr">
         <is>
           <t>晨光萌芽問候</t>
         </is>
       </c>
-      <c r="D3" s="16" t="inlineStr">
+      <c r="D3" s="22" t="inlineStr">
         <is>
           <t>小男生 (樂樂)</t>
         </is>
       </c>
-      <c r="E3" s="17" t="inlineStr">
-        <is>
-          <t>活力晨光、大步踏步</t>
-        </is>
-      </c>
-      <c r="F3" s="16" t="inlineStr">
+      <c r="E3" s="24" t="inlineStr">
+        <is>
+          <t>23 段</t>
+        </is>
+      </c>
+      <c r="F3" s="22" t="inlineStr">
+        <is>
+          <t>images/track_01/</t>
+        </is>
+      </c>
+      <c r="G3" s="23" t="inlineStr">
         <is>
           <t>a1_s01_seg01_boy.jpg</t>
         </is>
       </c>
-      <c r="G3" s="18" t="inlineStr">
+      <c r="H3" s="25" t="inlineStr">
+        <is>
+          <t>images/track_01/a1_s01_seg01_boy.jpg</t>
+        </is>
+      </c>
+      <c r="I3" s="23" t="inlineStr">
+        <is>
+          <t>a1_s01_seg01_boy.jpg ~ a1_s01_seg23_boy.jpg (共 23 張)</t>
+        </is>
+      </c>
+      <c r="J3" s="24" t="inlineStr">
         <is>
           <t>720x1280 (9:16)</t>
         </is>
       </c>
-      <c r="H3" s="17" t="inlineStr">
-        <is>
-          <t>[前奏] 晨光萌芽踏步
-(⏰ 精神小士兵，原地踩著節拍踏步走！)</t>
-        </is>
-      </c>
-      <c r="I3" s="18" t="inlineStr">
+      <c r="K3" s="24" t="inlineStr">
         <is>
           <t>march</t>
         </is>
       </c>
-      <c r="J3" s="17" t="inlineStr">
-        <is>
-          <t>Preschool animated dance video, 3D Pixar style. Using the starter keyframe a1_s01_seg01_boy.jpg, animate the cheerful 5-year-old boy dance coach in blue/orange athletic gym wear in the kindergarten dance studio. The boy coach starts [前奏] 晨光萌芽踏步, marching and swaying with high energy. Smooth preschool rhythmic motion, 60fps, joyful smile, continuous loop, 720p 9:16.</t>
+      <c r="L3" s="23" t="inlineStr">
+        <is>
+          <t>Preschool animated dance video, 3D Pixar style. Using starter keyframe images/track_01/a1_s01_seg01_boy.jpg, animate 小男生 (樂樂) in dance studio for [前奏] 晨光萌芽踏步. 60fps, joyful smile, continuous loop, 720p 9:16.</t>
         </is>
       </c>
     </row>
     <row r="4" ht="54" customHeight="1">
-      <c r="A4" s="16" t="inlineStr">
+      <c r="A4" s="22" t="inlineStr">
         <is>
           <t>#02</t>
         </is>
       </c>
-      <c r="B4" s="17" t="inlineStr">
+      <c r="B4" s="23" t="inlineStr">
         <is>
           <t>Count with Me 1 to 10</t>
         </is>
       </c>
-      <c r="C4" s="17" t="inlineStr">
+      <c r="C4" s="23" t="inlineStr">
         <is>
           <t>數數樂翻天 1 到 10</t>
         </is>
       </c>
-      <c r="D4" s="16" t="inlineStr">
+      <c r="D4" s="22" t="inlineStr">
         <is>
           <t>小女生 (美美)</t>
         </is>
       </c>
-      <c r="E4" s="17" t="inlineStr">
-        <is>
-          <t>歡快數數、手指遊戲</t>
-        </is>
-      </c>
-      <c r="F4" s="16" t="inlineStr">
+      <c r="E4" s="24" t="inlineStr">
+        <is>
+          <t>22 段</t>
+        </is>
+      </c>
+      <c r="F4" s="22" t="inlineStr">
+        <is>
+          <t>images/track_02/</t>
+        </is>
+      </c>
+      <c r="G4" s="23" t="inlineStr">
         <is>
           <t>a1_s02_seg01_girl.jpg</t>
         </is>
       </c>
-      <c r="G4" s="18" t="inlineStr">
+      <c r="H4" s="25" t="inlineStr">
+        <is>
+          <t>images/track_02/a1_s02_seg01_girl.jpg</t>
+        </is>
+      </c>
+      <c r="I4" s="23" t="inlineStr">
+        <is>
+          <t>a1_s02_seg01_girl.jpg ~ a1_s02_seg22_girl.jpg (共 22 張)</t>
+        </is>
+      </c>
+      <c r="J4" s="24" t="inlineStr">
         <is>
           <t>720x1280 (9:16)</t>
         </is>
       </c>
-      <c r="H4" s="17" t="inlineStr">
-        <is>
-          <t>[前奏] 數字小士兵預備踏步
-(🔢 準備好小手小腳，踩出節拍踏步走！)</t>
-        </is>
-      </c>
-      <c r="I4" s="18" t="inlineStr">
+      <c r="K4" s="24" t="inlineStr">
         <is>
           <t>march</t>
         </is>
       </c>
-      <c r="J4" s="17" t="inlineStr">
-        <is>
-          <t>Preschool animated dance video, 3D Pixar style. Using the starter keyframe a1_s02_seg01_girl.jpg, animate the cheerful 5-year-old girl dance coach with brown curly pigtails in pink star tee and yellow shorts in the kindergarten dance studio. The girl coach starts [前奏] 數字小士兵預備踏步, smiling sweetly and posing gracefully. Smooth preschool rhythmic motion, 60fps, joyful smile, continuous loop, 720p 9:16.</t>
+      <c r="L4" s="23" t="inlineStr">
+        <is>
+          <t>Preschool animated dance video, 3D Pixar style. Using starter keyframe images/track_02/a1_s02_seg01_girl.jpg, animate 小女生 (美美) in dance studio for [前奏] 數字小士兵預備踏步. 60fps, joyful smile, continuous loop, 720p 9:16.</t>
         </is>
       </c>
     </row>
     <row r="5" ht="54" customHeight="1">
-      <c r="A5" s="16" t="inlineStr">
+      <c r="A5" s="22" t="inlineStr">
         <is>
           <t>#03</t>
         </is>
       </c>
-      <c r="B5" s="17" t="inlineStr">
+      <c r="B5" s="23" t="inlineStr">
         <is>
           <t>Rainbow Color Splash</t>
         </is>
       </c>
-      <c r="C5" s="17" t="inlineStr">
+      <c r="C5" s="23" t="inlineStr">
         <is>
           <t>繽紛彩虹大塗鴉</t>
         </is>
       </c>
-      <c r="D5" s="16" t="inlineStr">
+      <c r="D5" s="22" t="inlineStr">
         <is>
           <t>小女生 (美美)</t>
         </is>
       </c>
-      <c r="E5" s="17" t="inlineStr">
-        <is>
-          <t>夢幻彩虹、色彩塗鴉</t>
-        </is>
-      </c>
-      <c r="F5" s="16" t="inlineStr">
+      <c r="E5" s="24" t="inlineStr">
+        <is>
+          <t>22 段</t>
+        </is>
+      </c>
+      <c r="F5" s="22" t="inlineStr">
+        <is>
+          <t>images/track_03/</t>
+        </is>
+      </c>
+      <c r="G5" s="23" t="inlineStr">
         <is>
           <t>a1_s03_seg01_girl.jpg</t>
         </is>
       </c>
-      <c r="G5" s="18" t="inlineStr">
+      <c r="H5" s="25" t="inlineStr">
+        <is>
+          <t>images/track_03/a1_s03_seg01_girl.jpg</t>
+        </is>
+      </c>
+      <c r="I5" s="23" t="inlineStr">
+        <is>
+          <t>a1_s03_seg01_girl.jpg ~ a1_s03_seg22_girl.jpg (共 22 張)</t>
+        </is>
+      </c>
+      <c r="J5" s="24" t="inlineStr">
         <is>
           <t>720x1280 (9:16)</t>
         </is>
       </c>
-      <c r="H5" s="17" t="inlineStr">
-        <is>
-          <t>[前奏] 彩虹畫筆小預備
-(🎨 拿起神奇彩色畫筆，準備為天空塗鴉！)</t>
-        </is>
-      </c>
-      <c r="I5" s="18" t="inlineStr">
+      <c r="K5" s="24" t="inlineStr">
         <is>
           <t>march</t>
         </is>
       </c>
-      <c r="J5" s="17" t="inlineStr">
-        <is>
-          <t>Preschool animated dance video, 3D Pixar style. Using the starter keyframe a1_s03_seg01_girl.jpg, animate the cheerful 5-year-old girl dance coach with brown curly pigtails in pink star tee and yellow shorts in the kindergarten dance studio. The girl coach starts [前奏] 彩虹畫筆小預備, smiling sweetly and posing gracefully. Smooth preschool rhythmic motion, 60fps, joyful smile, continuous loop, 720p 9:16.</t>
+      <c r="L5" s="23" t="inlineStr">
+        <is>
+          <t>Preschool animated dance video, 3D Pixar style. Using starter keyframe images/track_03/a1_s03_seg01_girl.jpg, animate 小女生 (美美) in dance studio for [前奏] 彩虹畫筆小預備. 60fps, joyful smile, continuous loop, 720p 9:16.</t>
         </is>
       </c>
     </row>
     <row r="6" ht="54" customHeight="1">
-      <c r="A6" s="16" t="inlineStr">
+      <c r="A6" s="22" t="inlineStr">
         <is>
           <t>#04</t>
         </is>
       </c>
-      <c r="B6" s="17" t="inlineStr">
+      <c r="B6" s="23" t="inlineStr">
         <is>
           <t>Animal Safari March</t>
         </is>
       </c>
-      <c r="C6" s="17" t="inlineStr">
+      <c r="C6" s="23" t="inlineStr">
         <is>
           <t>奇幻動物大巡遊</t>
         </is>
       </c>
-      <c r="D6" s="16" t="inlineStr">
+      <c r="D6" s="22" t="inlineStr">
         <is>
           <t>小男生 (樂樂)</t>
         </is>
       </c>
-      <c r="E6" s="17" t="inlineStr">
-        <is>
-          <t>森林冒險、號角行軍</t>
-        </is>
-      </c>
-      <c r="F6" s="16" t="inlineStr">
+      <c r="E6" s="24" t="inlineStr">
+        <is>
+          <t>26 段</t>
+        </is>
+      </c>
+      <c r="F6" s="22" t="inlineStr">
+        <is>
+          <t>images/track_04/</t>
+        </is>
+      </c>
+      <c r="G6" s="23" t="inlineStr">
         <is>
           <t>a1_s04_seg01_boy.jpg</t>
         </is>
       </c>
-      <c r="G6" s="18" t="inlineStr">
+      <c r="H6" s="25" t="inlineStr">
+        <is>
+          <t>images/track_04/a1_s04_seg01_boy.jpg</t>
+        </is>
+      </c>
+      <c r="I6" s="23" t="inlineStr">
+        <is>
+          <t>a1_s04_seg01_boy.jpg ~ a1_s04_seg26_boy.jpg (共 26 張)</t>
+        </is>
+      </c>
+      <c r="J6" s="24" t="inlineStr">
         <is>
           <t>720x1280 (9:16)</t>
         </is>
       </c>
-      <c r="H6" s="17" t="inlineStr">
-        <is>
-          <t>[前奏] 森林號角精神踏步
-(🎺 聽號角吹響！雙手插腰，膝蓋抬高大步踏走！)</t>
-        </is>
-      </c>
-      <c r="I6" s="18" t="inlineStr">
+      <c r="K6" s="24" t="inlineStr">
         <is>
           <t>march</t>
         </is>
       </c>
-      <c r="J6" s="17" t="inlineStr">
-        <is>
-          <t>Preschool animated dance video, 3D Pixar style. Using the starter keyframe a1_s04_seg01_boy.jpg, animate the cheerful 5-year-old boy dance coach in blue/orange athletic gym wear in the kindergarten dance studio. The boy coach starts [前奏] 森林號角精神踏步, marching and swaying with high energy. Smooth preschool rhythmic motion, 60fps, joyful smile, continuous loop, 720p 9:16.</t>
+      <c r="L6" s="23" t="inlineStr">
+        <is>
+          <t>Preschool animated dance video, 3D Pixar style. Using starter keyframe images/track_04/a1_s04_seg01_boy.jpg, animate 小男生 (樂樂) in dance studio for [前奏] 森林號角精神踏步. 60fps, joyful smile, continuous loop, 720p 9:16.</t>
         </is>
       </c>
     </row>
     <row r="7" ht="54" customHeight="1">
-      <c r="A7" s="16" t="inlineStr">
+      <c r="A7" s="22" t="inlineStr">
         <is>
           <t>#05</t>
         </is>
       </c>
-      <c r="B7" s="17" t="inlineStr">
+      <c r="B7" s="23" t="inlineStr">
         <is>
           <t>Clean Up Little Helpers</t>
         </is>
       </c>
-      <c r="C7" s="17" t="inlineStr">
+      <c r="C7" s="23" t="inlineStr">
         <is>
           <t>整理收納小幫手</t>
         </is>
       </c>
-      <c r="D7" s="16" t="inlineStr">
+      <c r="D7" s="22" t="inlineStr">
         <is>
           <t>小女生 (美美)</t>
         </is>
       </c>
-      <c r="E7" s="17" t="inlineStr">
-        <is>
-          <t>生活收納、整潔常規</t>
-        </is>
-      </c>
-      <c r="F7" s="16" t="inlineStr">
+      <c r="E7" s="24" t="inlineStr">
+        <is>
+          <t>26 段</t>
+        </is>
+      </c>
+      <c r="F7" s="22" t="inlineStr">
+        <is>
+          <t>images/track_05/</t>
+        </is>
+      </c>
+      <c r="G7" s="23" t="inlineStr">
         <is>
           <t>a1_s05_seg01_girl.jpg</t>
         </is>
       </c>
-      <c r="G7" s="18" t="inlineStr">
+      <c r="H7" s="25" t="inlineStr">
+        <is>
+          <t>images/track_05/a1_s05_seg01_girl.jpg</t>
+        </is>
+      </c>
+      <c r="I7" s="23" t="inlineStr">
+        <is>
+          <t>a1_s05_seg01_girl.jpg ~ a1_s05_seg26_girl.jpg (共 26 張)</t>
+        </is>
+      </c>
+      <c r="J7" s="24" t="inlineStr">
         <is>
           <t>720x1280 (9:16)</t>
         </is>
       </c>
-      <c r="H7" s="17" t="inlineStr">
-        <is>
-          <t>[前奏] 時鐘滴答整理預備
-(⏰ 時鐘滴答走，玩具小幫手挽起袖子集合！)</t>
-        </is>
-      </c>
-      <c r="I7" s="18" t="inlineStr">
+      <c r="K7" s="24" t="inlineStr">
         <is>
           <t>march</t>
         </is>
       </c>
-      <c r="J7" s="17" t="inlineStr">
-        <is>
-          <t>Preschool animated dance video, 3D Pixar style. Using the starter keyframe a1_s05_seg01_girl.jpg, animate the cheerful 5-year-old girl dance coach with brown curly pigtails in pink star tee and yellow shorts in the kindergarten dance studio. The girl coach starts [前奏] 時鐘滴答整理預備, smiling sweetly and posing gracefully. Smooth preschool rhythmic motion, 60fps, joyful smile, continuous loop, 720p 9:16.</t>
+      <c r="L7" s="23" t="inlineStr">
+        <is>
+          <t>Preschool animated dance video, 3D Pixar style. Using starter keyframe images/track_05/a1_s05_seg01_girl.jpg, animate 小女生 (美美) in dance studio for [前奏] 時鐘滴答整理預備. 60fps, joyful smile, continuous loop, 720p 9:16.</t>
         </is>
       </c>
     </row>
     <row r="8" ht="54" customHeight="1">
-      <c r="A8" s="16" t="inlineStr">
+      <c r="A8" s="22" t="inlineStr">
         <is>
           <t>#06</t>
         </is>
       </c>
-      <c r="B8" s="17" t="inlineStr">
+      <c r="B8" s="23" t="inlineStr">
         <is>
           <t>Space Rocket Countdown</t>
         </is>
       </c>
-      <c r="C8" s="17" t="inlineStr">
+      <c r="C8" s="23" t="inlineStr">
         <is>
           <t>太空火箭大倒數</t>
         </is>
       </c>
-      <c r="D8" s="16" t="inlineStr">
+      <c r="D8" s="22" t="inlineStr">
         <is>
           <t>小男生 (樂樂)</t>
         </is>
       </c>
-      <c r="E8" s="17" t="inlineStr">
-        <is>
-          <t>火箭升空、爆發衝刺</t>
-        </is>
-      </c>
-      <c r="F8" s="16" t="inlineStr">
+      <c r="E8" s="24" t="inlineStr">
+        <is>
+          <t>28 段</t>
+        </is>
+      </c>
+      <c r="F8" s="22" t="inlineStr">
+        <is>
+          <t>images/track_06/</t>
+        </is>
+      </c>
+      <c r="G8" s="23" t="inlineStr">
         <is>
           <t>a1_s06_seg01_boy.jpg</t>
         </is>
       </c>
-      <c r="G8" s="18" t="inlineStr">
+      <c r="H8" s="25" t="inlineStr">
+        <is>
+          <t>images/track_06/a1_s06_seg01_boy.jpg</t>
+        </is>
+      </c>
+      <c r="I8" s="23" t="inlineStr">
+        <is>
+          <t>a1_s06_seg01_boy.jpg ~ a1_s06_seg28_boy.jpg (共 28 張)</t>
+        </is>
+      </c>
+      <c r="J8" s="24" t="inlineStr">
         <is>
           <t>720x1280 (9:16)</t>
         </is>
       </c>
-      <c r="H8" s="17" t="inlineStr">
-        <is>
-          <t>[前奏] 宇宙電波呼叫訊號
-(📡 嗶嗶嗶！戴上太空頭盔，發射台準備完畢！)</t>
-        </is>
-      </c>
-      <c r="I8" s="18" t="inlineStr">
+      <c r="K8" s="24" t="inlineStr">
         <is>
           <t>march</t>
         </is>
       </c>
-      <c r="J8" s="17" t="inlineStr">
-        <is>
-          <t>Preschool animated dance video, 3D Pixar style. Using the starter keyframe a1_s06_seg01_boy.jpg, animate the cheerful 5-year-old boy dance coach in blue/orange athletic gym wear in the kindergarten dance studio. The boy coach starts [前奏] 宇宙電波呼叫訊號, marching and swaying with high energy. Smooth preschool rhythmic motion, 60fps, joyful smile, continuous loop, 720p 9:16.</t>
+      <c r="L8" s="23" t="inlineStr">
+        <is>
+          <t>Preschool animated dance video, 3D Pixar style. Using starter keyframe images/track_06/a1_s06_seg01_boy.jpg, animate 小男生 (樂樂) in dance studio for [前奏] 宇宙電波呼叫訊號. 60fps, joyful smile, continuous loop, 720p 9:16.</t>
         </is>
       </c>
     </row>
     <row r="9" ht="54" customHeight="1">
-      <c r="A9" s="16" t="inlineStr">
+      <c r="A9" s="22" t="inlineStr">
         <is>
           <t>#07</t>
         </is>
       </c>
-      <c r="B9" s="17" t="inlineStr">
+      <c r="B9" s="23" t="inlineStr">
         <is>
           <t>The Magic ABC Train</t>
         </is>
       </c>
-      <c r="C9" s="17" t="inlineStr">
+      <c r="C9" s="23" t="inlineStr">
         <is>
           <t>神奇 ABC 字母列車</t>
         </is>
       </c>
-      <c r="D9" s="16" t="inlineStr">
+      <c r="D9" s="22" t="inlineStr">
         <is>
           <t>小女生 (美美)</t>
         </is>
       </c>
-      <c r="E9" s="17" t="inlineStr">
-        <is>
-          <t>字母歡唱、輕快列車</t>
-        </is>
-      </c>
-      <c r="F9" s="16" t="inlineStr">
+      <c r="E9" s="24" t="inlineStr">
+        <is>
+          <t>26 段</t>
+        </is>
+      </c>
+      <c r="F9" s="22" t="inlineStr">
+        <is>
+          <t>images/track_07/</t>
+        </is>
+      </c>
+      <c r="G9" s="23" t="inlineStr">
         <is>
           <t>a1_s07_seg01_girl.jpg</t>
         </is>
       </c>
-      <c r="G9" s="18" t="inlineStr">
+      <c r="H9" s="25" t="inlineStr">
+        <is>
+          <t>images/track_07/a1_s07_seg01_girl.jpg</t>
+        </is>
+      </c>
+      <c r="I9" s="23" t="inlineStr">
+        <is>
+          <t>a1_s07_seg01_girl.jpg ~ a1_s07_seg26_girl.jpg (共 26 張)</t>
+        </is>
+      </c>
+      <c r="J9" s="24" t="inlineStr">
         <is>
           <t>720x1280 (9:16)</t>
         </is>
       </c>
-      <c r="H9" s="17" t="inlineStr">
-        <is>
-          <t>[前奏] 蒸汽火車汽笛響起
-(🚂 嗚嗚！拉響火車汽笛，ABC 字母列車準備開動！)</t>
-        </is>
-      </c>
-      <c r="I9" s="18" t="inlineStr">
+      <c r="K9" s="24" t="inlineStr">
         <is>
           <t>march</t>
         </is>
       </c>
-      <c r="J9" s="17" t="inlineStr">
-        <is>
-          <t>Preschool animated dance video, 3D Pixar style. Using the starter keyframe a1_s07_seg01_girl.jpg, animate the cheerful 5-year-old girl dance coach with brown curly pigtails in pink star tee and yellow shorts in the kindergarten dance studio. The girl coach starts [前奏] 蒸汽火車汽笛響起, smiling sweetly and posing gracefully. Smooth preschool rhythmic motion, 60fps, joyful smile, continuous loop, 720p 9:16.</t>
+      <c r="L9" s="23" t="inlineStr">
+        <is>
+          <t>Preschool animated dance video, 3D Pixar style. Using starter keyframe images/track_07/a1_s07_seg01_girl.jpg, animate 小女生 (美美) in dance studio for [前奏] 蒸汽火車汽笛響起. 60fps, joyful smile, continuous loop, 720p 9:16.</t>
         </is>
       </c>
     </row>
     <row r="10" ht="54" customHeight="1">
-      <c r="A10" s="16" t="inlineStr">
+      <c r="A10" s="22" t="inlineStr">
         <is>
           <t>#08</t>
         </is>
       </c>
-      <c r="B10" s="17" t="inlineStr">
+      <c r="B10" s="23" t="inlineStr">
         <is>
           <t>Wiggle &amp; Freeze!</t>
         </is>
       </c>
-      <c r="C10" s="17" t="inlineStr">
+      <c r="C10" s="23" t="inlineStr">
         <is>
           <t>扭扭定格大挑戰</t>
         </is>
       </c>
-      <c r="D10" s="16" t="inlineStr">
+      <c r="D10" s="22" t="inlineStr">
         <is>
           <t>小男生 (樂樂)</t>
         </is>
       </c>
-      <c r="E10" s="17" t="inlineStr">
-        <is>
-          <t>定格反應、節奏挑戰</t>
-        </is>
-      </c>
-      <c r="F10" s="16" t="inlineStr">
+      <c r="E10" s="24" t="inlineStr">
+        <is>
+          <t>27 段</t>
+        </is>
+      </c>
+      <c r="F10" s="22" t="inlineStr">
+        <is>
+          <t>images/track_08/</t>
+        </is>
+      </c>
+      <c r="G10" s="23" t="inlineStr">
         <is>
           <t>a1_s08_seg01_boy.jpg</t>
         </is>
       </c>
-      <c r="G10" s="18" t="inlineStr">
+      <c r="H10" s="25" t="inlineStr">
+        <is>
+          <t>images/track_08/a1_s08_seg01_boy.jpg</t>
+        </is>
+      </c>
+      <c r="I10" s="23" t="inlineStr">
+        <is>
+          <t>a1_s08_seg01_boy.jpg ~ a1_s08_seg27_boy.jpg (共 27 張)</t>
+        </is>
+      </c>
+      <c r="J10" s="24" t="inlineStr">
         <is>
           <t>720x1280 (9:16)</t>
         </is>
       </c>
-      <c r="H10" s="17" t="inlineStr">
-        <is>
-          <t>第 01 節: 節奏鼓點咚咚咚
-(🥁 腳尖踩拍子，雙手輕快拍拍大腿！)</t>
-        </is>
-      </c>
-      <c r="I10" s="18" t="inlineStr">
+      <c r="K10" s="24" t="inlineStr">
         <is>
           <t>march</t>
         </is>
       </c>
-      <c r="J10" s="17" t="inlineStr">
-        <is>
-          <t>Preschool animated dance video, 3D Pixar style. Using the starter keyframe a1_s08_seg01_boy.jpg, animate the cheerful 5-year-old boy dance coach in blue/orange athletic gym wear in the kindergarten dance studio. The boy coach starts 第 01 節: 節奏鼓點咚咚咚, marching and swaying with high energy. Smooth preschool rhythmic motion, 60fps, joyful smile, continuous loop, 720p 9:16.</t>
+      <c r="L10" s="23" t="inlineStr">
+        <is>
+          <t>Preschool animated dance video, 3D Pixar style. Using starter keyframe images/track_08/a1_s08_seg01_boy.jpg, animate 小男生 (樂樂) in dance studio for 第 01 節: 節奏鼓點咚咚咚. 60fps, joyful smile, continuous loop, 720p 9:16.</t>
         </is>
       </c>
     </row>
     <row r="11" ht="54" customHeight="1">
-      <c r="A11" s="16" t="inlineStr">
+      <c r="A11" s="22" t="inlineStr">
         <is>
           <t>#09</t>
         </is>
       </c>
-      <c r="B11" s="17" t="inlineStr">
+      <c r="B11" s="23" t="inlineStr">
         <is>
           <t>Yummy Healthy Snack</t>
         </is>
       </c>
-      <c r="C11" s="17" t="inlineStr">
+      <c r="C11" s="23" t="inlineStr">
         <is>
           <t>美味健康小點心</t>
         </is>
       </c>
-      <c r="D11" s="16" t="inlineStr">
+      <c r="D11" s="22" t="inlineStr">
         <is>
           <t>小男生 (樂樂)</t>
         </is>
       </c>
-      <c r="E11" s="17" t="inlineStr">
-        <is>
-          <t>健康美食、活力點心</t>
-        </is>
-      </c>
-      <c r="F11" s="16" t="inlineStr">
+      <c r="E11" s="24" t="inlineStr">
+        <is>
+          <t>24 段</t>
+        </is>
+      </c>
+      <c r="F11" s="22" t="inlineStr">
+        <is>
+          <t>images/track_09/</t>
+        </is>
+      </c>
+      <c r="G11" s="23" t="inlineStr">
         <is>
           <t>a1_s09_seg01_boy.jpg</t>
         </is>
       </c>
-      <c r="G11" s="18" t="inlineStr">
+      <c r="H11" s="25" t="inlineStr">
+        <is>
+          <t>images/track_09/a1_s09_seg01_boy.jpg</t>
+        </is>
+      </c>
+      <c r="I11" s="23" t="inlineStr">
+        <is>
+          <t>a1_s09_seg01_boy.jpg ~ a1_s09_seg24_boy.jpg (共 24 張)</t>
+        </is>
+      </c>
+      <c r="J11" s="24" t="inlineStr">
         <is>
           <t>720x1280 (9:16)</t>
         </is>
       </c>
-      <c r="H11" s="17" t="inlineStr">
-        <is>
-          <t>[前奏] 肚子咕嚕嚕美食預備
-(🥣 肚子咕嚕嚕！戴上小廚師帽，健康點心開動囉！)</t>
-        </is>
-      </c>
-      <c r="I11" s="18" t="inlineStr">
+      <c r="K11" s="24" t="inlineStr">
         <is>
           <t>march</t>
         </is>
       </c>
-      <c r="J11" s="17" t="inlineStr">
-        <is>
-          <t>Preschool animated dance video, 3D Pixar style. Using the starter keyframe a1_s09_seg01_boy.jpg, animate the cheerful 5-year-old boy dance coach in blue/orange athletic gym wear in the kindergarten dance studio. The boy coach starts [前奏] 肚子咕嚕嚕美食預備, marching and swaying with high energy. Smooth preschool rhythmic motion, 60fps, joyful smile, continuous loop, 720p 9:16.</t>
+      <c r="L11" s="23" t="inlineStr">
+        <is>
+          <t>Preschool animated dance video, 3D Pixar style. Using starter keyframe images/track_09/a1_s09_seg01_boy.jpg, animate 小男生 (樂樂) in dance studio for [前奏] 肚子咕嚕嚕美食預備. 60fps, joyful smile, continuous loop, 720p 9:16.</t>
         </is>
       </c>
     </row>
     <row r="12" ht="54" customHeight="1">
-      <c r="A12" s="16" t="inlineStr">
+      <c r="A12" s="22" t="inlineStr">
         <is>
           <t>#10</t>
         </is>
       </c>
-      <c r="B12" s="17" t="inlineStr">
+      <c r="B12" s="23" t="inlineStr">
         <is>
           <t>Soft Pillow Goodnight</t>
         </is>
       </c>
-      <c r="C12" s="17" t="inlineStr">
+      <c r="C12" s="23" t="inlineStr">
         <is>
           <t>柔軟枕頭晚安曲</t>
         </is>
       </c>
-      <c r="D12" s="16" t="inlineStr">
+      <c r="D12" s="22" t="inlineStr">
         <is>
           <t>小女生 (美美)</t>
         </is>
       </c>
-      <c r="E12" s="17" t="inlineStr">
-        <is>
-          <t>晚安搖籃、溫柔撫慰</t>
-        </is>
-      </c>
-      <c r="F12" s="16" t="inlineStr">
+      <c r="E12" s="24" t="inlineStr">
+        <is>
+          <t>21 段</t>
+        </is>
+      </c>
+      <c r="F12" s="22" t="inlineStr">
+        <is>
+          <t>images/track_10/</t>
+        </is>
+      </c>
+      <c r="G12" s="23" t="inlineStr">
         <is>
           <t>a1_s10_seg01_girl.jpg</t>
         </is>
       </c>
-      <c r="G12" s="18" t="inlineStr">
+      <c r="H12" s="25" t="inlineStr">
+        <is>
+          <t>images/track_10/a1_s10_seg01_girl.jpg</t>
+        </is>
+      </c>
+      <c r="I12" s="23" t="inlineStr">
+        <is>
+          <t>a1_s10_seg01_girl.jpg ~ a1_s10_seg21_girl.jpg (共 21 張)</t>
+        </is>
+      </c>
+      <c r="J12" s="24" t="inlineStr">
         <is>
           <t>720x1280 (9:16)</t>
         </is>
       </c>
-      <c r="H12" s="17" t="inlineStr">
-        <is>
-          <t>[前奏] 夜幕低垂搖籃曲
-(🌙 月亮升起，微風吹拂，輕輕左右搖擺放鬆身體！)</t>
-        </is>
-      </c>
-      <c r="I12" s="18" t="inlineStr">
+      <c r="K12" s="24" t="inlineStr">
         <is>
           <t>sway</t>
         </is>
       </c>
-      <c r="J12" s="17" t="inlineStr">
-        <is>
-          <t>Preschool animated dance video, 3D Pixar style. Using the starter keyframe a1_s10_seg01_girl.jpg, animate the cheerful 5-year-old girl dance coach with brown curly pigtails in pink star tee and yellow shorts in the kindergarten dance studio. The girl coach starts [前奏] 夜幕低垂搖籃曲, smiling sweetly and posing gracefully. Smooth preschool rhythmic motion, 60fps, joyful smile, continuous loop, 720p 9:16.</t>
+      <c r="L12" s="23" t="inlineStr">
+        <is>
+          <t>Preschool animated dance video, 3D Pixar style. Using starter keyframe images/track_10/a1_s10_seg01_girl.jpg, animate 小女生 (美美) in dance studio for [前奏] 夜幕低垂搖籃曲. 60fps, joyful smile, continuous loop, 720p 9:16.</t>
         </is>
       </c>
     </row>
   </sheetData>
-  <mergeCells count="1">
+  <mergeCells count="2">
     <mergeCell ref="A1:J1"/>
+    <mergeCell ref="A1:L1"/>
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
@@ -18535,7 +19196,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J25"/>
+  <dimension ref="A1:K25"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="18" customWidth="1" min="1" max="1"/>
@@ -18548,6 +19209,7 @@
     <col width="30" customWidth="1" min="8" max="8"/>
     <col width="12" customWidth="1" min="9" max="9"/>
     <col width="55" customWidth="1" min="10" max="10"/>
+    <col width="34" customWidth="1" min="11" max="11"/>
   </cols>
   <sheetData>
     <row r="1" ht="32" customHeight="1">
@@ -18608,6 +19270,11 @@
           <t>AI 影片動畫生成提示詞 (Prompt)</t>
         </is>
       </c>
+      <c r="K2" s="19" t="inlineStr">
+        <is>
+          <t>首張圖片路徑 (9:16 720p)</t>
+        </is>
+      </c>
     </row>
     <row r="3" ht="30" customHeight="1">
       <c r="A3" s="10" t="inlineStr">
@@ -18656,6 +19323,11 @@
           <t>3D Pixar Disney style preschool animation video keyframe, vertical 9:16 aspect ratio 720p HD. Full body standing shot of the cheerful 5-year-old boy dance coach in bright blue athletic t-shirt with orange center and KIDS DANCE logo, blue shorts, orange running sneakers. In colorful kindergarten dance studio. Starter keyframe for action "[前奏] 晨光萌芽踏步" (⏰ 精神小士兵，原地踩著節拍踏步走！). The character is in lively dance starter pose, joyful radiant beaming smile, sparkling expressive eyes. 4k 3D Pixar render, clean frame without text overlay, starter keyframe for image-to-video generation (a1_s01_seg01_boy.jpg).</t>
         </is>
       </c>
+      <c r="K3" s="20" t="inlineStr">
+        <is>
+          <t>images/track_01/a1_s01_seg01_boy.jpg</t>
+        </is>
+      </c>
     </row>
     <row r="4" ht="30" customHeight="1">
       <c r="A4" s="8" t="inlineStr">
@@ -18704,6 +19376,11 @@
           <t>3D Pixar Disney style cheerful toddler dance coach, smooth playful animation, vibrant kindergarten studio, soft bright volumetric lighting, clean studio background, highly expressive face, full body dynamic camera shot: Song 'Morning Sunshine Hello', Action '第 01 節: 托起太陽高高舉'. ☀️ 雙手從胸前托起大太陽高高升起！. The character is lifting arms from heart to sky creating a big golden sun circle, chest open, radiant beaming joyful smile. 4k resolution, 60fps, Disney Pixar render, joyful preschool music video style.</t>
         </is>
       </c>
+      <c r="K4" s="20" t="inlineStr">
+        <is>
+          <t>images/track_01/a1_s01_seg02_boy.jpg</t>
+        </is>
+      </c>
     </row>
     <row r="5" ht="30" customHeight="1">
       <c r="A5" s="10" t="inlineStr">
@@ -18752,6 +19429,11 @@
           <t>3D Pixar Disney style cheerful toddler dance coach, smooth playful animation, vibrant kindergarten studio, soft bright volumetric lighting, clean studio background, highly expressive face, full body dynamic camera shot: Song 'Morning Sunshine Hello', Action '第 02 節: 金色小手大招手'. 👋 雙手在天空左右大弧度歡快招手！. The character is waving both hands overhead in friendly wide arcs, swaying gently from side to side, sparkling excited eyes. 4k resolution, 60fps, Disney Pixar render, joyful preschool music video style.</t>
         </is>
       </c>
+      <c r="K5" s="20" t="inlineStr">
+        <is>
+          <t>images/track_01/a1_s01_seg03_boy.jpg</t>
+        </is>
+      </c>
     </row>
     <row r="6" ht="30" customHeight="1">
       <c r="A6" s="8" t="inlineStr">
@@ -18800,6 +19482,11 @@
           <t>3D Pixar Disney style cheerful toddler dance coach, smooth playful animation, vibrant kindergarten studio, soft bright volumetric lighting, clean studio background, highly expressive face, full body dynamic camera shot: Song 'Morning Sunshine Hello', Action '第 03 節: 刷刷小牙笑一笑'. 🪥 小牙刷刷刷刷，露出最燦爛笑容！. The character is marching in place energetically, hands on hips, knees lifting high in rhythmic bounce, enthusiastic happy smile. 4k resolution, 60fps, Disney Pixar render, joyful preschool music video style.</t>
         </is>
       </c>
+      <c r="K6" s="20" t="inlineStr">
+        <is>
+          <t>images/track_01/a1_s01_seg04_boy.jpg</t>
+        </is>
+      </c>
     </row>
     <row r="7" ht="30" customHeight="1">
       <c r="A7" s="10" t="inlineStr">
@@ -18848,6 +19535,11 @@
           <t>3D Pixar Disney style cheerful toddler dance coach, smooth playful animation, vibrant kindergarten studio, soft bright volumetric lighting, clean studio background, highly expressive face, full body dynamic camera shot: Song 'Morning Sunshine Hello', Action '第 04 節: 邁開大步出發囉'. 👟 雙手插腰精神抖擻，大步邁開去探險！. The character is marching in place energetically, hands on hips, knees lifting high in rhythmic bounce, enthusiastic happy smile. 4k resolution, 60fps, Disney Pixar render, joyful preschool music video style.</t>
         </is>
       </c>
+      <c r="K7" s="20" t="inlineStr">
+        <is>
+          <t>images/track_01/a1_s01_seg05_boy.jpg</t>
+        </is>
+      </c>
     </row>
     <row r="8" ht="30" customHeight="1">
       <c r="A8" s="8" t="inlineStr">
@@ -18896,6 +19588,11 @@
           <t>3D Pixar Disney style cheerful toddler dance coach, smooth playful animation, vibrant kindergarten studio, soft bright volumetric lighting, clean studio background, highly expressive face, full body dynamic camera shot: Song 'Morning Sunshine Hello', Action '第 05 節: 樹梢小鳥展翅飛'. 🐦 雙臂輕快拍動，學小鳥在樹梢滑翔！. The character is swaying hips and arms like a breeze, smooth fluid body roll, playful rhythmic dancing, friendly warm smile. 4k resolution, 60fps, Disney Pixar render, joyful preschool music video style.</t>
         </is>
       </c>
+      <c r="K8" s="20" t="inlineStr">
+        <is>
+          <t>images/track_01/a1_s01_seg06_boy.jpg</t>
+        </is>
+      </c>
     </row>
     <row r="9" ht="30" customHeight="1">
       <c r="A9" s="10" t="inlineStr">
@@ -18944,6 +19641,11 @@
           <t>3D Pixar Disney style cheerful toddler dance coach, smooth playful animation, vibrant kindergarten studio, soft bright volumetric lighting, clean studio background, highly expressive face, full body dynamic camera shot: Song 'Morning Sunshine Hello', Action '第 06 節: 貼耳聽清晨鳥鳴'. 🎶 小手貼耳，身體左右輕輕搖擺聽晨曲！. The character is swaying hips and arms like a breeze, smooth fluid body roll, playful rhythmic dancing, friendly warm smile. 4k resolution, 60fps, Disney Pixar render, joyful preschool music video style.</t>
         </is>
       </c>
+      <c r="K9" s="20" t="inlineStr">
+        <is>
+          <t>images/track_01/a1_s01_seg07_boy.jpg</t>
+        </is>
+      </c>
     </row>
     <row r="10" ht="30" customHeight="1">
       <c r="A10" s="8" t="inlineStr">
@@ -18992,6 +19694,11 @@
           <t>3D Pixar Disney style cheerful toddler dance coach, smooth playful animation, vibrant kindergarten studio, soft bright volumetric lighting, clean studio background, highly expressive face, full body dynamic camera shot: Song 'Morning Sunshine Hello', Action '第 07 節: 熱情招手說哈囉'. 👋 揮舞雙手大聲喊 Hello，全新一天開始！. The character is waving both hands overhead in friendly wide arcs, swaying gently from side to side, sparkling excited eyes. 4k resolution, 60fps, Disney Pixar render, joyful preschool music video style.</t>
         </is>
       </c>
+      <c r="K10" s="20" t="inlineStr">
+        <is>
+          <t>images/track_01/a1_s01_seg08_boy.jpg</t>
+        </is>
+      </c>
     </row>
     <row r="11" ht="30" customHeight="1">
       <c r="A11" s="10" t="inlineStr">
@@ -19040,6 +19747,11 @@
           <t>3D Pixar Disney style cheerful toddler dance coach, smooth playful animation, vibrant kindergarten studio, soft bright volumetric lighting, clean studio background, highly expressive face, full body dynamic camera shot: Song 'Morning Sunshine Hello', Action '第 08 節: 活力蹦跳喊萬歲'. ⭐ 雙膝下蹲蓄力，高高跳起喊萬歲！. The character is squatting down and bursting into a high happy jump, feet kicking joyfully in mid-air, both fists punching the sky in victory. 4k resolution, 60fps, Disney Pixar render, joyful preschool music video style.</t>
         </is>
       </c>
+      <c r="K11" s="20" t="inlineStr">
+        <is>
+          <t>images/track_01/a1_s01_seg09_boy.jpg</t>
+        </is>
+      </c>
     </row>
     <row r="12" ht="30" customHeight="1">
       <c r="A12" s="8" t="inlineStr">
@@ -19088,6 +19800,11 @@
           <t>3D Pixar Disney style cheerful toddler dance coach, smooth playful animation, vibrant kindergarten studio, soft bright volumetric lighting, clean studio background, highly expressive face, full body dynamic camera shot: Song 'Morning Sunshine Hello', Action '第 09 節: 穿上小鞋數一二三'. 👟 摸摸左右小鞋子，伸指數：一、二、三！. The character is stretching arms up high to reach floating elements, standing on tiptoes, joyful posture, looking up with wonder. 4k resolution, 60fps, Disney Pixar render, joyful preschool music video style.</t>
         </is>
       </c>
+      <c r="K12" s="20" t="inlineStr">
+        <is>
+          <t>images/track_01/a1_s01_seg10_boy.jpg</t>
+        </is>
+      </c>
     </row>
     <row r="13" ht="30" customHeight="1">
       <c r="A13" s="10" t="inlineStr">
@@ -19136,6 +19853,11 @@
           <t>3D Pixar Disney style cheerful toddler dance coach, smooth playful animation, vibrant kindergarten studio, soft bright volumetric lighting, clean studio background, highly expressive face, full body dynamic camera shot: Song 'Morning Sunshine Hello', Action '第 10 節: 張開雙手齊邀請'. 🎶 雙手像花朵向外盛開，邀請好朋友唱歌！. The character is stretching arms up high to reach floating elements, standing on tiptoes, joyful posture, looking up with wonder. 4k resolution, 60fps, Disney Pixar render, joyful preschool music video style.</t>
         </is>
       </c>
+      <c r="K13" s="20" t="inlineStr">
+        <is>
+          <t>images/track_01/a1_s01_seg11_boy.jpg</t>
+        </is>
+      </c>
     </row>
     <row r="14" ht="30" customHeight="1">
       <c r="A14" s="8" t="inlineStr">
@@ -19184,6 +19906,11 @@
           <t>3D Pixar Disney style cheerful toddler dance coach, smooth playful animation, vibrant kindergarten studio, soft bright volumetric lighting, clean studio background, highly expressive face, full body dynamic camera shot: Song 'Morning Sunshine Hello', Action '第 11 節: 同唱早安小圓舞'. 🌸 雙手插腰轉個歡樂大圓圈，站定比個花！. The character is swaying hips and arms like a breeze, smooth fluid body roll, playful rhythmic dancing, friendly warm smile. 4k resolution, 60fps, Disney Pixar render, joyful preschool music video style.</t>
         </is>
       </c>
+      <c r="K14" s="20" t="inlineStr">
+        <is>
+          <t>images/track_01/a1_s01_seg12_boy.jpg</t>
+        </is>
+      </c>
     </row>
     <row r="15" ht="30" customHeight="1">
       <c r="A15" s="10" t="inlineStr">
@@ -19232,6 +19959,11 @@
           <t>3D Pixar Disney style cheerful toddler dance coach, smooth playful animation, vibrant kindergarten studio, soft bright volumetric lighting, clean studio background, highly expressive face, full body dynamic camera shot: Song 'Morning Sunshine Hello', Action '第 12 節: 背起書包戴正帽'. 🎒 背起小書包、摸摸小帽子，準備好！. The character is marching in place energetically, hands on hips, knees lifting high in rhythmic bounce, enthusiastic happy smile. 4k resolution, 60fps, Disney Pixar render, joyful preschool music video style.</t>
         </is>
       </c>
+      <c r="K15" s="20" t="inlineStr">
+        <is>
+          <t>images/track_01/a1_s01_seg13_boy.jpg</t>
+        </is>
+      </c>
     </row>
     <row r="16" ht="30" customHeight="1">
       <c r="A16" s="8" t="inlineStr">
@@ -19280,6 +20012,11 @@
           <t>3D Pixar Disney style cheerful toddler dance coach, smooth playful animation, vibrant kindergarten studio, soft bright volumetric lighting, clean studio background, highly expressive face, full body dynamic camera shot: Song 'Morning Sunshine Hello', Action '第 13 節: 跟貪睡小貓說拜拜'. 🐱 雙手揉揉眼睛學小貓咪，俏皮說拜拜！. The character is waving both hands overhead in friendly wide arcs, swaying gently from side to side, sparkling excited eyes. 4k resolution, 60fps, Disney Pixar render, joyful preschool music video style.</t>
         </is>
       </c>
+      <c r="K16" s="20" t="inlineStr">
+        <is>
+          <t>images/track_01/a1_s01_seg14_boy.jpg</t>
+        </is>
+      </c>
     </row>
     <row r="17" ht="30" customHeight="1">
       <c r="A17" s="10" t="inlineStr">
@@ -19328,6 +20065,11 @@
           <t>3D Pixar Disney style cheerful toddler dance coach, smooth playful animation, vibrant kindergarten studio, soft bright volumetric lighting, clean studio background, highly expressive face, full body dynamic camera shot: Song 'Morning Sunshine Hello', Action '第 14 節: 抬頭看天空好藍'. ☁️ 墊起腳尖手遮額頭，抬頭仰望美麗藍天！. The character is stretching arms up high to reach floating elements, standing on tiptoes, joyful posture, looking up with wonder. 4k resolution, 60fps, Disney Pixar render, joyful preschool music video style.</t>
         </is>
       </c>
+      <c r="K17" s="20" t="inlineStr">
+        <is>
+          <t>images/track_01/a1_s01_seg15_boy.jpg</t>
+        </is>
+      </c>
     </row>
     <row r="18" ht="30" customHeight="1">
       <c r="A18" s="8" t="inlineStr">
@@ -19376,6 +20118,11 @@
           <t>3D Pixar Disney style cheerful toddler dance coach, smooth playful animation, vibrant kindergarten studio, soft bright volumetric lighting, clean studio background, highly expressive face, full body dynamic camera shot: Song 'Morning Sunshine Hello', Action '第 15 節: 精彩探險等著你'. 💖 雙手在胸前比個大愛心，滿滿期待！. The character is bringing hands together at the chest forming an adorable glowing heart shape, leaning slightly forward, loving gentle smile. 4k resolution, 60fps, Disney Pixar render, joyful preschool music video style.</t>
         </is>
       </c>
+      <c r="K18" s="20" t="inlineStr">
+        <is>
+          <t>images/track_01/a1_s01_seg16_boy.jpg</t>
+        </is>
+      </c>
     </row>
     <row r="19" ht="30" customHeight="1">
       <c r="A19" s="10" t="inlineStr">
@@ -19424,6 +20171,11 @@
           <t>3D Pixar Disney style cheerful toddler dance coach, smooth playful animation, vibrant kindergarten studio, soft bright volumetric lighting, clean studio background, highly expressive face, full body dynamic camera shot: Song 'Morning Sunshine Hello', Action '第 16 節: 再次熱情大招手'. 👋 雙腳踩節奏，雙手像波浪歡樂招手！. The character is waving both hands overhead in friendly wide arcs, swaying gently from side to side, sparkling excited eyes. 4k resolution, 60fps, Disney Pixar render, joyful preschool music video style.</t>
         </is>
       </c>
+      <c r="K19" s="20" t="inlineStr">
+        <is>
+          <t>images/track_01/a1_s01_seg17_boy.jpg</t>
+        </is>
+      </c>
     </row>
     <row r="20" ht="30" customHeight="1">
       <c r="A20" s="8" t="inlineStr">
@@ -19472,6 +20224,11 @@
           <t>3D Pixar Disney style cheerful toddler dance coach, smooth playful animation, vibrant kindergarten studio, soft bright volumetric lighting, clean studio background, highly expressive face, full body dynamic camera shot: Song 'Morning Sunshine Hello', Action '第 17 節: 深蹲起跳歡呼耶'. 🐰 蹲下蓄力、高高起飛，小拳頭喊耶！. The character is squatting down and bursting into a high happy jump, feet kicking joyfully in mid-air, both fists punching the sky in victory. 4k resolution, 60fps, Disney Pixar render, joyful preschool music video style.</t>
         </is>
       </c>
+      <c r="K20" s="20" t="inlineStr">
+        <is>
+          <t>images/track_01/a1_s01_seg18_boy.jpg</t>
+        </is>
+      </c>
     </row>
     <row r="21" ht="30" customHeight="1">
       <c r="A21" s="10" t="inlineStr">
@@ -19520,6 +20277,11 @@
           <t>3D Pixar Disney style cheerful toddler dance coach, smooth playful animation, vibrant kindergarten studio, soft bright volumetric lighting, clean studio background, highly expressive face, full body dynamic camera shot: Song 'Morning Sunshine Hello', Action '第 18 節: 動感腳尖踢點步'. 👟 雙手插腰，左右小腳尖輕輕點地數數！. The character is marching in place energetically, hands on hips, knees lifting high in rhythmic bounce, enthusiastic happy smile. 4k resolution, 60fps, Disney Pixar render, joyful preschool music video style.</t>
         </is>
       </c>
+      <c r="K21" s="20" t="inlineStr">
+        <is>
+          <t>images/track_01/a1_s01_seg19_boy.jpg</t>
+        </is>
+      </c>
     </row>
     <row r="22" ht="30" customHeight="1">
       <c r="A22" s="8" t="inlineStr">
@@ -19568,6 +20330,11 @@
           <t>3D Pixar Disney style cheerful toddler dance coach, smooth playful animation, vibrant kindergarten studio, soft bright volumetric lighting, clean studio background, highly expressive face, full body dynamic camera shot: Song 'Morning Sunshine Hello', Action '第 19 節: 歡樂拍手合唱曲'. 👏 胸前大聲拍手：啪啪啪，身體彈動！. The character is waving both hands overhead in friendly wide arcs, swaying gently from side to side, sparkling excited eyes. 4k resolution, 60fps, Disney Pixar render, joyful preschool music video style.</t>
         </is>
       </c>
+      <c r="K22" s="20" t="inlineStr">
+        <is>
+          <t>images/track_01/a1_s01_seg20_boy.jpg</t>
+        </is>
+      </c>
     </row>
     <row r="23" ht="30" customHeight="1">
       <c r="A23" s="10" t="inlineStr">
@@ -19616,6 +20383,11 @@
           <t>3D Pixar Disney style cheerful toddler dance coach, smooth playful animation, vibrant kindergarten studio, soft bright volumetric lighting, clean studio background, highly expressive face, full body dynamic camera shot: Song 'Morning Sunshine Hello', Action '第 20 節: 白鴿展翅大滑翔'. 🕊️ 雙手水平展開像大鳥，隨微風滑翔！. The character is swaying hips and arms like a breeze, smooth fluid body roll, playful rhythmic dancing, friendly warm smile. 4k resolution, 60fps, Disney Pixar render, joyful preschool music video style.</t>
         </is>
       </c>
+      <c r="K23" s="20" t="inlineStr">
+        <is>
+          <t>images/track_01/a1_s01_seg21_boy.jpg</t>
+        </is>
+      </c>
     </row>
     <row r="24" ht="30" customHeight="1">
       <c r="A24" s="8" t="inlineStr">
@@ -19664,6 +20436,11 @@
           <t>3D Pixar Disney style cheerful toddler dance coach, smooth playful animation, vibrant kindergarten studio, soft bright volumetric lighting, clean studio background, highly expressive face, full body dynamic camera shot: Song 'Morning Sunshine Hello', Action '第 21 節: 擁抱世界道早安'. 🌍 雙臂向外畫大圓，擁抱美麗全世界！. The character is lifting arms from heart to sky creating a big golden sun circle, chest open, radiant beaming joyful smile. 4k resolution, 60fps, Disney Pixar render, joyful preschool music video style.</t>
         </is>
       </c>
+      <c r="K24" s="20" t="inlineStr">
+        <is>
+          <t>images/track_01/a1_s01_seg22_boy.jpg</t>
+        </is>
+      </c>
     </row>
     <row r="25" ht="30" customHeight="1">
       <c r="A25" s="10" t="inlineStr">
@@ -19710,6 +20487,11 @@
       <c r="J25" s="11" t="inlineStr">
         <is>
           <t>3D Pixar Disney style cheerful toddler dance coach, smooth playful animation, vibrant kindergarten studio, soft bright volumetric lighting, clean studio background, highly expressive face, full body dynamic camera shot: Song 'Morning Sunshine Hello', Action '第 22 節: 定格燦爛大微笑'. 🌟 雙手胸前比心鞠躬，定格燦爛笑容！. The character is bringing hands together at the chest forming an adorable glowing heart shape, leaning slightly forward, loving gentle smile. 4k resolution, 60fps, Disney Pixar render, joyful preschool music video style.</t>
+        </is>
+      </c>
+      <c r="K25" s="20" t="inlineStr">
+        <is>
+          <t>images/track_01/a1_s01_seg23_boy.jpg</t>
         </is>
       </c>
     </row>
@@ -19727,7 +20509,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J24"/>
+  <dimension ref="A1:K24"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="18" customWidth="1" min="1" max="1"/>
@@ -19740,6 +20522,7 @@
     <col width="30" customWidth="1" min="8" max="8"/>
     <col width="12" customWidth="1" min="9" max="9"/>
     <col width="55" customWidth="1" min="10" max="10"/>
+    <col width="34" customWidth="1" min="11" max="11"/>
   </cols>
   <sheetData>
     <row r="1" ht="32" customHeight="1">
@@ -19800,6 +20583,11 @@
           <t>AI 影片動畫生成提示詞 (Prompt)</t>
         </is>
       </c>
+      <c r="K2" s="19" t="inlineStr">
+        <is>
+          <t>首張圖片路徑 (9:16 720p)</t>
+        </is>
+      </c>
     </row>
     <row r="3" ht="30" customHeight="1">
       <c r="A3" s="10" t="inlineStr">
@@ -19848,6 +20636,11 @@
           <t>3D Pixar Disney style preschool animation video keyframe, vertical 9:16 aspect ratio 720p HD. Full body standing shot of the cheerful 5-year-old girl dance coach with brown curly pigtails tied with yellow ribbons, pink dance tee with smiling yellow star, yellow shorts, pink sneakers. In colorful kindergarten dance studio. Starter keyframe for action "[前奏] 數字小士兵預備踏步" (🔢 準備好小手小腳，踩出節拍踏步走！). The character is in lively dance starter pose, joyful radiant beaming smile, sparkling expressive eyes. 4k 3D Pixar render, clean frame without text overlay, starter keyframe for image-to-video generation (a1_s02_seg01_girl.jpg).</t>
         </is>
       </c>
+      <c r="K3" s="20" t="inlineStr">
+        <is>
+          <t>images/track_02/a1_s02_seg01_girl.jpg</t>
+        </is>
+      </c>
     </row>
     <row r="4" ht="30" customHeight="1">
       <c r="A4" s="8" t="inlineStr">
@@ -19896,6 +20689,11 @@
           <t>3D Pixar Disney style cheerful toddler dance coach, smooth playful animation, vibrant kindergarten studio, soft bright volumetric lighting, clean studio background, highly expressive face, full body dynamic camera shot: Song 'Count with Me 1 to 10', Action '第 01 節: 伸指比 1 摸蘋果'. 🍎 右手比 1 摘樹上紅蘋果！. The character is stretching arms up high to reach floating elements, standing on tiptoes, joyful posture, looking up with wonder. 4k resolution, 60fps, Disney Pixar render, joyful preschool music video style.</t>
         </is>
       </c>
+      <c r="K4" s="20" t="inlineStr">
+        <is>
+          <t>images/track_02/a1_s02_seg02_girl.jpg</t>
+        </is>
+      </c>
     </row>
     <row r="5" ht="30" customHeight="1">
       <c r="A5" s="10" t="inlineStr">
@@ -19944,6 +20742,11 @@
           <t>3D Pixar Disney style cheerful toddler dance coach, smooth playful animation, vibrant kindergarten studio, soft bright volumetric lighting, clean studio background, highly expressive face, full body dynamic camera shot: Song 'Count with Me 1 to 10', Action '第 02 節: 伸指比 2 學小鳥'. 🐦 雙手比 2 當小鳥翅膀搧呀搧！. The character is waving both hands overhead in friendly wide arcs, swaying gently from side to side, sparkling excited eyes. 4k resolution, 60fps, Disney Pixar render, joyful preschool music video style.</t>
         </is>
       </c>
+      <c r="K5" s="20" t="inlineStr">
+        <is>
+          <t>images/track_02/a1_s02_seg03_girl.jpg</t>
+        </is>
+      </c>
     </row>
     <row r="6" ht="30" customHeight="1">
       <c r="A6" s="8" t="inlineStr">
@@ -19992,6 +20795,11 @@
           <t>3D Pixar Disney style cheerful toddler dance coach, smooth playful animation, vibrant kindergarten studio, soft bright volumetric lighting, clean studio background, highly expressive face, full body dynamic camera shot: Song 'Count with Me 1 to 10', Action '第 03 節: 伸指比 3 滾滾球'. ⚽ 雙手比 3 在地面滾滾彩色小球！. The character is swaying hips and arms like a breeze, smooth fluid body roll, playful rhythmic dancing, friendly warm smile. 4k resolution, 60fps, Disney Pixar render, joyful preschool music video style.</t>
         </is>
       </c>
+      <c r="K6" s="20" t="inlineStr">
+        <is>
+          <t>images/track_02/a1_s02_seg04_girl.jpg</t>
+        </is>
+      </c>
     </row>
     <row r="7" ht="30" customHeight="1">
       <c r="A7" s="10" t="inlineStr">
@@ -20040,6 +20848,11 @@
           <t>3D Pixar Disney style cheerful toddler dance coach, smooth playful animation, vibrant kindergarten studio, soft bright volumetric lighting, clean studio background, highly expressive face, full body dynamic camera shot: Song 'Count with Me 1 to 10', Action '第 04 節: 伸指比 4 敲敲門'. 🐱 伸出 4 隻手指學小貓敲門咚咚咚！. The character is marching in place energetically, hands on hips, knees lifting high in rhythmic bounce, enthusiastic happy smile. 4k resolution, 60fps, Disney Pixar render, joyful preschool music video style.</t>
         </is>
       </c>
+      <c r="K7" s="20" t="inlineStr">
+        <is>
+          <t>images/track_02/a1_s02_seg05_girl.jpg</t>
+        </is>
+      </c>
     </row>
     <row r="8" ht="30" customHeight="1">
       <c r="A8" s="8" t="inlineStr">
@@ -20088,6 +20901,11 @@
           <t>3D Pixar Disney style cheerful toddler dance coach, smooth playful animation, vibrant kindergarten studio, soft bright volumetric lighting, clean studio background, highly expressive face, full body dynamic camera shot: Song 'Count with Me 1 to 10', Action '第 05 節: 伸出 5 指小蜜蜂'. 🐝 張開 5 隻手指學蜜蜂嗡嗡飛！. The character is waving both hands overhead in friendly wide arcs, swaying gently from side to side, sparkling excited eyes. 4k resolution, 60fps, Disney Pixar render, joyful preschool music video style.</t>
         </is>
       </c>
+      <c r="K8" s="20" t="inlineStr">
+        <is>
+          <t>images/track_02/a1_s02_seg06_girl.jpg</t>
+        </is>
+      </c>
     </row>
     <row r="9" ht="30" customHeight="1">
       <c r="A9" s="10" t="inlineStr">
@@ -20136,6 +20954,11 @@
           <t>3D Pixar Disney style cheerful toddler dance coach, smooth playful animation, vibrant kindergarten studio, soft bright volumetric lighting, clean studio background, highly expressive face, full body dynamic camera shot: Song 'Count with Me 1 to 10', Action '第 06 節: 數數朋友 1 到 5'. 🔢 伸出手指數一數身邊好朋友！. The character is marching in place energetically, hands on hips, knees lifting high in rhythmic bounce, enthusiastic happy smile. 4k resolution, 60fps, Disney Pixar render, joyful preschool music video style.</t>
         </is>
       </c>
+      <c r="K9" s="20" t="inlineStr">
+        <is>
+          <t>images/track_02/a1_s02_seg07_girl.jpg</t>
+        </is>
+      </c>
     </row>
     <row r="10" ht="30" customHeight="1">
       <c r="A10" s="8" t="inlineStr">
@@ -20184,6 +21007,11 @@
           <t>3D Pixar Disney style cheerful toddler dance coach, smooth playful animation, vibrant kindergarten studio, soft bright volumetric lighting, clean studio background, highly expressive face, full body dynamic camera shot: Song 'Count with Me 1 to 10', Action '第 07 節: 節奏拍手 1 2 3 4 5'. 👏 跟著重音連拍 5 下：1、2、3、4、5！. The character is squatting down and bursting into a high happy jump, feet kicking joyfully in mid-air, both fists punching the sky in victory. 4k resolution, 60fps, Disney Pixar render, joyful preschool music video style.</t>
         </is>
       </c>
+      <c r="K10" s="20" t="inlineStr">
+        <is>
+          <t>images/track_02/a1_s02_seg08_girl.jpg</t>
+        </is>
+      </c>
     </row>
     <row r="11" ht="30" customHeight="1">
       <c r="A11" s="10" t="inlineStr">
@@ -20232,6 +21060,11 @@
           <t>3D Pixar Disney style cheerful toddler dance coach, smooth playful animation, vibrant kindergarten studio, soft bright volumetric lighting, clean studio background, highly expressive face, full body dynamic camera shot: Song 'Count with Me 1 to 10', Action '第 08 節: 數字寶寶動起來'. ✨ 雙手插腰身體左右快樂扭一扭！. The character is swaying hips and arms like a breeze, smooth fluid body roll, playful rhythmic dancing, friendly warm smile. 4k resolution, 60fps, Disney Pixar render, joyful preschool music video style.</t>
         </is>
       </c>
+      <c r="K11" s="20" t="inlineStr">
+        <is>
+          <t>images/track_02/a1_s02_seg09_girl.jpg</t>
+        </is>
+      </c>
     </row>
     <row r="12" ht="30" customHeight="1">
       <c r="A12" s="8" t="inlineStr">
@@ -20280,6 +21113,11 @@
           <t>3D Pixar Disney style cheerful toddler dance coach, smooth playful animation, vibrant kindergarten studio, soft bright volumetric lighting, clean studio background, highly expressive face, full body dynamic camera shot: Song 'Count with Me 1 to 10', Action '第 09 節: 拍拍雙手踩踩鞋'. 👟 胸前大聲拍手，腳尖輕快踏地！. The character is marching in place energetically, hands on hips, knees lifting high in rhythmic bounce, enthusiastic happy smile. 4k resolution, 60fps, Disney Pixar render, joyful preschool music video style.</t>
         </is>
       </c>
+      <c r="K12" s="20" t="inlineStr">
+        <is>
+          <t>images/track_02/a1_s02_seg10_girl.jpg</t>
+        </is>
+      </c>
     </row>
     <row r="13" ht="30" customHeight="1">
       <c r="A13" s="10" t="inlineStr">
@@ -20328,6 +21166,11 @@
           <t>3D Pixar Disney style cheerful toddler dance coach, smooth playful animation, vibrant kindergarten studio, soft bright volumetric lighting, clean studio background, highly expressive face, full body dynamic camera shot: Song 'Count with Me 1 to 10', Action '第 10 節: 大家數數真開心'. 🌟 雙手高舉揮舞，數數越數越開心！. The character is lifting arms from heart to sky creating a big golden sun circle, chest open, radiant beaming joyful smile. 4k resolution, 60fps, Disney Pixar render, joyful preschool music video style.</t>
         </is>
       </c>
+      <c r="K13" s="20" t="inlineStr">
+        <is>
+          <t>images/track_02/a1_s02_seg11_girl.jpg</t>
+        </is>
+      </c>
     </row>
     <row r="14" ht="30" customHeight="1">
       <c r="A14" s="8" t="inlineStr">
@@ -20376,6 +21219,11 @@
           <t>3D Pixar Disney style cheerful toddler dance coach, smooth playful animation, vibrant kindergarten studio, soft bright volumetric lighting, clean studio background, highly expressive face, full body dynamic camera shot: Song 'Count with Me 1 to 10', Action '第 11 節: 伸指比 6 游水鴨'. 🦆 雙手比 6 學小鴨搖擺游游水！. The character is waving both hands overhead in friendly wide arcs, swaying gently from side to side, sparkling excited eyes. 4k resolution, 60fps, Disney Pixar render, joyful preschool music video style.</t>
         </is>
       </c>
+      <c r="K14" s="20" t="inlineStr">
+        <is>
+          <t>images/track_02/a1_s02_seg12_girl.jpg</t>
+        </is>
+      </c>
     </row>
     <row r="15" ht="30" customHeight="1">
       <c r="A15" s="10" t="inlineStr">
@@ -20424,6 +21272,11 @@
           <t>3D Pixar Disney style cheerful toddler dance coach, smooth playful animation, vibrant kindergarten studio, soft bright volumetric lighting, clean studio background, highly expressive face, full body dynamic camera shot: Song 'Count with Me 1 to 10', Action '第 12 節: 伸指比 7 吹蠟燭'. 🎂 雙手比 7 當生日蛋糕上的閃亮蠟燭！. The character is stretching arms up high to reach floating elements, standing on tiptoes, joyful posture, looking up with wonder. 4k resolution, 60fps, Disney Pixar render, joyful preschool music video style.</t>
         </is>
       </c>
+      <c r="K15" s="20" t="inlineStr">
+        <is>
+          <t>images/track_02/a1_s02_seg13_girl.jpg</t>
+        </is>
+      </c>
     </row>
     <row r="16" ht="30" customHeight="1">
       <c r="A16" s="8" t="inlineStr">
@@ -20472,6 +21325,11 @@
           <t>3D Pixar Disney style cheerful toddler dance coach, smooth playful animation, vibrant kindergarten studio, soft bright volumetric lighting, clean studio background, highly expressive face, full body dynamic camera shot: Song 'Count with Me 1 to 10', Action '第 13 節: 伸指比 8 划小船'. ⛵ 雙手比 8 當小帆船雙手划槳！. The character is swaying hips and arms like a breeze, smooth fluid body roll, playful rhythmic dancing, friendly warm smile. 4k resolution, 60fps, Disney Pixar render, joyful preschool music video style.</t>
         </is>
       </c>
+      <c r="K16" s="20" t="inlineStr">
+        <is>
+          <t>images/track_02/a1_s02_seg14_girl.jpg</t>
+        </is>
+      </c>
     </row>
     <row r="17" ht="30" customHeight="1">
       <c r="A17" s="10" t="inlineStr">
@@ -20520,6 +21378,11 @@
           <t>3D Pixar Disney style cheerful toddler dance coach, smooth playful animation, vibrant kindergarten studio, soft bright volumetric lighting, clean studio background, highly expressive face, full body dynamic camera shot: Song 'Count with Me 1 to 10', Action '第 14 節: 伸指比 9 升氣球'. 🎈 伸指比 9 抬頭看彩色氣球飄上天！. The character is stretching arms up high to reach floating elements, standing on tiptoes, joyful posture, looking up with wonder. 4k resolution, 60fps, Disney Pixar render, joyful preschool music video style.</t>
         </is>
       </c>
+      <c r="K17" s="20" t="inlineStr">
+        <is>
+          <t>images/track_02/a1_s02_seg15_girl.jpg</t>
+        </is>
+      </c>
     </row>
     <row r="18" ht="30" customHeight="1">
       <c r="A18" s="8" t="inlineStr">
@@ -20568,6 +21431,11 @@
           <t>3D Pixar Disney style cheerful toddler dance coach, smooth playful animation, vibrant kindergarten studio, soft bright volumetric lighting, clean studio background, highly expressive face, full body dynamic camera shot: Song 'Count with Me 1 to 10', Action '第 15 節: 十顆星星閃亮亮'. ⭐ 雙手高舉十指張開，像繁星閃爍！. The character is lifting arms from heart to sky creating a big golden sun circle, chest open, radiant beaming joyful smile. 4k resolution, 60fps, Disney Pixar render, joyful preschool music video style.</t>
         </is>
       </c>
+      <c r="K18" s="20" t="inlineStr">
+        <is>
+          <t>images/track_02/a1_s02_seg16_girl.jpg</t>
+        </is>
+      </c>
     </row>
     <row r="19" ht="30" customHeight="1">
       <c r="A19" s="10" t="inlineStr">
@@ -20616,6 +21484,11 @@
           <t>3D Pixar Disney style cheerful toddler dance coach, smooth playful animation, vibrant kindergarten studio, soft bright volumetric lighting, clean studio background, highly expressive face, full body dynamic camera shot: Song 'Count with Me 1 to 10', Action '第 16 節: 點亮夜空數數星'. ✨ 左右輕柔擺手，繁星照亮整片天空！. The character is swaying hips and arms like a breeze, smooth fluid body roll, playful rhythmic dancing, friendly warm smile. 4k resolution, 60fps, Disney Pixar render, joyful preschool music video style.</t>
         </is>
       </c>
+      <c r="K19" s="20" t="inlineStr">
+        <is>
+          <t>images/track_02/a1_s02_seg17_girl.jpg</t>
+        </is>
+      </c>
     </row>
     <row r="20" ht="30" customHeight="1">
       <c r="A20" s="8" t="inlineStr">
@@ -20664,6 +21537,11 @@
           <t>3D Pixar Disney style cheerful toddler dance coach, smooth playful animation, vibrant kindergarten studio, soft bright volumetric lighting, clean studio background, highly expressive face, full body dynamic camera shot: Song 'Count with Me 1 to 10', Action '第 17 節: 大家齊數 1 到 10'. 🔢 伸出十根手指頭，大聲數 1 到 10！. The character is marching in place energetically, hands on hips, knees lifting high in rhythmic bounce, enthusiastic happy smile. 4k resolution, 60fps, Disney Pixar render, joyful preschool music video style.</t>
         </is>
       </c>
+      <c r="K20" s="20" t="inlineStr">
+        <is>
+          <t>images/track_02/a1_s02_seg18_girl.jpg</t>
+        </is>
+      </c>
     </row>
     <row r="21" ht="30" customHeight="1">
       <c r="A21" s="10" t="inlineStr">
@@ -20712,6 +21590,11 @@
           <t>3D Pixar Disney style cheerful toddler dance coach, smooth playful animation, vibrant kindergarten studio, soft bright volumetric lighting, clean studio background, highly expressive face, full body dynamic camera shot: Song 'Count with Me 1 to 10', Action '第 18 節: 全體高聲齊歡唱'. 🎶 張開雙臂放聲歌唱，整齊踩步！. The character is stretching arms up high to reach floating elements, standing on tiptoes, joyful posture, looking up with wonder. 4k resolution, 60fps, Disney Pixar render, joyful preschool music video style.</t>
         </is>
       </c>
+      <c r="K21" s="20" t="inlineStr">
+        <is>
+          <t>images/track_02/a1_s02_seg19_girl.jpg</t>
+        </is>
+      </c>
     </row>
     <row r="22" ht="30" customHeight="1">
       <c r="A22" s="8" t="inlineStr">
@@ -20760,6 +21643,11 @@
           <t>3D Pixar Disney style cheerful toddler dance coach, smooth playful animation, vibrant kindergarten studio, soft bright volumetric lighting, clean studio background, highly expressive face, full body dynamic camera shot: Song 'Count with Me 1 to 10', Action '第 19 節: 動感拍手踩踩鞋'. 👟 拍拍手拍拍膝蓋，小腳踏踏踏！. The character is marching in place energetically, hands on hips, knees lifting high in rhythmic bounce, enthusiastic happy smile. 4k resolution, 60fps, Disney Pixar render, joyful preschool music video style.</t>
         </is>
       </c>
+      <c r="K22" s="20" t="inlineStr">
+        <is>
+          <t>images/track_02/a1_s02_seg20_girl.jpg</t>
+        </is>
+      </c>
     </row>
     <row r="23" ht="30" customHeight="1">
       <c r="A23" s="10" t="inlineStr">
@@ -20808,6 +21696,11 @@
           <t>3D Pixar Disney style cheerful toddler dance coach, smooth playful animation, vibrant kindergarten studio, soft bright volumetric lighting, clean studio background, highly expressive face, full body dynamic camera shot: Song 'Count with Me 1 to 10', Action '第 20 節: 數數大師好神氣'. 🎉 雙手叉腰挺胸，我們都是數數小神童！. The character is bringing hands together at the chest forming an adorable glowing heart shape, leaning slightly forward, loving gentle smile. 4k resolution, 60fps, Disney Pixar render, joyful preschool music video style.</t>
         </is>
       </c>
+      <c r="K23" s="20" t="inlineStr">
+        <is>
+          <t>images/track_02/a1_s02_seg21_girl.jpg</t>
+        </is>
+      </c>
     </row>
     <row r="24" ht="30" customHeight="1">
       <c r="A24" s="8" t="inlineStr">
@@ -20854,6 +21747,11 @@
       <c r="J24" s="9" t="inlineStr">
         <is>
           <t>3D Pixar Disney style cheerful toddler dance coach, smooth playful animation, vibrant kindergarten studio, soft bright volumetric lighting, clean studio background, highly expressive face, full body dynamic camera shot: Song 'Count with Me 1 to 10', Action '第 21 節: 完美的 10 大定格'. ⭐ 雙手比出十全十美大招手定格！. The character is lifting arms from heart to sky creating a big golden sun circle, chest open, radiant beaming joyful smile. 4k resolution, 60fps, Disney Pixar render, joyful preschool music video style.</t>
+        </is>
+      </c>
+      <c r="K24" s="20" t="inlineStr">
+        <is>
+          <t>images/track_02/a1_s02_seg22_girl.jpg</t>
         </is>
       </c>
     </row>
@@ -20871,7 +21769,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J24"/>
+  <dimension ref="A1:K24"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="18" customWidth="1" min="1" max="1"/>
@@ -20884,6 +21782,7 @@
     <col width="30" customWidth="1" min="8" max="8"/>
     <col width="12" customWidth="1" min="9" max="9"/>
     <col width="55" customWidth="1" min="10" max="10"/>
+    <col width="34" customWidth="1" min="11" max="11"/>
   </cols>
   <sheetData>
     <row r="1" ht="32" customHeight="1">
@@ -20944,6 +21843,11 @@
           <t>AI 影片動畫生成提示詞 (Prompt)</t>
         </is>
       </c>
+      <c r="K2" s="19" t="inlineStr">
+        <is>
+          <t>首張圖片路徑 (9:16 720p)</t>
+        </is>
+      </c>
     </row>
     <row r="3" ht="30" customHeight="1">
       <c r="A3" s="10" t="inlineStr">
@@ -20992,6 +21896,11 @@
           <t>3D Pixar Disney style preschool animation video keyframe, vertical 9:16 aspect ratio 720p HD. Full body standing shot of the cheerful 5-year-old girl dance coach with brown curly pigtails tied with yellow ribbons, pink dance tee with smiling yellow star, yellow shorts, pink sneakers. In colorful kindergarten dance studio. Starter keyframe for action "[前奏] 彩虹畫筆小預備" (🎨 拿起神奇彩色畫筆，準備為天空塗鴉！). The character is in lively dance starter pose, joyful radiant beaming smile, sparkling expressive eyes. 4k 3D Pixar render, clean frame without text overlay, starter keyframe for image-to-video generation (a1_s03_seg01_girl.jpg).</t>
         </is>
       </c>
+      <c r="K3" s="20" t="inlineStr">
+        <is>
+          <t>images/track_03/a1_s03_seg01_girl.jpg</t>
+        </is>
+      </c>
     </row>
     <row r="4" ht="30" customHeight="1">
       <c r="A4" s="8" t="inlineStr">
@@ -21040,6 +21949,11 @@
           <t>3D Pixar Disney style cheerful toddler dance coach, smooth playful animation, vibrant kindergarten studio, soft bright volumetric lighting, clean studio background, highly expressive face, full body dynamic camera shot: Song 'Rainbow Color Splash', Action '第 01 節: 紅紅櫻桃與玫瑰'. 🍒 雙手胸前抱大圓，比出紅紅甜櫻桃！. The character is bringing hands together at the chest forming an adorable glowing heart shape, leaning slightly forward, loving gentle smile. 4k resolution, 60fps, Disney Pixar render, joyful preschool music video style.</t>
         </is>
       </c>
+      <c r="K4" s="20" t="inlineStr">
+        <is>
+          <t>images/track_03/a1_s03_seg02_girl.jpg</t>
+        </is>
+      </c>
     </row>
     <row r="5" ht="30" customHeight="1">
       <c r="A5" s="10" t="inlineStr">
@@ -21088,6 +22002,11 @@
           <t>3D Pixar Disney style cheerful toddler dance coach, smooth playful animation, vibrant kindergarten studio, soft bright volumetric lighting, clean studio background, highly expressive face, full body dynamic camera shot: Song 'Rainbow Color Splash', Action '第 02 節: 紅紅按鈕小鼻子'. 👃 食指輕輕點點小鼻子，俏皮笑一笑！. The character is stretching arms up high to reach floating elements, standing on tiptoes, joyful posture, looking up with wonder. 4k resolution, 60fps, Disney Pixar render, joyful preschool music video style.</t>
         </is>
       </c>
+      <c r="K5" s="20" t="inlineStr">
+        <is>
+          <t>images/track_03/a1_s03_seg03_girl.jpg</t>
+        </is>
+      </c>
     </row>
     <row r="6" ht="30" customHeight="1">
       <c r="A6" s="8" t="inlineStr">
@@ -21136,6 +22055,11 @@
           <t>3D Pixar Disney style cheerful toddler dance coach, smooth playful animation, vibrant kindergarten studio, soft bright volumetric lighting, clean studio background, highly expressive face, full body dynamic camera shot: Song 'Rainbow Color Splash', Action '第 03 節: 暖暖金黃大太陽'. ☀️ 雙手向外劃出金色大圓圈，暖洋洋！. The character is lifting arms from heart to sky creating a big golden sun circle, chest open, radiant beaming joyful smile. 4k resolution, 60fps, Disney Pixar render, joyful preschool music video style.</t>
         </is>
       </c>
+      <c r="K6" s="20" t="inlineStr">
+        <is>
+          <t>images/track_03/a1_s03_seg04_girl.jpg</t>
+        </is>
+      </c>
     </row>
     <row r="7" ht="30" customHeight="1">
       <c r="A7" s="10" t="inlineStr">
@@ -21184,6 +22108,11 @@
           <t>3D Pixar Disney style cheerful toddler dance coach, smooth playful animation, vibrant kindergarten studio, soft bright volumetric lighting, clean studio background, highly expressive face, full body dynamic camera shot: Song 'Rainbow Color Splash', Action '第 04 節: 夜空星星黃澄澄'. ⭐ 雙手向上摘星星，小手指眨呀眨！. The character is stretching arms up high to reach floating elements, standing on tiptoes, joyful posture, looking up with wonder. 4k resolution, 60fps, Disney Pixar render, joyful preschool music video style.</t>
         </is>
       </c>
+      <c r="K7" s="20" t="inlineStr">
+        <is>
+          <t>images/track_03/a1_s03_seg05_girl.jpg</t>
+        </is>
+      </c>
     </row>
     <row r="8" ht="30" customHeight="1">
       <c r="A8" s="8" t="inlineStr">
@@ -21232,6 +22161,11 @@
           <t>3D Pixar Disney style cheerful toddler dance coach, smooth playful animation, vibrant kindergarten studio, soft bright volumetric lighting, clean studio background, highly expressive face, full body dynamic camera shot: Song 'Rainbow Color Splash', Action '第 05 節: 大海蔚藍又寬廣'. 🌊 雙臂像波浪左右推動，學大海起伏！. The character is swaying hips and arms like a breeze, smooth fluid body roll, playful rhythmic dancing, friendly warm smile. 4k resolution, 60fps, Disney Pixar render, joyful preschool music video style.</t>
         </is>
       </c>
+      <c r="K8" s="20" t="inlineStr">
+        <is>
+          <t>images/track_03/a1_s03_seg06_girl.jpg</t>
+        </is>
+      </c>
     </row>
     <row r="9" ht="30" customHeight="1">
       <c r="A9" s="10" t="inlineStr">
@@ -21280,6 +22214,11 @@
           <t>3D Pixar Disney style cheerful toddler dance coach, smooth playful animation, vibrant kindergarten studio, soft bright volumetric lighting, clean studio background, highly expressive face, full body dynamic camera shot: Song 'Rainbow Color Splash', Action '第 06 節: 藍色浪花向前衝'. 🏄 身體微蹲向前划水，浪花四濺！. The character is marching in place energetically, hands on hips, knees lifting high in rhythmic bounce, enthusiastic happy smile. 4k resolution, 60fps, Disney Pixar render, joyful preschool music video style.</t>
         </is>
       </c>
+      <c r="K9" s="20" t="inlineStr">
+        <is>
+          <t>images/track_03/a1_s03_seg07_girl.jpg</t>
+        </is>
+      </c>
     </row>
     <row r="10" ht="30" customHeight="1">
       <c r="A10" s="8" t="inlineStr">
@@ -21328,6 +22267,11 @@
           <t>3D Pixar Disney style cheerful toddler dance coach, smooth playful animation, vibrant kindergarten studio, soft bright volumetric lighting, clean studio background, highly expressive face, full body dynamic camera shot: Song 'Rainbow Color Splash', Action '第 07 節: 紅黃綠藍齊點名'. 🎨 雙手輪流前推點出四種神奇顏色！. The character is waving both hands overhead in friendly wide arcs, swaying gently from side to side, sparkling excited eyes. 4k resolution, 60fps, Disney Pixar render, joyful preschool music video style.</t>
         </is>
       </c>
+      <c r="K10" s="20" t="inlineStr">
+        <is>
+          <t>images/track_03/a1_s03_seg08_girl.jpg</t>
+        </is>
+      </c>
     </row>
     <row r="11" ht="30" customHeight="1">
       <c r="A11" s="10" t="inlineStr">
@@ -21376,6 +22320,11 @@
           <t>3D Pixar Disney style cheerful toddler dance coach, smooth playful animation, vibrant kindergarten studio, soft bright volumetric lighting, clean studio background, highly expressive face, full body dynamic camera shot: Song 'Rainbow Color Splash', Action '第 08 節: 搭起彩色大虹橋'. 🌈 雙臂在頭頂畫出橫跨天空的彩虹橋！. The character is lifting arms from heart to sky creating a big golden sun circle, chest open, radiant beaming joyful smile. 4k resolution, 60fps, Disney Pixar render, joyful preschool music video style.</t>
         </is>
       </c>
+      <c r="K11" s="20" t="inlineStr">
+        <is>
+          <t>images/track_03/a1_s03_seg09_girl.jpg</t>
+        </is>
+      </c>
     </row>
     <row r="12" ht="30" customHeight="1">
       <c r="A12" s="8" t="inlineStr">
@@ -21424,6 +22373,11 @@
           <t>3D Pixar Disney style cheerful toddler dance coach, smooth playful animation, vibrant kindergarten studio, soft bright volumetric lighting, clean studio background, highly expressive face, full body dynamic camera shot: Song 'Rainbow Color Splash', Action '第 09 節: 色彩魔法融合轉'. 🔄 雙手交疊攪拌魔法色彩，轉個小圈！. The character is swaying hips and arms like a breeze, smooth fluid body roll, playful rhythmic dancing, friendly warm smile. 4k resolution, 60fps, Disney Pixar render, joyful preschool music video style.</t>
         </is>
       </c>
+      <c r="K12" s="20" t="inlineStr">
+        <is>
+          <t>images/track_03/a1_s03_seg10_girl.jpg</t>
+        </is>
+      </c>
     </row>
     <row r="13" ht="30" customHeight="1">
       <c r="A13" s="10" t="inlineStr">
@@ -21472,6 +22426,11 @@
           <t>3D Pixar Disney style cheerful toddler dance coach, smooth playful animation, vibrant kindergarten studio, soft bright volumetric lighting, clean studio background, highly expressive face, full body dynamic camera shot: Song 'Rainbow Color Splash', Action '第 10 節: 閃亮色彩好耀眼'. ✨ 雙手十指向外綻放，像煙火閃爍！. The character is squatting down and bursting into a high happy jump, feet kicking joyfully in mid-air, both fists punching the sky in victory. 4k resolution, 60fps, Disney Pixar render, joyful preschool music video style.</t>
         </is>
       </c>
+      <c r="K13" s="20" t="inlineStr">
+        <is>
+          <t>images/track_03/a1_s03_seg11_girl.jpg</t>
+        </is>
+      </c>
     </row>
     <row r="14" ht="30" customHeight="1">
       <c r="A14" s="8" t="inlineStr">
@@ -21520,6 +22479,11 @@
           <t>3D Pixar Disney style cheerful toddler dance coach, smooth playful animation, vibrant kindergarten studio, soft bright volumetric lighting, clean studio background, highly expressive face, full body dynamic camera shot: Song 'Rainbow Color Splash', Action '第 11 節: 青青小草小兔跳'. 🐰 雙手放頭頂當兔耳，輕快蹦蹦跳！. The character is squatting down and bursting into a high happy jump, feet kicking joyfully in mid-air, both fists punching the sky in victory. 4k resolution, 60fps, Disney Pixar render, joyful preschool music video style.</t>
         </is>
       </c>
+      <c r="K14" s="20" t="inlineStr">
+        <is>
+          <t>images/track_03/a1_s03_seg12_girl.jpg</t>
+        </is>
+      </c>
     </row>
     <row r="15" ht="30" customHeight="1">
       <c r="A15" s="10" t="inlineStr">
@@ -21568,6 +22532,11 @@
           <t>3D Pixar Disney style cheerful toddler dance coach, smooth playful animation, vibrant kindergarten studio, soft bright volumetric lighting, clean studio background, highly expressive face, full body dynamic camera shot: Song 'Rainbow Color Splash', Action '第 12 節: 綠綠大樹參天長'. 🌲 雙腳站穩雙手上伸，像大樹高高生長！. The character is lifting arms from heart to sky creating a big golden sun circle, chest open, radiant beaming joyful smile. 4k resolution, 60fps, Disney Pixar render, joyful preschool music video style.</t>
         </is>
       </c>
+      <c r="K15" s="20" t="inlineStr">
+        <is>
+          <t>images/track_03/a1_s03_seg13_girl.jpg</t>
+        </is>
+      </c>
     </row>
     <row r="16" ht="30" customHeight="1">
       <c r="A16" s="8" t="inlineStr">
@@ -21616,6 +22585,11 @@
           <t>3D Pixar Disney style cheerful toddler dance coach, smooth playful animation, vibrant kindergarten studio, soft bright volumetric lighting, clean studio background, highly expressive face, full body dynamic camera shot: Song 'Rainbow Color Splash', Action '第 13 節: 圓圓南瓜甜又香'. 🎃 雙臂胸前抱出圓滾滾大南瓜！. The character is bringing hands together at the chest forming an adorable glowing heart shape, leaning slightly forward, loving gentle smile. 4k resolution, 60fps, Disney Pixar render, joyful preschool music video style.</t>
         </is>
       </c>
+      <c r="K16" s="20" t="inlineStr">
+        <is>
+          <t>images/track_03/a1_s03_seg14_girl.jpg</t>
+        </is>
+      </c>
     </row>
     <row r="17" ht="30" customHeight="1">
       <c r="A17" s="10" t="inlineStr">
@@ -21664,6 +22638,11 @@
           <t>3D Pixar Disney style cheerful toddler dance coach, smooth playful animation, vibrant kindergarten studio, soft bright volumetric lighting, clean studio background, highly expressive face, full body dynamic camera shot: Song 'Rainbow Color Splash', Action '第 14 節: 紫色葡萄摘一串'. 🍇 伸手向上摘葡萄，大口吃進嘴裡！. The character is stretching arms up high to reach floating elements, standing on tiptoes, joyful posture, looking up with wonder. 4k resolution, 60fps, Disney Pixar render, joyful preschool music video style.</t>
         </is>
       </c>
+      <c r="K17" s="20" t="inlineStr">
+        <is>
+          <t>images/track_03/a1_s03_seg15_girl.jpg</t>
+        </is>
+      </c>
     </row>
     <row r="18" ht="30" customHeight="1">
       <c r="A18" s="8" t="inlineStr">
@@ -21712,6 +22691,11 @@
           <t>3D Pixar Disney style cheerful toddler dance coach, smooth playful animation, vibrant kindergarten studio, soft bright volumetric lighting, clean studio background, highly expressive face, full body dynamic camera shot: Song 'Rainbow Color Splash', Action '第 15 節: 畫筆蘸色轉一轉'. 🖌️ 手握大畫筆在空中旋轉畫圈圈！. The character is swaying hips and arms like a breeze, smooth fluid body roll, playful rhythmic dancing, friendly warm smile. 4k resolution, 60fps, Disney Pixar render, joyful preschool music video style.</t>
         </is>
       </c>
+      <c r="K18" s="20" t="inlineStr">
+        <is>
+          <t>images/track_03/a1_s03_seg16_girl.jpg</t>
+        </is>
+      </c>
     </row>
     <row r="19" ht="30" customHeight="1">
       <c r="A19" s="10" t="inlineStr">
@@ -21760,6 +22744,11 @@
           <t>3D Pixar Disney style cheerful toddler dance coach, smooth playful animation, vibrant kindergarten studio, soft bright volumetric lighting, clean studio background, highly expressive face, full body dynamic camera shot: Song 'Rainbow Color Splash', Action '第 16 節: 彩繪快樂全世界'. 🌍 雙手大幅度揮灑，給全世界塗上色彩！. The character is waving both hands overhead in friendly wide arcs, swaying gently from side to side, sparkling excited eyes. 4k resolution, 60fps, Disney Pixar render, joyful preschool music video style.</t>
         </is>
       </c>
+      <c r="K19" s="20" t="inlineStr">
+        <is>
+          <t>images/track_03/a1_s03_seg17_girl.jpg</t>
+        </is>
+      </c>
     </row>
     <row r="20" ht="30" customHeight="1">
       <c r="A20" s="8" t="inlineStr">
@@ -21808,6 +22797,11 @@
           <t>3D Pixar Disney style cheerful toddler dance coach, smooth playful animation, vibrant kindergarten studio, soft bright volumetric lighting, clean studio background, highly expressive face, full body dynamic camera shot: Song 'Rainbow Color Splash', Action '第 17 節: 紅黃綠藍唱彩虹'. 🎶 跟著節拍拍拍手，唱響彩虹之歌！. The character is marching in place energetically, hands on hips, knees lifting high in rhythmic bounce, enthusiastic happy smile. 4k resolution, 60fps, Disney Pixar render, joyful preschool music video style.</t>
         </is>
       </c>
+      <c r="K20" s="20" t="inlineStr">
+        <is>
+          <t>images/track_03/a1_s03_seg18_girl.jpg</t>
+        </is>
+      </c>
     </row>
     <row r="21" ht="30" customHeight="1">
       <c r="A21" s="10" t="inlineStr">
@@ -21856,6 +22850,11 @@
           <t>3D Pixar Disney style cheerful toddler dance coach, smooth playful animation, vibrant kindergarten studio, soft bright volumetric lighting, clean studio background, highly expressive face, full body dynamic camera shot: Song 'Rainbow Color Splash', Action '第 18 節: 友情彩虹永相連'. 🤝 雙手向兩側伸出，搭起友誼橋樑！. The character is stretching arms up high to reach floating elements, standing on tiptoes, joyful posture, looking up with wonder. 4k resolution, 60fps, Disney Pixar render, joyful preschool music video style.</t>
         </is>
       </c>
+      <c r="K21" s="20" t="inlineStr">
+        <is>
+          <t>images/track_03/a1_s03_seg19_girl.jpg</t>
+        </is>
+      </c>
     </row>
     <row r="22" ht="30" customHeight="1">
       <c r="A22" s="8" t="inlineStr">
@@ -21904,6 +22903,11 @@
           <t>3D Pixar Disney style cheerful toddler dance coach, smooth playful animation, vibrant kindergarten studio, soft bright volumetric lighting, clean studio background, highly expressive face, full body dynamic camera shot: Song 'Rainbow Color Splash', Action '第 19 節: 魔法色彩閃閃光'. ✨ 身體輕快彈動，十指閃爍小星星！. The character is squatting down and bursting into a high happy jump, feet kicking joyfully in mid-air, both fists punching the sky in victory. 4k resolution, 60fps, Disney Pixar render, joyful preschool music video style.</t>
         </is>
       </c>
+      <c r="K22" s="20" t="inlineStr">
+        <is>
+          <t>images/track_03/a1_s03_seg20_girl.jpg</t>
+        </is>
+      </c>
     </row>
     <row r="23" ht="30" customHeight="1">
       <c r="A23" s="10" t="inlineStr">
@@ -21952,6 +22956,11 @@
           <t>3D Pixar Disney style cheerful toddler dance coach, smooth playful animation, vibrant kindergarten studio, soft bright volumetric lighting, clean studio background, highly expressive face, full body dynamic camera shot: Song 'Rainbow Color Splash', Action '第 20 節: 繽紛色彩你和我'. 💖 雙手收回胸前比愛心，相親相愛！. The character is bringing hands together at the chest forming an adorable glowing heart shape, leaning slightly forward, loving gentle smile. 4k resolution, 60fps, Disney Pixar render, joyful preschool music video style.</t>
         </is>
       </c>
+      <c r="K23" s="20" t="inlineStr">
+        <is>
+          <t>images/track_03/a1_s03_seg21_girl.jpg</t>
+        </is>
+      </c>
     </row>
     <row r="24" ht="30" customHeight="1">
       <c r="A24" s="8" t="inlineStr">
@@ -21998,6 +23007,11 @@
       <c r="J24" s="9" t="inlineStr">
         <is>
           <t>3D Pixar Disney style cheerful toddler dance coach, smooth playful animation, vibrant kindergarten studio, soft bright volumetric lighting, clean studio background, highly expressive face, full body dynamic camera shot: Song 'Rainbow Color Splash', Action '第 21 節: 天空彩虹好美麗'. 🌈 雙手由兩側向上畫大彩虹，定格微笑！. The character is lifting arms from heart to sky creating a big golden sun circle, chest open, radiant beaming joyful smile. 4k resolution, 60fps, Disney Pixar render, joyful preschool music video style.</t>
+        </is>
+      </c>
+      <c r="K24" s="20" t="inlineStr">
+        <is>
+          <t>images/track_03/a1_s03_seg22_girl.jpg</t>
         </is>
       </c>
     </row>
@@ -22015,7 +23029,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J28"/>
+  <dimension ref="A1:K28"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="18" customWidth="1" min="1" max="1"/>
@@ -22028,6 +23042,7 @@
     <col width="30" customWidth="1" min="8" max="8"/>
     <col width="12" customWidth="1" min="9" max="9"/>
     <col width="55" customWidth="1" min="10" max="10"/>
+    <col width="34" customWidth="1" min="11" max="11"/>
   </cols>
   <sheetData>
     <row r="1" ht="32" customHeight="1">
@@ -22088,6 +23103,11 @@
           <t>AI 影片動畫生成提示詞 (Prompt)</t>
         </is>
       </c>
+      <c r="K2" s="19" t="inlineStr">
+        <is>
+          <t>首張圖片路徑 (9:16 720p)</t>
+        </is>
+      </c>
     </row>
     <row r="3" ht="30" customHeight="1">
       <c r="A3" s="10" t="inlineStr">
@@ -22136,6 +23156,11 @@
           <t>3D Pixar Disney style preschool animation video keyframe, vertical 9:16 aspect ratio 720p HD. Full body standing shot of the cheerful 5-year-old boy dance coach in bright blue athletic t-shirt with orange center and KIDS DANCE logo, blue shorts, orange running sneakers. In colorful kindergarten dance studio. Starter keyframe for action "[前奏] 森林號角精神踏步" (🎺 聽號角吹響！雙手插腰，膝蓋抬高大步踏走！). The character is in lively dance starter pose, joyful radiant beaming smile, sparkling expressive eyes. 4k 3D Pixar render, clean frame without text overlay, starter keyframe for image-to-video generation (a1_s04_seg01_boy.jpg).</t>
         </is>
       </c>
+      <c r="K3" s="20" t="inlineStr">
+        <is>
+          <t>images/track_04/a1_s04_seg01_boy.jpg</t>
+        </is>
+      </c>
     </row>
     <row r="4" ht="30" customHeight="1">
       <c r="A4" s="8" t="inlineStr">
@@ -22184,6 +23209,11 @@
           <t>3D Pixar Disney style cheerful toddler dance coach, smooth playful animation, vibrant kindergarten studio, soft bright volumetric lighting, clean studio background, highly expressive face, full body dynamic camera shot: Song 'Animal Safari March', Action '第 01 節: 一二踏步進行曲'. 🥁 喊出一二一二，整齊精神原地踏步！. The character is marching in place energetically, hands on hips, knees lifting high in rhythmic bounce, enthusiastic happy smile. 4k resolution, 60fps, Disney Pixar render, joyful preschool music video style.</t>
         </is>
       </c>
+      <c r="K4" s="20" t="inlineStr">
+        <is>
+          <t>images/track_04/a1_s04_seg02_boy.jpg</t>
+        </is>
+      </c>
     </row>
     <row r="5" ht="30" customHeight="1">
       <c r="A5" s="10" t="inlineStr">
@@ -22232,6 +23262,11 @@
           <t>3D Pixar Disney style cheerful toddler dance coach, smooth playful animation, vibrant kindergarten studio, soft bright volumetric lighting, clean studio background, highly expressive face, full body dynamic camera shot: Song 'Animal Safari March', Action '[旋律間奏] 動作接續歡樂跳'. 🔄 雙手插腰踩小碎步，轉個歡樂大圓圈，保持微笑！. The character is swaying hips and arms like a breeze, smooth fluid body roll, playful rhythmic dancing, friendly warm smile. 4k resolution, 60fps, Disney Pixar render, joyful preschool music video style.</t>
         </is>
       </c>
+      <c r="K5" s="20" t="inlineStr">
+        <is>
+          <t>images/track_04/a1_s04_seg03_boy.jpg</t>
+        </is>
+      </c>
     </row>
     <row r="6" ht="30" customHeight="1">
       <c r="A6" s="8" t="inlineStr">
@@ -22280,6 +23315,11 @@
           <t>3D Pixar Disney style cheerful toddler dance coach, smooth playful animation, vibrant kindergarten studio, soft bright volumetric lighting, clean studio background, highly expressive face, full body dynamic camera shot: Song 'Animal Safari March', Action '第 02 節: 大象重重踏步走'. 🐘 雙手放鼻子前做長長鼻子，重重踏步！. The character is marching in place energetically, hands on hips, knees lifting high in rhythmic bounce, enthusiastic happy smile. 4k resolution, 60fps, Disney Pixar render, joyful preschool music video style.</t>
         </is>
       </c>
+      <c r="K6" s="20" t="inlineStr">
+        <is>
+          <t>images/track_04/a1_s04_seg04_boy.jpg</t>
+        </is>
+      </c>
     </row>
     <row r="7" ht="30" customHeight="1">
       <c r="A7" s="10" t="inlineStr">
@@ -22328,6 +23368,11 @@
           <t>3D Pixar Disney style cheerful toddler dance coach, smooth playful animation, vibrant kindergarten studio, soft bright volumetric lighting, clean studio background, highly expressive face, full body dynamic camera shot: Song 'Animal Safari March', Action '第 03 節: 粉紅小豬泥巴滾'. 🐷 雙手小拳揉鼻鼻，學小豬拱拱叫！. The character is swaying hips and arms like a breeze, smooth fluid body roll, playful rhythmic dancing, friendly warm smile. 4k resolution, 60fps, Disney Pixar render, joyful preschool music video style.</t>
         </is>
       </c>
+      <c r="K7" s="20" t="inlineStr">
+        <is>
+          <t>images/track_04/a1_s04_seg05_boy.jpg</t>
+        </is>
+      </c>
     </row>
     <row r="8" ht="30" customHeight="1">
       <c r="A8" s="8" t="inlineStr">
@@ -22376,6 +23421,11 @@
           <t>3D Pixar Disney style cheerful toddler dance coach, smooth playful animation, vibrant kindergarten studio, soft bright volumetric lighting, clean studio background, highly expressive face, full body dynamic camera shot: Song 'Animal Safari March', Action '第 04 節: 猴子樹梢盪鞦韆'. 🐵 雙手交替向上攀爬樹枝，身體擺盪！. The character is stretching arms up high to reach floating elements, standing on tiptoes, joyful posture, looking up with wonder. 4k resolution, 60fps, Disney Pixar render, joyful preschool music video style.</t>
         </is>
       </c>
+      <c r="K8" s="20" t="inlineStr">
+        <is>
+          <t>images/track_04/a1_s04_seg06_boy.jpg</t>
+        </is>
+      </c>
     </row>
     <row r="9" ht="30" customHeight="1">
       <c r="A9" s="10" t="inlineStr">
@@ -22424,6 +23474,11 @@
           <t>3D Pixar Disney style cheerful toddler dance coach, smooth playful animation, vibrant kindergarten studio, soft bright volumetric lighting, clean studio background, highly expressive face, full body dynamic camera shot: Song 'Animal Safari March', Action '第 05 節: 叢林高處真自在'. 🌴 展開雙手左右搖晃，像猴子自由快樂！. The character is waving both hands overhead in friendly wide arcs, swaying gently from side to side, sparkling excited eyes. 4k resolution, 60fps, Disney Pixar render, joyful preschool music video style.</t>
         </is>
       </c>
+      <c r="K9" s="20" t="inlineStr">
+        <is>
+          <t>images/track_04/a1_s04_seg07_boy.jpg</t>
+        </is>
+      </c>
     </row>
     <row r="10" ht="30" customHeight="1">
       <c r="A10" s="8" t="inlineStr">
@@ -22472,6 +23527,11 @@
           <t>3D Pixar Disney style cheerful toddler dance coach, smooth playful animation, vibrant kindergarten studio, soft bright volumetric lighting, clean studio background, highly expressive face, full body dynamic camera shot: Song 'Animal Safari March', Action '第 06 節: 小狗汪汪小貓喵'. 🐶 雙手放在耳邊搖搖，伸出小貓爪抓抓！. The character is stretching arms up high to reach floating elements, standing on tiptoes, joyful posture, looking up with wonder. 4k resolution, 60fps, Disney Pixar render, joyful preschool music video style.</t>
         </is>
       </c>
+      <c r="K10" s="20" t="inlineStr">
+        <is>
+          <t>images/track_04/a1_s04_seg08_boy.jpg</t>
+        </is>
+      </c>
     </row>
     <row r="11" ht="30" customHeight="1">
       <c r="A11" s="10" t="inlineStr">
@@ -22520,6 +23580,11 @@
           <t>3D Pixar Disney style cheerful toddler dance coach, smooth playful animation, vibrant kindergarten studio, soft bright volumetric lighting, clean studio background, highly expressive face, full body dynamic camera shot: Song 'Animal Safari March', Action '第 07 節: 大家一起學叫聲'. 🐾 拍拍小手，開開心心模仿動物叫！. The character is marching in place energetically, hands on hips, knees lifting high in rhythmic bounce, enthusiastic happy smile. 4k resolution, 60fps, Disney Pixar render, joyful preschool music video style.</t>
         </is>
       </c>
+      <c r="K11" s="20" t="inlineStr">
+        <is>
+          <t>images/track_04/a1_s04_seg09_boy.jpg</t>
+        </is>
+      </c>
     </row>
     <row r="12" ht="30" customHeight="1">
       <c r="A12" s="8" t="inlineStr">
@@ -22568,6 +23633,11 @@
           <t>3D Pixar Disney style cheerful toddler dance coach, smooth playful animation, vibrant kindergarten studio, soft bright volumetric lighting, clean studio background, highly expressive face, full body dynamic camera shot: Song 'Animal Safari March', Action '第 08 節: 齊步走過綠叢林'. 🌿 挺起胸膛踏步前進，穿過茂密森林！. The character is marching in place energetically, hands on hips, knees lifting high in rhythmic bounce, enthusiastic happy smile. 4k resolution, 60fps, Disney Pixar render, joyful preschool music video style.</t>
         </is>
       </c>
+      <c r="K12" s="20" t="inlineStr">
+        <is>
+          <t>images/track_04/a1_s04_seg10_boy.jpg</t>
+        </is>
+      </c>
     </row>
     <row r="13" ht="30" customHeight="1">
       <c r="A13" s="10" t="inlineStr">
@@ -22616,6 +23686,11 @@
           <t>3D Pixar Disney style cheerful toddler dance coach, smooth playful animation, vibrant kindergarten studio, soft bright volumetric lighting, clean studio background, highly expressive face, full body dynamic camera shot: Song 'Animal Safari March', Action '第 09 節: 最開心的動物群'. ⭐ 歡樂轉個圈圈，每隻動物都笑嘻嘻！. The character is swaying hips and arms like a breeze, smooth fluid body roll, playful rhythmic dancing, friendly warm smile. 4k resolution, 60fps, Disney Pixar render, joyful preschool music video style.</t>
         </is>
       </c>
+      <c r="K13" s="20" t="inlineStr">
+        <is>
+          <t>images/track_04/a1_s04_seg11_boy.jpg</t>
+        </is>
+      </c>
     </row>
     <row r="14" ht="30" customHeight="1">
       <c r="A14" s="8" t="inlineStr">
@@ -22664,6 +23739,11 @@
           <t>3D Pixar Disney style cheerful toddler dance coach, smooth playful animation, vibrant kindergarten studio, soft bright volumetric lighting, clean studio background, highly expressive face, full body dynamic camera shot: Song 'Animal Safari March', Action '第 10 節: 搖搖尾巴拍拍翅'. 🦚 雙手放背後扭動尾巴，雙臂輕拍翅膀！. The character is waving both hands overhead in friendly wide arcs, swaying gently from side to side, sparkling excited eyes. 4k resolution, 60fps, Disney Pixar render, joyful preschool music video style.</t>
         </is>
       </c>
+      <c r="K14" s="20" t="inlineStr">
+        <is>
+          <t>images/track_04/a1_s04_seg12_boy.jpg</t>
+        </is>
+      </c>
     </row>
     <row r="15" ht="30" customHeight="1">
       <c r="A15" s="10" t="inlineStr">
@@ -22712,6 +23792,11 @@
           <t>3D Pixar Disney style cheerful toddler dance coach, smooth playful animation, vibrant kindergarten studio, soft bright volumetric lighting, clean studio background, highly expressive face, full body dynamic camera shot: Song 'Animal Safari March', Action '第 11 節: 森林合唱團開唱'. 🎶 雙手像花朵盛開，全體高聲齊合唱！. The character is lifting arms from heart to sky creating a big golden sun circle, chest open, radiant beaming joyful smile. 4k resolution, 60fps, Disney Pixar render, joyful preschool music video style.</t>
         </is>
       </c>
+      <c r="K15" s="20" t="inlineStr">
+        <is>
+          <t>images/track_04/a1_s04_seg13_boy.jpg</t>
+        </is>
+      </c>
     </row>
     <row r="16" ht="30" customHeight="1">
       <c r="A16" s="8" t="inlineStr">
@@ -22760,6 +23845,11 @@
           <t>3D Pixar Disney style cheerful toddler dance coach, smooth playful animation, vibrant kindergarten studio, soft bright volumetric lighting, clean studio background, highly expressive face, full body dynamic camera shot: Song 'Animal Safari March', Action '[旋律間奏] 動作接續歡樂跳'. 🔄 雙手插腰踩小碎步，轉個歡樂大圓圈，保持微笑！. The character is swaying hips and arms like a breeze, smooth fluid body roll, playful rhythmic dancing, friendly warm smile. 4k resolution, 60fps, Disney Pixar render, joyful preschool music video style.</t>
         </is>
       </c>
+      <c r="K16" s="20" t="inlineStr">
+        <is>
+          <t>images/track_04/a1_s04_seg14_boy.jpg</t>
+        </is>
+      </c>
     </row>
     <row r="17" ht="30" customHeight="1">
       <c r="A17" s="10" t="inlineStr">
@@ -22808,6 +23898,11 @@
           <t>3D Pixar Disney style cheerful toddler dance coach, smooth playful animation, vibrant kindergarten studio, soft bright volumetric lighting, clean studio background, highly expressive face, full body dynamic camera shot: Song 'Animal Safari March', Action '第 12 節: 小兔草地蹦蹦跳'. 🐰 雙手放頭頂比兔耳，雙腳輕輕彈跳！. The character is squatting down and bursting into a high happy jump, feet kicking joyfully in mid-air, both fists punching the sky in victory. 4k resolution, 60fps, Disney Pixar render, joyful preschool music video style.</t>
         </is>
       </c>
+      <c r="K17" s="20" t="inlineStr">
+        <is>
+          <t>images/track_04/a1_s04_seg15_boy.jpg</t>
+        </is>
+      </c>
     </row>
     <row r="18" ht="30" customHeight="1">
       <c r="A18" s="8" t="inlineStr">
@@ -22856,6 +23951,11 @@
           <t>3D Pixar Disney style cheerful toddler dance coach, smooth playful animation, vibrant kindergarten studio, soft bright volumetric lighting, clean studio background, highly expressive face, full body dynamic camera shot: Song 'Animal Safari March', Action '第 13 節: 高高長頸鹿走過'. 🦒 單手高高舉過頭頂，脖子長長漫步！. The character is stretching arms up high to reach floating elements, standing on tiptoes, joyful posture, looking up with wonder. 4k resolution, 60fps, Disney Pixar render, joyful preschool music video style.</t>
         </is>
       </c>
+      <c r="K18" s="20" t="inlineStr">
+        <is>
+          <t>images/track_04/a1_s04_seg16_boy.jpg</t>
+        </is>
+      </c>
     </row>
     <row r="19" ht="30" customHeight="1">
       <c r="A19" s="10" t="inlineStr">
@@ -22904,6 +24004,11 @@
           <t>3D Pixar Disney style cheerful toddler dance coach, smooth playful animation, vibrant kindergarten studio, soft bright volumetric lighting, clean studio background, highly expressive face, full body dynamic camera shot: Song 'Animal Safari March', Action '第 14 節: 獅子大王威武吼'. 🦁 雙手張開成尖爪胸前用力一吼：Roar！. The character is squatting down and bursting into a high happy jump, feet kicking joyfully in mid-air, both fists punching the sky in victory. 4k resolution, 60fps, Disney Pixar render, joyful preschool music video style.</t>
         </is>
       </c>
+      <c r="K19" s="20" t="inlineStr">
+        <is>
+          <t>images/track_04/a1_s04_seg17_boy.jpg</t>
+        </is>
+      </c>
     </row>
     <row r="20" ht="30" customHeight="1">
       <c r="A20" s="8" t="inlineStr">
@@ -22952,6 +24057,11 @@
           <t>3D Pixar Disney style cheerful toddler dance coach, smooth playful animation, vibrant kindergarten studio, soft bright volumetric lighting, clean studio background, highly expressive face, full body dynamic camera shot: Song 'Animal Safari March', Action '第 15 節: 小企鵝搖擺招手'. 🐧 雙臂貼大腿內側，左右小碎步搖擺招手！. The character is waving both hands overhead in friendly wide arcs, swaying gently from side to side, sparkling excited eyes. 4k resolution, 60fps, Disney Pixar render, joyful preschool music video style.</t>
         </is>
       </c>
+      <c r="K20" s="20" t="inlineStr">
+        <is>
+          <t>images/track_04/a1_s04_seg18_boy.jpg</t>
+        </is>
+      </c>
     </row>
     <row r="21" ht="30" customHeight="1">
       <c r="A21" s="10" t="inlineStr">
@@ -23000,6 +24110,11 @@
           <t>3D Pixar Disney style cheerful toddler dance coach, smooth playful animation, vibrant kindergarten studio, soft bright volumetric lighting, clean studio background, highly expressive face, full body dynamic camera shot: Song 'Animal Safari March', Action '第 16 節: 小鴨嘎嘎叫不停'. 🦆 雙手在嘴前開合做鴨嘴巴：嘎嘎嘎！. The character is stretching arms up high to reach floating elements, standing on tiptoes, joyful posture, looking up with wonder. 4k resolution, 60fps, Disney Pixar render, joyful preschool music video style.</t>
         </is>
       </c>
+      <c r="K21" s="20" t="inlineStr">
+        <is>
+          <t>images/track_04/a1_s04_seg19_boy.jpg</t>
+        </is>
+      </c>
     </row>
     <row r="22" ht="30" customHeight="1">
       <c r="A22" s="8" t="inlineStr">
@@ -23048,6 +24163,11 @@
           <t>3D Pixar Disney style cheerful toddler dance coach, smooth playful animation, vibrant kindergarten studio, soft bright volumetric lighting, clean studio background, highly expressive face, full body dynamic camera shot: Song 'Animal Safari March', Action '第 17 節: 小青蛙呱呱大跳'. 🐸 蹲下雙手撐地，用力蹦起呱呱叫！. The character is squatting down and bursting into a high happy jump, feet kicking joyfully in mid-air, both fists punching the sky in victory. 4k resolution, 60fps, Disney Pixar render, joyful preschool music video style.</t>
         </is>
       </c>
+      <c r="K22" s="20" t="inlineStr">
+        <is>
+          <t>images/track_04/a1_s04_seg20_boy.jpg</t>
+        </is>
+      </c>
     </row>
     <row r="23" ht="30" customHeight="1">
       <c r="A23" s="10" t="inlineStr">
@@ -23096,6 +24216,11 @@
           <t>3D Pixar Disney style cheerful toddler dance coach, smooth playful animation, vibrant kindergarten studio, soft bright volumetric lighting, clean studio background, highly expressive face, full body dynamic camera shot: Song 'Animal Safari March', Action '第 18 節: 池塘濺起小水花'. 💦 雙腳輕輕踩踏，雙手拍水花四濺！. The character is marching in place energetically, hands on hips, knees lifting high in rhythmic bounce, enthusiastic happy smile. 4k resolution, 60fps, Disney Pixar render, joyful preschool music video style.</t>
         </is>
       </c>
+      <c r="K23" s="20" t="inlineStr">
+        <is>
+          <t>images/track_04/a1_s04_seg21_boy.jpg</t>
+        </is>
+      </c>
     </row>
     <row r="24" ht="30" customHeight="1">
       <c r="A24" s="8" t="inlineStr">
@@ -23144,6 +24269,11 @@
           <t>3D Pixar Disney style cheerful toddler dance coach, smooth playful animation, vibrant kindergarten studio, soft bright volumetric lighting, clean studio background, highly expressive face, full body dynamic camera shot: Song 'Animal Safari March', Action '第 19 節: 動物大軍向前進'. 🥁 踩著堅定有力的節拍，精神大步邁！. The character is marching in place energetically, hands on hips, knees lifting high in rhythmic bounce, enthusiastic happy smile. 4k resolution, 60fps, Disney Pixar render, joyful preschool music video style.</t>
         </is>
       </c>
+      <c r="K24" s="20" t="inlineStr">
+        <is>
+          <t>images/track_04/a1_s04_seg22_boy.jpg</t>
+        </is>
+      </c>
     </row>
     <row r="25" ht="30" customHeight="1">
       <c r="A25" s="10" t="inlineStr">
@@ -23192,6 +24322,11 @@
           <t>3D Pixar Disney style cheerful toddler dance coach, smooth playful animation, vibrant kindergarten studio, soft bright volumetric lighting, clean studio background, highly expressive face, full body dynamic camera shot: Song 'Animal Safari March', Action '第 20 節: 歡樂巡遊最精彩'. ✨ 雙手高高揮舞，全場動物熱情巡遊！. The character is lifting arms from heart to sky creating a big golden sun circle, chest open, radiant beaming joyful smile. 4k resolution, 60fps, Disney Pixar render, joyful preschool music video style.</t>
         </is>
       </c>
+      <c r="K25" s="20" t="inlineStr">
+        <is>
+          <t>images/track_04/a1_s04_seg23_boy.jpg</t>
+        </is>
+      </c>
     </row>
     <row r="26" ht="30" customHeight="1">
       <c r="A26" s="8" t="inlineStr">
@@ -23240,6 +24375,11 @@
           <t>3D Pixar Disney style cheerful toddler dance coach, smooth playful animation, vibrant kindergarten studio, soft bright volumetric lighting, clean studio background, highly expressive face, full body dynamic camera shot: Song 'Animal Safari March', Action '第 21 節: 擺尾拍翅再齊舞'. 🐾 左右快速搖擺，拍動翅膀一起跳！. The character is waving both hands overhead in friendly wide arcs, swaying gently from side to side, sparkling excited eyes. 4k resolution, 60fps, Disney Pixar render, joyful preschool music video style.</t>
         </is>
       </c>
+      <c r="K26" s="20" t="inlineStr">
+        <is>
+          <t>images/track_04/a1_s04_seg24_boy.jpg</t>
+        </is>
+      </c>
     </row>
     <row r="27" ht="30" customHeight="1">
       <c r="A27" s="10" t="inlineStr">
@@ -23288,6 +24428,11 @@
           <t>3D Pixar Disney style cheerful toddler dance coach, smooth playful animation, vibrant kindergarten studio, soft bright volumetric lighting, clean studio background, highly expressive face, full body dynamic camera shot: Song 'Animal Safari March', Action '第 22 節: 森林大合奏吼叫'. 🦁 獅子吼！鴨子叫！小貓喵！全場合奏！. The character is bringing hands together at the chest forming an adorable glowing heart shape, leaning slightly forward, loving gentle smile. 4k resolution, 60fps, Disney Pixar render, joyful preschool music video style.</t>
         </is>
       </c>
+      <c r="K27" s="20" t="inlineStr">
+        <is>
+          <t>images/track_04/a1_s04_seg25_boy.jpg</t>
+        </is>
+      </c>
     </row>
     <row r="28" ht="30" customHeight="1">
       <c r="A28" s="8" t="inlineStr">
@@ -23334,6 +24479,11 @@
       <c r="J28" s="9" t="inlineStr">
         <is>
           <t>3D Pixar Disney style cheerful toddler dance coach, smooth playful animation, vibrant kindergarten studio, soft bright volumetric lighting, clean studio background, highly expressive face, full body dynamic camera shot: Song 'Animal Safari March', Action '第 23 節: 軍鼓重響定格秀'. 🌟 雙手叉腰胸前定格，最棒動物探險家！. The character is lifting arms from heart to sky creating a big golden sun circle, chest open, radiant beaming joyful smile. 4k resolution, 60fps, Disney Pixar render, joyful preschool music video style.</t>
+        </is>
+      </c>
+      <c r="K28" s="20" t="inlineStr">
+        <is>
+          <t>images/track_04/a1_s04_seg26_boy.jpg</t>
         </is>
       </c>
     </row>
@@ -23351,7 +24501,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J28"/>
+  <dimension ref="A1:K28"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="18" customWidth="1" min="1" max="1"/>
@@ -23364,6 +24514,7 @@
     <col width="30" customWidth="1" min="8" max="8"/>
     <col width="12" customWidth="1" min="9" max="9"/>
     <col width="55" customWidth="1" min="10" max="10"/>
+    <col width="34" customWidth="1" min="11" max="11"/>
   </cols>
   <sheetData>
     <row r="1" ht="32" customHeight="1">
@@ -23424,6 +24575,11 @@
           <t>AI 影片動畫生成提示詞 (Prompt)</t>
         </is>
       </c>
+      <c r="K2" s="19" t="inlineStr">
+        <is>
+          <t>首張圖片路徑 (9:16 720p)</t>
+        </is>
+      </c>
     </row>
     <row r="3" ht="30" customHeight="1">
       <c r="A3" s="10" t="inlineStr">
@@ -23472,6 +24628,11 @@
           <t>3D Pixar Disney style preschool animation video keyframe, vertical 9:16 aspect ratio 720p HD. Full body standing shot of the cheerful 5-year-old girl dance coach with brown curly pigtails tied with yellow ribbons, pink dance tee with smiling yellow star, yellow shorts, pink sneakers. In colorful kindergarten dance studio. Starter keyframe for action "[前奏] 時鐘滴答整理預備" (⏰ 時鐘滴答走，玩具小幫手挽起袖子集合！). The character is in lively dance starter pose, joyful radiant beaming smile, sparkling expressive eyes. 4k 3D Pixar render, clean frame without text overlay, starter keyframe for image-to-video generation (a1_s05_seg01_girl.jpg).</t>
         </is>
       </c>
+      <c r="K3" s="20" t="inlineStr">
+        <is>
+          <t>images/track_05/a1_s05_seg01_girl.jpg</t>
+        </is>
+      </c>
     </row>
     <row r="4" ht="30" customHeight="1">
       <c r="A4" s="8" t="inlineStr">
@@ -23520,6 +24681,11 @@
           <t>3D Pixar Disney style cheerful toddler dance coach, smooth playful animation, vibrant kindergarten studio, soft bright volumetric lighting, clean studio background, highly expressive face, full body dynamic camera shot: Song 'Clean Up Little Helpers', Action '第 01 節: 遊戲結束時鐘響'. ⏰ 雙手叉腰身體跟著時鐘左右擺動！. The character is swaying hips and arms like a breeze, smooth fluid body roll, playful rhythmic dancing, friendly warm smile. 4k resolution, 60fps, Disney Pixar render, joyful preschool music video style.</t>
         </is>
       </c>
+      <c r="K4" s="20" t="inlineStr">
+        <is>
+          <t>images/track_05/a1_s05_seg02_girl.jpg</t>
+        </is>
+      </c>
     </row>
     <row r="5" ht="30" customHeight="1">
       <c r="A5" s="10" t="inlineStr">
@@ -23568,6 +24734,11 @@
           <t>3D Pixar Disney style cheerful toddler dance coach, smooth playful animation, vibrant kindergarten studio, soft bright volumetric lighting, clean studio background, highly expressive face, full body dynamic camera shot: Song 'Clean Up Little Helpers', Action '第 02 節: 收拾積木排排隊'. 🧱 彎下腰撿起積木，輕輕放進收納籃！. The character is stretching arms up high to reach floating elements, standing on tiptoes, joyful posture, looking up with wonder. 4k resolution, 60fps, Disney Pixar render, joyful preschool music video style.</t>
         </is>
       </c>
+      <c r="K5" s="20" t="inlineStr">
+        <is>
+          <t>images/track_05/a1_s05_seg03_girl.jpg</t>
+        </is>
+      </c>
     </row>
     <row r="6" ht="30" customHeight="1">
       <c r="A6" s="8" t="inlineStr">
@@ -23616,6 +24787,11 @@
           <t>3D Pixar Disney style cheerful toddler dance coach, smooth playful animation, vibrant kindergarten studio, soft bright volumetric lighting, clean studio background, highly expressive face, full body dynamic camera shot: Song 'Clean Up Little Helpers', Action '第 03 節: 鉛筆蠟筆回小盒'. ✏️ 雙手捧著筆筒，把彩色蠟筆放進盒子！. The character is marching in place energetically, hands on hips, knees lifting high in rhythmic bounce, enthusiastic happy smile. 4k resolution, 60fps, Disney Pixar render, joyful preschool music video style.</t>
         </is>
       </c>
+      <c r="K6" s="20" t="inlineStr">
+        <is>
+          <t>images/track_05/a1_s05_seg04_girl.jpg</t>
+        </is>
+      </c>
     </row>
     <row r="7" ht="30" customHeight="1">
       <c r="A7" s="10" t="inlineStr">
@@ -23664,6 +24840,11 @@
           <t>3D Pixar Disney style cheerful toddler dance coach, smooth playful animation, vibrant kindergarten studio, soft bright volumetric lighting, clean studio background, highly expressive face, full body dynamic camera shot: Song 'Clean Up Little Helpers', Action '第 04 節: 幫小熊襪子配對'. 🧸 雙手拍拍小腳踝，幫小熊摺好小襪子！. The character is stretching arms up high to reach floating elements, standing on tiptoes, joyful posture, looking up with wonder. 4k resolution, 60fps, Disney Pixar render, joyful preschool music video style.</t>
         </is>
       </c>
+      <c r="K7" s="20" t="inlineStr">
+        <is>
+          <t>images/track_05/a1_s05_seg05_girl.jpg</t>
+        </is>
+      </c>
     </row>
     <row r="8" ht="30" customHeight="1">
       <c r="A8" s="8" t="inlineStr">
@@ -23712,6 +24893,11 @@
           <t>3D Pixar Disney style cheerful toddler dance coach, smooth playful animation, vibrant kindergarten studio, soft bright volumetric lighting, clean studio background, highly expressive face, full body dynamic camera shot: Song 'Clean Up Little Helpers', Action '第 05 節: 看看桌子看看毯'. 👀 彎腰轉頭找一找，桌面地毯都乾淨！. The character is swaying hips and arms like a breeze, smooth fluid body roll, playful rhythmic dancing, friendly warm smile. 4k resolution, 60fps, Disney Pixar render, joyful preschool music video style.</t>
         </is>
       </c>
+      <c r="K8" s="20" t="inlineStr">
+        <is>
+          <t>images/track_05/a1_s05_seg06_girl.jpg</t>
+        </is>
+      </c>
     </row>
     <row r="9" ht="30" customHeight="1">
       <c r="A9" s="10" t="inlineStr">
@@ -23760,6 +24946,11 @@
           <t>3D Pixar Disney style cheerful toddler dance coach, smooth playful animation, vibrant kindergarten studio, soft bright volumetric lighting, clean studio background, highly expressive face, full body dynamic camera shot: Song 'Clean Up Little Helpers', Action '第 06 節: 給房間一個大擁抱'. 💖 雙臂張開大大環抱，給房間滿滿愛！. The character is bringing hands together at the chest forming an adorable glowing heart shape, leaning slightly forward, loving gentle smile. 4k resolution, 60fps, Disney Pixar render, joyful preschool music video style.</t>
         </is>
       </c>
+      <c r="K9" s="20" t="inlineStr">
+        <is>
+          <t>images/track_05/a1_s05_seg07_girl.jpg</t>
+        </is>
+      </c>
     </row>
     <row r="10" ht="30" customHeight="1">
       <c r="A10" s="8" t="inlineStr">
@@ -23808,6 +24999,11 @@
           <t>3D Pixar Disney style cheerful toddler dance coach, smooth playful animation, vibrant kindergarten studio, soft bright volumetric lighting, clean studio background, highly expressive face, full body dynamic camera shot: Song 'Clean Up Little Helpers', Action '第 07 節: 動作快快收乾淨'. ⚡ 腳步輕快小碎步，快快收拾小房間！. The character is marching in place energetically, hands on hips, knees lifting high in rhythmic bounce, enthusiastic happy smile. 4k resolution, 60fps, Disney Pixar render, joyful preschool music video style.</t>
         </is>
       </c>
+      <c r="K10" s="20" t="inlineStr">
+        <is>
+          <t>images/track_05/a1_s05_seg08_girl.jpg</t>
+        </is>
+      </c>
     </row>
     <row r="11" ht="30" customHeight="1">
       <c r="A11" s="10" t="inlineStr">
@@ -23856,6 +25052,11 @@
           <t>3D Pixar Disney style cheerful toddler dance coach, smooth playful animation, vibrant kindergarten studio, soft bright volumetric lighting, clean studio background, highly expressive face, full body dynamic camera shot: Song 'Clean Up Little Helpers', Action '第 08 節: 人人幫忙好計畫'. 🤝 拍拍雙手豎起大拇指，大家都是小幫手！. The character is waving both hands overhead in friendly wide arcs, swaying gently from side to side, sparkling excited eyes. 4k resolution, 60fps, Disney Pixar render, joyful preschool music video style.</t>
         </is>
       </c>
+      <c r="K11" s="20" t="inlineStr">
+        <is>
+          <t>images/track_05/a1_s05_seg09_girl.jpg</t>
+        </is>
+      </c>
     </row>
     <row r="12" ht="30" customHeight="1">
       <c r="A12" s="8" t="inlineStr">
@@ -23904,6 +25105,11 @@
           <t>3D Pixar Disney style cheerful toddler dance coach, smooth playful animation, vibrant kindergarten studio, soft bright volumetric lighting, clean studio background, highly expressive face, full body dynamic camera shot: Song 'Clean Up Little Helpers', Action '第 09 節: 物歸原位放整齊'. 📦 雙手由低到高把物品整齊歸位！. The character is stretching arms up high to reach floating elements, standing on tiptoes, joyful posture, looking up with wonder. 4k resolution, 60fps, Disney Pixar render, joyful preschool music video style.</t>
         </is>
       </c>
+      <c r="K12" s="20" t="inlineStr">
+        <is>
+          <t>images/track_05/a1_s05_seg10_girl.jpg</t>
+        </is>
+      </c>
     </row>
     <row r="13" ht="30" customHeight="1">
       <c r="A13" s="10" t="inlineStr">
@@ -23952,6 +25158,11 @@
           <t>3D Pixar Disney style cheerful toddler dance coach, smooth playful animation, vibrant kindergarten studio, soft bright volumetric lighting, clean studio background, highly expressive face, full body dynamic camera shot: Song 'Clean Up Little Helpers', Action '第 10 節: 迎接快樂新一天'. ☀️ 雙手高舉托起朝陽，迎接全新明天！. The character is lifting arms from heart to sky creating a big golden sun circle, chest open, radiant beaming joyful smile. 4k resolution, 60fps, Disney Pixar render, joyful preschool music video style.</t>
         </is>
       </c>
+      <c r="K13" s="20" t="inlineStr">
+        <is>
+          <t>images/track_05/a1_s05_seg11_girl.jpg</t>
+        </is>
+      </c>
     </row>
     <row r="14" ht="30" customHeight="1">
       <c r="A14" s="8" t="inlineStr">
@@ -24000,6 +25211,11 @@
           <t>3D Pixar Disney style cheerful toddler dance coach, smooth playful animation, vibrant kindergarten studio, soft bright volumetric lighting, clean studio background, highly expressive face, full body dynamic camera shot: Song 'Clean Up Little Helpers', Action '[旋律間奏] 動作接續歡樂跳'. 🔄 雙手插腰踩小碎步，轉個歡樂大圓圈，保持微笑！. The character is swaying hips and arms like a breeze, smooth fluid body roll, playful rhythmic dancing, friendly warm smile. 4k resolution, 60fps, Disney Pixar render, joyful preschool music video style.</t>
         </is>
       </c>
+      <c r="K14" s="20" t="inlineStr">
+        <is>
+          <t>images/track_05/a1_s05_seg12_girl.jpg</t>
+        </is>
+      </c>
     </row>
     <row r="15" ht="30" customHeight="1">
       <c r="A15" s="10" t="inlineStr">
@@ -24048,6 +25264,11 @@
           <t>3D Pixar Disney style cheerful toddler dance coach, smooth playful animation, vibrant kindergarten studio, soft bright volumetric lighting, clean studio background, highly expressive face, full body dynamic camera shot: Song 'Clean Up Little Helpers', Action '第 11 節: 圖書立在書架上'. 📚 雙手合十像小書本，整齊排排站好！. The character is marching in place energetically, hands on hips, knees lifting high in rhythmic bounce, enthusiastic happy smile. 4k resolution, 60fps, Disney Pixar render, joyful preschool music video style.</t>
         </is>
       </c>
+      <c r="K15" s="20" t="inlineStr">
+        <is>
+          <t>images/track_05/a1_s05_seg13_girl.jpg</t>
+        </is>
+      </c>
     </row>
     <row r="16" ht="30" customHeight="1">
       <c r="A16" s="8" t="inlineStr">
@@ -24096,6 +25317,11 @@
           <t>3D Pixar Disney style cheerful toddler dance coach, smooth playful animation, vibrant kindergarten studio, soft bright volumetric lighting, clean studio background, highly expressive face, full body dynamic camera shot: Song 'Clean Up Little Helpers', Action '第 12 節: 玩具小車回小籃'. 🚗 雙手握方向盤轉轉，開進玩具籃！. The character is swaying hips and arms like a breeze, smooth fluid body roll, playful rhythmic dancing, friendly warm smile. 4k resolution, 60fps, Disney Pixar render, joyful preschool music video style.</t>
         </is>
       </c>
+      <c r="K16" s="20" t="inlineStr">
+        <is>
+          <t>images/track_05/a1_s05_seg14_girl.jpg</t>
+        </is>
+      </c>
     </row>
     <row r="17" ht="30" customHeight="1">
       <c r="A17" s="10" t="inlineStr">
@@ -24144,6 +25370,11 @@
           <t>3D Pixar Disney style cheerful toddler dance coach, smooth playful animation, vibrant kindergarten studio, soft bright volumetric lighting, clean studio background, highly expressive face, full body dynamic camera shot: Song 'Clean Up Little Helpers', Action '第 13 節: 一二三樣樣乾淨'. ✨ 數數一二三，房間變得整整齊齊！. The character is stretching arms up high to reach floating elements, standing on tiptoes, joyful posture, looking up with wonder. 4k resolution, 60fps, Disney Pixar render, joyful preschool music video style.</t>
         </is>
       </c>
+      <c r="K17" s="20" t="inlineStr">
+        <is>
+          <t>images/track_05/a1_s05_seg15_girl.jpg</t>
+        </is>
+      </c>
     </row>
     <row r="18" ht="30" customHeight="1">
       <c r="A18" s="8" t="inlineStr">
@@ -24192,6 +25423,11 @@
           <t>3D Pixar Disney style cheerful toddler dance coach, smooth playful animation, vibrant kindergarten studio, soft bright volumetric lighting, clean studio background, highly expressive face, full body dynamic camera shot: Song 'Clean Up Little Helpers', Action '第 14 節: 擊掌好朋友拍個手'. ✋ 伸出雙手向同伴高高擊掌：High-Five！. The character is waving both hands overhead in friendly wide arcs, swaying gently from side to side, sparkling excited eyes. 4k resolution, 60fps, Disney Pixar render, joyful preschool music video style.</t>
         </is>
       </c>
+      <c r="K18" s="20" t="inlineStr">
+        <is>
+          <t>images/track_05/a1_s05_seg16_girl.jpg</t>
+        </is>
+      </c>
     </row>
     <row r="19" ht="30" customHeight="1">
       <c r="A19" s="10" t="inlineStr">
@@ -24240,6 +25476,11 @@
           <t>3D Pixar Disney style cheerful toddler dance coach, smooth playful animation, vibrant kindergarten studio, soft bright volumetric lighting, clean studio background, highly expressive face, full body dynamic camera shot: Song 'Clean Up Little Helpers', Action '第 15 節: 整齊任務大成功'. 🎉 歡快原地小跳步，任務順利通關！. The character is squatting down and bursting into a high happy jump, feet kicking joyfully in mid-air, both fists punching the sky in victory. 4k resolution, 60fps, Disney Pixar render, joyful preschool music video style.</t>
         </is>
       </c>
+      <c r="K19" s="20" t="inlineStr">
+        <is>
+          <t>images/track_05/a1_s05_seg17_girl.jpg</t>
+        </is>
+      </c>
     </row>
     <row r="20" ht="30" customHeight="1">
       <c r="A20" s="8" t="inlineStr">
@@ -24288,6 +25529,11 @@
           <t>3D Pixar Disney style cheerful toddler dance coach, smooth playful animation, vibrant kindergarten studio, soft bright volumetric lighting, clean studio background, highly expressive face, full body dynamic camera shot: Song 'Clean Up Little Helpers', Action '第 16 節: 收拾乾淨速度快'. ⚡ 雙手左右揮舞，保持乾淨不落後！. The character is marching in place energetically, hands on hips, knees lifting high in rhythmic bounce, enthusiastic happy smile. 4k resolution, 60fps, Disney Pixar render, joyful preschool music video style.</t>
         </is>
       </c>
+      <c r="K20" s="20" t="inlineStr">
+        <is>
+          <t>images/track_05/a1_s05_seg18_girl.jpg</t>
+        </is>
+      </c>
     </row>
     <row r="21" ht="30" customHeight="1">
       <c r="A21" s="10" t="inlineStr">
@@ -24336,6 +25582,11 @@
           <t>3D Pixar Disney style cheerful toddler dance coach, smooth playful animation, vibrant kindergarten studio, soft bright volumetric lighting, clean studio background, highly expressive face, full body dynamic camera shot: Song 'Clean Up Little Helpers', Action '第 17 節: 大家團結力量大'. 🤝 握緊小拳頭胸前一拉，團結第一名！. The character is bringing hands together at the chest forming an adorable glowing heart shape, leaning slightly forward, loving gentle smile. 4k resolution, 60fps, Disney Pixar render, joyful preschool music video style.</t>
         </is>
       </c>
+      <c r="K21" s="20" t="inlineStr">
+        <is>
+          <t>images/track_05/a1_s05_seg19_girl.jpg</t>
+        </is>
+      </c>
     </row>
     <row r="22" ht="30" customHeight="1">
       <c r="A22" s="8" t="inlineStr">
@@ -24384,6 +25635,11 @@
           <t>3D Pixar Disney style cheerful toddler dance coach, smooth playful animation, vibrant kindergarten studio, soft bright volumetric lighting, clean studio background, highly expressive face, full body dynamic camera shot: Song 'Clean Up Little Helpers', Action '第 18 節: 撿起放好不亂丟'. 📦 彎腰再放好，地板乾乾淨淨！. The character is stretching arms up high to reach floating elements, standing on tiptoes, joyful posture, looking up with wonder. 4k resolution, 60fps, Disney Pixar render, joyful preschool music video style.</t>
         </is>
       </c>
+      <c r="K22" s="20" t="inlineStr">
+        <is>
+          <t>images/track_05/a1_s05_seg20_girl.jpg</t>
+        </is>
+      </c>
     </row>
     <row r="23" ht="30" customHeight="1">
       <c r="A23" s="10" t="inlineStr">
@@ -24432,6 +25688,11 @@
           <t>3D Pixar Disney style cheerful toddler dance coach, smooth playful animation, vibrant kindergarten studio, soft bright volumetric lighting, clean studio background, highly expressive face, full body dynamic camera shot: Song 'Clean Up Little Helpers', Action '第 19 節: 天天都是開心天'. 🌟 雙手比出大愛心，每天都開心！. The character is bringing hands together at the chest forming an adorable glowing heart shape, leaning slightly forward, loving gentle smile. 4k resolution, 60fps, Disney Pixar render, joyful preschool music video style.</t>
         </is>
       </c>
+      <c r="K23" s="20" t="inlineStr">
+        <is>
+          <t>images/track_05/a1_s05_seg21_girl.jpg</t>
+        </is>
+      </c>
     </row>
     <row r="24" ht="30" customHeight="1">
       <c r="A24" s="8" t="inlineStr">
@@ -24480,6 +25741,11 @@
           <t>3D Pixar Disney style cheerful toddler dance coach, smooth playful animation, vibrant kindergarten studio, soft bright volumetric lighting, clean studio background, highly expressive face, full body dynamic camera shot: Song 'Clean Up Little Helpers', Action '[旋律間奏] 動作接續歡樂跳'. 🔄 雙手插腰踩小碎步，轉個歡樂大圓圈，保持微笑！. The character is swaying hips and arms like a breeze, smooth fluid body roll, playful rhythmic dancing, friendly warm smile. 4k resolution, 60fps, Disney Pixar render, joyful preschool music video style.</t>
         </is>
       </c>
+      <c r="K24" s="20" t="inlineStr">
+        <is>
+          <t>images/track_05/a1_s05_seg22_girl.jpg</t>
+        </is>
+      </c>
     </row>
     <row r="25" ht="30" customHeight="1">
       <c r="A25" s="10" t="inlineStr">
@@ -24528,6 +25794,11 @@
           <t>3D Pixar Disney style cheerful toddler dance coach, smooth playful animation, vibrant kindergarten studio, soft bright volumetric lighting, clean studio background, highly expressive face, full body dynamic camera shot: Song 'Clean Up Little Helpers', Action '第 20 節: 超級幫手大明星'. ⭐ 雙手高高舉起，我們是家務大明星！. The character is lifting arms from heart to sky creating a big golden sun circle, chest open, radiant beaming joyful smile. 4k resolution, 60fps, Disney Pixar render, joyful preschool music video style.</t>
         </is>
       </c>
+      <c r="K25" s="20" t="inlineStr">
+        <is>
+          <t>images/track_05/a1_s05_seg23_girl.jpg</t>
+        </is>
+      </c>
     </row>
     <row r="26" ht="30" customHeight="1">
       <c r="A26" s="8" t="inlineStr">
@@ -24576,6 +25847,11 @@
           <t>3D Pixar Disney style cheerful toddler dance coach, smooth playful animation, vibrant kindergarten studio, soft bright volumetric lighting, clean studio background, highly expressive face, full body dynamic camera shot: Song 'Clean Up Little Helpers', Action '第 22 節: 歡呼 Oh Oh 再跳躍'. 🎶 再喊一聲 Oh Oh，拍拍小手！. The character is squatting down and bursting into a high happy jump, feet kicking joyfully in mid-air, both fists punching the sky in victory. 4k resolution, 60fps, Disney Pixar render, joyful preschool music video style.</t>
         </is>
       </c>
+      <c r="K26" s="20" t="inlineStr">
+        <is>
+          <t>images/track_05/a1_s05_seg24_girl.jpg</t>
+        </is>
+      </c>
     </row>
     <row r="27" ht="30" customHeight="1">
       <c r="A27" s="10" t="inlineStr">
@@ -24624,6 +25900,11 @@
           <t>3D Pixar Disney style cheerful toddler dance coach, smooth playful animation, vibrant kindergarten studio, soft bright volumetric lighting, clean studio background, highly expressive face, full body dynamic camera shot: Song 'Clean Up Little Helpers', Action '第 23 節: 歡呼 Oh Oh 燦爛定格'. 🌟 雙手叉腰豎大拇指，完美定格大笑容！. The character is lifting arms from heart to sky creating a big golden sun circle, chest open, radiant beaming joyful smile. 4k resolution, 60fps, Disney Pixar render, joyful preschool music video style.</t>
         </is>
       </c>
+      <c r="K27" s="20" t="inlineStr">
+        <is>
+          <t>images/track_05/a1_s05_seg25_girl.jpg</t>
+        </is>
+      </c>
     </row>
     <row r="28" ht="30" customHeight="1">
       <c r="A28" s="8" t="inlineStr">
@@ -24670,6 +25951,11 @@
       <c r="J28" s="9" t="inlineStr">
         <is>
           <t>3D Pixar Disney style cheerful toddler dance coach, smooth playful animation, vibrant kindergarten studio, soft bright volumetric lighting, clean studio background, highly expressive face, full body dynamic camera shot: Song 'Clean Up Little Helpers', Action '第 24 節: 歡呼 Oh Oh 燦爛定格'. 🌟 雙手叉腰豎大拇指，完美定格大笑容！. The character is lifting arms from heart to sky creating a big golden sun circle, chest open, radiant beaming joyful smile. 4k resolution, 60fps, Disney Pixar render, joyful preschool music video style.</t>
+        </is>
+      </c>
+      <c r="K28" s="20" t="inlineStr">
+        <is>
+          <t>images/track_05/a1_s05_seg26_girl.jpg</t>
         </is>
       </c>
     </row>
@@ -24687,7 +25973,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J30"/>
+  <dimension ref="A1:K30"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="18" customWidth="1" min="1" max="1"/>
@@ -24700,6 +25986,7 @@
     <col width="30" customWidth="1" min="8" max="8"/>
     <col width="12" customWidth="1" min="9" max="9"/>
     <col width="55" customWidth="1" min="10" max="10"/>
+    <col width="34" customWidth="1" min="11" max="11"/>
   </cols>
   <sheetData>
     <row r="1" ht="32" customHeight="1">
@@ -24760,6 +26047,11 @@
           <t>AI 影片動畫生成提示詞 (Prompt)</t>
         </is>
       </c>
+      <c r="K2" s="19" t="inlineStr">
+        <is>
+          <t>首張圖片路徑 (9:16 720p)</t>
+        </is>
+      </c>
     </row>
     <row r="3" ht="30" customHeight="1">
       <c r="A3" s="10" t="inlineStr">
@@ -24808,6 +26100,11 @@
           <t>3D Pixar Disney style preschool animation video keyframe, vertical 9:16 aspect ratio 720p HD. Full body standing shot of the cheerful 5-year-old boy dance coach in bright blue athletic t-shirt with orange center and KIDS DANCE logo, blue shorts, orange running sneakers. In colorful kindergarten dance studio. Starter keyframe for action "[前奏] 宇宙電波呼叫訊號" (📡 嗶嗶嗶！戴上太空頭盔，發射台準備完畢！). The character is in lively dance starter pose, joyful radiant beaming smile, sparkling expressive eyes. 4k 3D Pixar render, clean frame without text overlay, starter keyframe for image-to-video generation (a1_s06_seg01_boy.jpg).</t>
         </is>
       </c>
+      <c r="K3" s="20" t="inlineStr">
+        <is>
+          <t>images/track_06/a1_s06_seg01_boy.jpg</t>
+        </is>
+      </c>
     </row>
     <row r="4" ht="30" customHeight="1">
       <c r="A4" s="8" t="inlineStr">
@@ -24856,6 +26153,11 @@
           <t>3D Pixar Disney style cheerful toddler dance coach, smooth playful animation, vibrant kindergarten studio, soft bright volumetric lighting, clean studio background, highly expressive face, full body dynamic camera shot: Song 'Space Rocket Countdown', Action '第 01 節: 宇宙電波嗶嗶響'. 🛸 小手放耳邊，接收太空站訊號！. The character is stretching arms up high to reach floating elements, standing on tiptoes, joyful posture, looking up with wonder. 4k resolution, 60fps, Disney Pixar render, joyful preschool music video style.</t>
         </is>
       </c>
+      <c r="K4" s="20" t="inlineStr">
+        <is>
+          <t>images/track_06/a1_s06_seg02_boy.jpg</t>
+        </is>
+      </c>
     </row>
     <row r="5" ht="30" customHeight="1">
       <c r="A5" s="10" t="inlineStr">
@@ -24904,6 +26206,11 @@
           <t>3D Pixar Disney style cheerful toddler dance coach, smooth playful animation, vibrant kindergarten studio, soft bright volumetric lighting, clean studio background, highly expressive face, full body dynamic camera shot: Song 'Space Rocket Countdown', Action '第 02 節: 太空任務準備好'. 👨‍🚀 雙手叉腰立正站好，準備起飛！. The character is marching in place energetically, hands on hips, knees lifting high in rhythmic bounce, enthusiastic happy smile. 4k resolution, 60fps, Disney Pixar render, joyful preschool music video style.</t>
         </is>
       </c>
+      <c r="K5" s="20" t="inlineStr">
+        <is>
+          <t>images/track_06/a1_s06_seg03_boy.jpg</t>
+        </is>
+      </c>
     </row>
     <row r="6" ht="30" customHeight="1">
       <c r="A6" s="8" t="inlineStr">
@@ -24952,6 +26259,11 @@
           <t>3D Pixar Disney style cheerful toddler dance coach, smooth playful animation, vibrant kindergarten studio, soft bright volumetric lighting, clean studio background, highly expressive face, full body dynamic camera shot: Song 'Space Rocket Countdown', Action '第 03 節: 五四三二一倒數'. 🚀 雙膝微蹲蓄力，跟著大聲倒數：5 4 3 2 1！. The character is marching in place energetically, hands on hips, knees lifting high in rhythmic bounce, enthusiastic happy smile. 4k resolution, 60fps, Disney Pixar render, joyful preschool music video style.</t>
         </is>
       </c>
+      <c r="K6" s="20" t="inlineStr">
+        <is>
+          <t>images/track_06/a1_s06_seg04_boy.jpg</t>
+        </is>
+      </c>
     </row>
     <row r="7" ht="30" customHeight="1">
       <c r="A7" s="10" t="inlineStr">
@@ -25000,6 +26312,11 @@
           <t>3D Pixar Disney style cheerful toddler dance coach, smooth playful animation, vibrant kindergarten studio, soft bright volumetric lighting, clean studio background, highly expressive face, full body dynamic camera shot: Song 'Space Rocket Countdown', Action '第 04 節: 穿好太空服太空靴'. 👢 摸摸雙腿穿上太空靴，拉緊拉鍊！. The character is stretching arms up high to reach floating elements, standing on tiptoes, joyful posture, looking up with wonder. 4k resolution, 60fps, Disney Pixar render, joyful preschool music video style.</t>
         </is>
       </c>
+      <c r="K7" s="20" t="inlineStr">
+        <is>
+          <t>images/track_06/a1_s06_seg05_boy.jpg</t>
+        </is>
+      </c>
     </row>
     <row r="8" ht="30" customHeight="1">
       <c r="A8" s="8" t="inlineStr">
@@ -25048,6 +26365,11 @@
           <t>3D Pixar Disney style cheerful toddler dance coach, smooth playful animation, vibrant kindergarten studio, soft bright volumetric lighting, clean studio background, highly expressive face, full body dynamic camera shot: Song 'Space Rocket Countdown', Action '第 05 節: 扣緊銀色安全帶'. 💺 雙手交叉胸前扣緊安全帶，穩穩坐好！. The character is bringing hands together at the chest forming an adorable glowing heart shape, leaning slightly forward, loving gentle smile. 4k resolution, 60fps, Disney Pixar render, joyful preschool music video style.</t>
         </is>
       </c>
+      <c r="K8" s="20" t="inlineStr">
+        <is>
+          <t>images/track_06/a1_s06_seg06_boy.jpg</t>
+        </is>
+      </c>
     </row>
     <row r="9" ht="30" customHeight="1">
       <c r="A9" s="10" t="inlineStr">
@@ -25096,6 +26418,11 @@
           <t>3D Pixar Disney style cheerful toddler dance coach, smooth playful animation, vibrant kindergarten studio, soft bright volumetric lighting, clean studio background, highly expressive face, full body dynamic camera shot: Song 'Space Rocket Countdown', Action '第 06 節: 檢查紅綠儀表板'. 🎛️ 手指在前方點擊紅燈與綠燈按鈕！. The character is waving both hands overhead in friendly wide arcs, swaying gently from side to side, sparkling excited eyes. 4k resolution, 60fps, Disney Pixar render, joyful preschool music video style.</t>
         </is>
       </c>
+      <c r="K9" s="20" t="inlineStr">
+        <is>
+          <t>images/track_06/a1_s06_seg07_boy.jpg</t>
+        </is>
+      </c>
     </row>
     <row r="10" ht="30" customHeight="1">
       <c r="A10" s="8" t="inlineStr">
@@ -25144,6 +26471,11 @@
           <t>3D Pixar Disney style cheerful toddler dance coach, smooth playful animation, vibrant kindergarten studio, soft bright volumetric lighting, clean studio background, highly expressive face, full body dynamic camera shot: Song 'Space Rocket Countdown', Action '第 07 節: 最酷銀河太空船'. ✨ 雙臂張開像銀色機翼，左右平穩滑動！. The character is swaying hips and arms like a breeze, smooth fluid body roll, playful rhythmic dancing, friendly warm smile. 4k resolution, 60fps, Disney Pixar render, joyful preschool music video style.</t>
         </is>
       </c>
+      <c r="K10" s="20" t="inlineStr">
+        <is>
+          <t>images/track_06/a1_s06_seg08_boy.jpg</t>
+        </is>
+      </c>
     </row>
     <row r="11" ht="30" customHeight="1">
       <c r="A11" s="10" t="inlineStr">
@@ -25192,6 +26524,11 @@
           <t>3D Pixar Disney style cheerful toddler dance coach, smooth playful animation, vibrant kindergarten studio, soft bright volumetric lighting, clean studio background, highly expressive face, full body dynamic camera shot: Song 'Space Rocket Countdown', Action '第 08 節: 引擎轟鳴準備點火'. 🔥 雙手握拳身旁蓄力震動，引擎啟動！. The character is marching in place energetically, hands on hips, knees lifting high in rhythmic bounce, enthusiastic happy smile. 4k resolution, 60fps, Disney Pixar render, joyful preschool music video style.</t>
         </is>
       </c>
+      <c r="K11" s="20" t="inlineStr">
+        <is>
+          <t>images/track_06/a1_s06_seg09_boy.jpg</t>
+        </is>
+      </c>
     </row>
     <row r="12" ht="30" customHeight="1">
       <c r="A12" s="8" t="inlineStr">
@@ -25240,6 +26577,11 @@
           <t>3D Pixar Disney style cheerful toddler dance coach, smooth playful animation, vibrant kindergarten studio, soft bright volumetric lighting, clean studio background, highly expressive face, full body dynamic camera shot: Song 'Space Rocket Countdown', Action '第 09 節: 衝入燦爛星空中'. ⭐ 雙手向上發射，直衝燦爛星空！. The character is lifting arms from heart to sky creating a big golden sun circle, chest open, radiant beaming joyful smile. 4k resolution, 60fps, Disney Pixar render, joyful preschool music video style.</t>
         </is>
       </c>
+      <c r="K12" s="20" t="inlineStr">
+        <is>
+          <t>images/track_06/a1_s06_seg10_boy.jpg</t>
+        </is>
+      </c>
     </row>
     <row r="13" ht="30" customHeight="1">
       <c r="A13" s="10" t="inlineStr">
@@ -25288,6 +26630,11 @@
           <t>3D Pixar Disney style cheerful toddler dance coach, smooth playful animation, vibrant kindergarten studio, soft bright volumetric lighting, clean studio background, highly expressive face, full body dynamic camera shot: Song 'Space Rocket Countdown', Action '第 10 節: 咻咻咻急速出發'. 🚀 雙手在頭頂合攏成火箭尖，用力高跳！. The character is squatting down and bursting into a high happy jump, feet kicking joyfully in mid-air, both fists punching the sky in victory. 4k resolution, 60fps, Disney Pixar render, joyful preschool music video style.</t>
         </is>
       </c>
+      <c r="K13" s="20" t="inlineStr">
+        <is>
+          <t>images/track_06/a1_s06_seg11_boy.jpg</t>
+        </is>
+      </c>
     </row>
     <row r="14" ht="30" customHeight="1">
       <c r="A14" s="8" t="inlineStr">
@@ -25336,6 +26683,11 @@
           <t>3D Pixar Disney style cheerful toddler dance coach, smooth playful animation, vibrant kindergarten studio, soft bright volumetric lighting, clean studio background, highly expressive face, full body dynamic camera shot: Song 'Space Rocket Countdown', Action '第 11 節: 閃耀神秘宇宙光'. 🌌 雙手在身側輕輕波浪搖動，沐浴星光！. The character is swaying hips and arms like a breeze, smooth fluid body roll, playful rhythmic dancing, friendly warm smile. 4k resolution, 60fps, Disney Pixar render, joyful preschool music video style.</t>
         </is>
       </c>
+      <c r="K14" s="20" t="inlineStr">
+        <is>
+          <t>images/track_06/a1_s06_seg12_boy.jpg</t>
+        </is>
+      </c>
     </row>
     <row r="15" ht="30" customHeight="1">
       <c r="A15" s="10" t="inlineStr">
@@ -25384,6 +26736,11 @@
           <t>3D Pixar Disney style cheerful toddler dance coach, smooth playful animation, vibrant kindergarten studio, soft bright volumetric lighting, clean studio background, highly expressive face, full body dynamic camera shot: Song 'Space Rocket Countdown', Action '第 12 節: 飛越月球比天高'. 🌙 腳尖點地伸手飛越圓圓大月亮！. The character is stretching arms up high to reach floating elements, standing on tiptoes, joyful posture, looking up with wonder. 4k resolution, 60fps, Disney Pixar render, joyful preschool music video style.</t>
         </is>
       </c>
+      <c r="K15" s="20" t="inlineStr">
+        <is>
+          <t>images/track_06/a1_s06_seg13_boy.jpg</t>
+        </is>
+      </c>
     </row>
     <row r="16" ht="30" customHeight="1">
       <c r="A16" s="8" t="inlineStr">
@@ -25432,6 +26789,11 @@
           <t>3D Pixar Disney style cheerful toddler dance coach, smooth playful animation, vibrant kindergarten studio, soft bright volumetric lighting, clean studio background, highly expressive face, full body dynamic camera shot: Song 'Space Rocket Countdown', Action '第 13 節: 銀色小火箭穿黑夜'. 🚀 身體前傾平穩飛行，穿越黑夜！. The character is waving both hands overhead in friendly wide arcs, swaying gently from side to side, sparkling excited eyes. 4k resolution, 60fps, Disney Pixar render, joyful preschool music video style.</t>
         </is>
       </c>
+      <c r="K16" s="20" t="inlineStr">
+        <is>
+          <t>images/track_06/a1_s06_seg14_boy.jpg</t>
+        </is>
+      </c>
     </row>
     <row r="17" ht="30" customHeight="1">
       <c r="A17" s="10" t="inlineStr">
@@ -25480,6 +26842,11 @@
           <t>3D Pixar Disney style cheerful toddler dance coach, smooth playful animation, vibrant kindergarten studio, soft bright volumetric lighting, clean studio background, highly expressive face, full body dynamic camera shot: Song 'Space Rocket Countdown', Action '[旋律間奏] 動作接續歡樂跳'. 🔄 雙手插腰踩小碎步，轉個歡樂大圓圈，保持微笑！. The character is swaying hips and arms like a breeze, smooth fluid body roll, playful rhythmic dancing, friendly warm smile. 4k resolution, 60fps, Disney Pixar render, joyful preschool music video style.</t>
         </is>
       </c>
+      <c r="K17" s="20" t="inlineStr">
+        <is>
+          <t>images/track_06/a1_s06_seg15_boy.jpg</t>
+        </is>
+      </c>
     </row>
     <row r="18" ht="30" customHeight="1">
       <c r="A18" s="8" t="inlineStr">
@@ -25528,6 +26895,11 @@
           <t>3D Pixar Disney style cheerful toddler dance coach, smooth playful animation, vibrant kindergarten studio, soft bright volumetric lighting, clean studio background, highly expressive face, full body dynamic camera shot: Song 'Space Rocket Countdown', Action '第 14 節: 看火星緩緩轉動'. 🪐 雙臂在身前畫出旋轉的火星大球！. The character is lifting arms from heart to sky creating a big golden sun circle, chest open, radiant beaming joyful smile. 4k resolution, 60fps, Disney Pixar render, joyful preschool music video style.</t>
         </is>
       </c>
+      <c r="K18" s="20" t="inlineStr">
+        <is>
+          <t>images/track_06/a1_s06_seg16_boy.jpg</t>
+        </is>
+      </c>
     </row>
     <row r="19" ht="30" customHeight="1">
       <c r="A19" s="10" t="inlineStr">
@@ -25576,6 +26948,11 @@
           <t>3D Pixar Disney style cheerful toddler dance coach, smooth playful animation, vibrant kindergarten studio, soft bright volumetric lighting, clean studio background, highly expressive face, full body dynamic camera shot: Song 'Space Rocket Countdown', Action '第 15 節: 太空安靜無聲息'. 🤫 食指放嘴唇輕輕噓，感受安靜！. The character is stretching arms up high to reach floating elements, standing on tiptoes, joyful posture, looking up with wonder. 4k resolution, 60fps, Disney Pixar render, joyful preschool music video style.</t>
         </is>
       </c>
+      <c r="K19" s="20" t="inlineStr">
+        <is>
+          <t>images/track_06/a1_s06_seg17_boy.jpg</t>
+        </is>
+      </c>
     </row>
     <row r="20" ht="30" customHeight="1">
       <c r="A20" s="8" t="inlineStr">
@@ -25624,6 +27001,11 @@
           <t>3D Pixar Disney style cheerful toddler dance coach, smooth playful animation, vibrant kindergarten studio, soft bright volumetric lighting, clean studio background, highly expressive face, full body dynamic camera shot: Song 'Space Rocket Countdown', Action '第 16 節: 跟土星光環大招手'. 🪐 伸出雙手向美麗土星光環大招手！. The character is waving both hands overhead in friendly wide arcs, swaying gently from side to side, sparkling excited eyes. 4k resolution, 60fps, Disney Pixar render, joyful preschool music video style.</t>
         </is>
       </c>
+      <c r="K20" s="20" t="inlineStr">
+        <is>
+          <t>images/track_06/a1_s06_seg18_boy.jpg</t>
+        </is>
+      </c>
     </row>
     <row r="21" ht="30" customHeight="1">
       <c r="A21" s="10" t="inlineStr">
@@ -25672,6 +27054,11 @@
           <t>3D Pixar Disney style cheerful toddler dance coach, smooth playful animation, vibrant kindergarten studio, soft bright volumetric lighting, clean studio background, highly expressive face, full body dynamic camera shot: Song 'Space Rocket Countdown', Action '第 17 節: 無線電滴答唱歌'. 📻 小手放耳邊，跟著無線電節奏拍手！. The character is marching in place energetically, hands on hips, knees lifting high in rhythmic bounce, enthusiastic happy smile. 4k resolution, 60fps, Disney Pixar render, joyful preschool music video style.</t>
         </is>
       </c>
+      <c r="K21" s="20" t="inlineStr">
+        <is>
+          <t>images/track_06/a1_s06_seg19_boy.jpg</t>
+        </is>
+      </c>
     </row>
     <row r="22" ht="30" customHeight="1">
       <c r="A22" s="8" t="inlineStr">
@@ -25720,6 +27107,11 @@
           <t>3D Pixar Disney style cheerful toddler dance coach, smooth playful animation, vibrant kindergarten studio, soft bright volumetric lighting, clean studio background, highly expressive face, full body dynamic camera shot: Song 'Space Rocket Countdown', Action '第 18 節: 無重力漂浮漫步'. 🎈 雙腳緩慢踩步，像失重一樣輕飄飄！. The character is swaying hips and arms like a breeze, smooth fluid body roll, playful rhythmic dancing, friendly warm smile. 4k resolution, 60fps, Disney Pixar render, joyful preschool music video style.</t>
         </is>
       </c>
+      <c r="K22" s="20" t="inlineStr">
+        <is>
+          <t>images/track_06/a1_s06_seg20_boy.jpg</t>
+        </is>
+      </c>
     </row>
     <row r="23" ht="30" customHeight="1">
       <c r="A23" s="10" t="inlineStr">
@@ -25768,6 +27160,11 @@
           <t>3D Pixar Disney style cheerful toddler dance coach, smooth playful animation, vibrant kindergarten studio, soft bright volumetric lighting, clean studio background, highly expressive face, full body dynamic camera shot: Song 'Space Rocket Countdown', Action '第 19 節: 抓一把星塵閃光'. ✨ 雙手在空中抓取閃亮星光放進口袋！. The character is stretching arms up high to reach floating elements, standing on tiptoes, joyful posture, looking up with wonder. 4k resolution, 60fps, Disney Pixar render, joyful preschool music video style.</t>
         </is>
       </c>
+      <c r="K23" s="20" t="inlineStr">
+        <is>
+          <t>images/track_06/a1_s06_seg21_boy.jpg</t>
+        </is>
+      </c>
     </row>
     <row r="24" ht="30" customHeight="1">
       <c r="A24" s="8" t="inlineStr">
@@ -25816,6 +27213,11 @@
           <t>3D Pixar Disney style cheerful toddler dance coach, smooth playful animation, vibrant kindergarten studio, soft bright volumetric lighting, clean studio background, highly expressive face, full body dynamic camera shot: Song 'Space Rocket Countdown', Action '第 20 節: 咻咻咻再次衝刺'. 🚀 火箭尖尖再次指向宇宙，全力加速！. The character is squatting down and bursting into a high happy jump, feet kicking joyfully in mid-air, both fists punching the sky in victory. 4k resolution, 60fps, Disney Pixar render, joyful preschool music video style.</t>
         </is>
       </c>
+      <c r="K24" s="20" t="inlineStr">
+        <is>
+          <t>images/track_06/a1_s06_seg22_boy.jpg</t>
+        </is>
+      </c>
     </row>
     <row r="25" ht="30" customHeight="1">
       <c r="A25" s="10" t="inlineStr">
@@ -25864,6 +27266,11 @@
           <t>3D Pixar Disney style cheerful toddler dance coach, smooth playful animation, vibrant kindergarten studio, soft bright volumetric lighting, clean studio background, highly expressive face, full body dynamic camera shot: Song 'Space Rocket Countdown', Action '第 21 節: 穿越銀河大光芒'. 🌌 雙手由內向外綻放，穿過光芒！. The character is lifting arms from heart to sky creating a big golden sun circle, chest open, radiant beaming joyful smile. 4k resolution, 60fps, Disney Pixar render, joyful preschool music video style.</t>
         </is>
       </c>
+      <c r="K25" s="20" t="inlineStr">
+        <is>
+          <t>images/track_06/a1_s06_seg23_boy.jpg</t>
+        </is>
+      </c>
     </row>
     <row r="26" ht="30" customHeight="1">
       <c r="A26" s="8" t="inlineStr">
@@ -25912,6 +27319,11 @@
           <t>3D Pixar Disney style cheerful toddler dance coach, smooth playful animation, vibrant kindergarten studio, soft bright volumetric lighting, clean studio background, highly expressive face, full body dynamic camera shot: Song 'Space Rocket Countdown', Action '第 22 節: 飛越高山與月球'. 🌙 單腿微抬雙臂翱翔，比天空更高！. The character is stretching arms up high to reach floating elements, standing on tiptoes, joyful posture, looking up with wonder. 4k resolution, 60fps, Disney Pixar render, joyful preschool music video style.</t>
         </is>
       </c>
+      <c r="K26" s="20" t="inlineStr">
+        <is>
+          <t>images/track_06/a1_s06_seg24_boy.jpg</t>
+        </is>
+      </c>
     </row>
     <row r="27" ht="30" customHeight="1">
       <c r="A27" s="10" t="inlineStr">
@@ -25960,6 +27372,11 @@
           <t>3D Pixar Disney style cheerful toddler dance coach, smooth playful animation, vibrant kindergarten studio, soft bright volumetric lighting, clean studio background, highly expressive face, full body dynamic camera shot: Song 'Space Rocket Countdown', Action '第 23 節: 最棒火箭在夜空'. ⭐ 雙手向上托起星空，神氣無比！. The character is lifting arms from heart to sky creating a big golden sun circle, chest open, radiant beaming joyful smile. 4k resolution, 60fps, Disney Pixar render, joyful preschool music video style.</t>
         </is>
       </c>
+      <c r="K27" s="20" t="inlineStr">
+        <is>
+          <t>images/track_06/a1_s06_seg25_boy.jpg</t>
+        </is>
+      </c>
     </row>
     <row r="28" ht="30" customHeight="1">
       <c r="A28" s="8" t="inlineStr">
@@ -26008,6 +27425,11 @@
           <t>3D Pixar Disney style cheerful toddler dance coach, smooth playful animation, vibrant kindergarten studio, soft bright volumetric lighting, clean studio background, highly expressive face, full body dynamic camera shot: Song 'Space Rocket Countdown', Action '第 24 節: 太空任務大成功'. 🎉 雙手叉腰歡呼大喊：任務完成！. The character is bringing hands together at the chest forming an adorable glowing heart shape, leaning slightly forward, loving gentle smile. 4k resolution, 60fps, Disney Pixar render, joyful preschool music video style.</t>
         </is>
       </c>
+      <c r="K28" s="20" t="inlineStr">
+        <is>
+          <t>images/track_06/a1_s06_seg26_boy.jpg</t>
+        </is>
+      </c>
     </row>
     <row r="29" ht="30" customHeight="1">
       <c r="A29" s="10" t="inlineStr">
@@ -26056,6 +27478,11 @@
           <t>3D Pixar Disney style cheerful toddler dance coach, smooth playful animation, vibrant kindergarten studio, soft bright volumetric lighting, clean studio background, highly expressive face, full body dynamic camera shot: Song 'Space Rocket Countdown', Action '第 25 節: 平穩降落回地球'. 🌍 雙手緩慢下落，平穩降落藍色地球！. The character is marching in place energetically, hands on hips, knees lifting high in rhythmic bounce, enthusiastic happy smile. 4k resolution, 60fps, Disney Pixar render, joyful preschool music video style.</t>
         </is>
       </c>
+      <c r="K29" s="20" t="inlineStr">
+        <is>
+          <t>images/track_06/a1_s06_seg27_boy.jpg</t>
+        </is>
+      </c>
     </row>
     <row r="30" ht="30" customHeight="1">
       <c r="A30" s="8" t="inlineStr">
@@ -26102,6 +27529,11 @@
       <c r="J30" s="9" t="inlineStr">
         <is>
           <t>3D Pixar Disney style cheerful toddler dance coach, smooth playful animation, vibrant kindergarten studio, soft bright volumetric lighting, clean studio background, highly expressive face, full body dynamic camera shot: Song 'Space Rocket Countdown', Action '第 26 節: 外星朋友揮手告別'. 👽 雙手放頭頂比外星觸角，定格大笑！. The character is waving both hands overhead in friendly wide arcs, swaying gently from side to side, sparkling excited eyes. 4k resolution, 60fps, Disney Pixar render, joyful preschool music video style.</t>
+        </is>
+      </c>
+      <c r="K30" s="20" t="inlineStr">
+        <is>
+          <t>images/track_06/a1_s06_seg28_boy.jpg</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
feat: integrate full 23 segment coach videos for Track 1 in videos/T1 directory
</commit_message>
<xml_diff>
--- a/docs/Album1_Dance_Production_Spec.xlsx
+++ b/docs/Album1_Dance_Production_Spec.xlsx
@@ -29,7 +29,7 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <numFmts count="0"/>
-  <fonts count="12">
+  <fonts count="13">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
@@ -98,6 +98,12 @@
     <font>
       <name val="Microsoft JhengHei"/>
       <color rgb="00334155"/>
+      <sz val="9"/>
+    </font>
+    <font>
+      <name val="Microsoft JhengHei"/>
+      <b val="1"/>
+      <color rgb="004338CA"/>
       <sz val="9"/>
     </font>
   </fonts>
@@ -185,7 +191,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="26">
+  <cellXfs count="27">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
@@ -260,6 +266,9 @@
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="10" fillId="0" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="12" fillId="0" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
   </cellXfs>
@@ -19196,7 +19205,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:K25"/>
+  <dimension ref="A1:L25"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="18" customWidth="1" min="1" max="1"/>
@@ -19210,6 +19219,7 @@
     <col width="12" customWidth="1" min="9" max="9"/>
     <col width="55" customWidth="1" min="10" max="10"/>
     <col width="34" customWidth="1" min="11" max="11"/>
+    <col width="32" customWidth="1" min="12" max="12"/>
   </cols>
   <sheetData>
     <row r="1" ht="32" customHeight="1">
@@ -19275,6 +19285,11 @@
           <t>首張圖片路徑 (9:16 720p)</t>
         </is>
       </c>
+      <c r="L2" s="21" t="inlineStr">
+        <is>
+          <t>AI 影片動畫路徑 (T1 目錄)</t>
+        </is>
+      </c>
     </row>
     <row r="3" ht="30" customHeight="1">
       <c r="A3" s="10" t="inlineStr">
@@ -19328,6 +19343,11 @@
           <t>images/track_01/a1_s01_seg01_boy.jpg</t>
         </is>
       </c>
+      <c r="L3" s="26" t="inlineStr">
+        <is>
+          <t>videos/T1/t1_seg_01.mp4</t>
+        </is>
+      </c>
     </row>
     <row r="4" ht="30" customHeight="1">
       <c r="A4" s="8" t="inlineStr">
@@ -19381,6 +19401,11 @@
           <t>images/track_01/a1_s01_seg02_boy.jpg</t>
         </is>
       </c>
+      <c r="L4" s="26" t="inlineStr">
+        <is>
+          <t>videos/T1/t1_seg_02.mp4</t>
+        </is>
+      </c>
     </row>
     <row r="5" ht="30" customHeight="1">
       <c r="A5" s="10" t="inlineStr">
@@ -19434,6 +19459,11 @@
           <t>images/track_01/a1_s01_seg03_boy.jpg</t>
         </is>
       </c>
+      <c r="L5" s="26" t="inlineStr">
+        <is>
+          <t>videos/T1/t1_seg_03.mp4</t>
+        </is>
+      </c>
     </row>
     <row r="6" ht="30" customHeight="1">
       <c r="A6" s="8" t="inlineStr">
@@ -19487,6 +19517,11 @@
           <t>images/track_01/a1_s01_seg04_boy.jpg</t>
         </is>
       </c>
+      <c r="L6" s="26" t="inlineStr">
+        <is>
+          <t>videos/T1/t1_seg_04.mp4</t>
+        </is>
+      </c>
     </row>
     <row r="7" ht="30" customHeight="1">
       <c r="A7" s="10" t="inlineStr">
@@ -19540,6 +19575,11 @@
           <t>images/track_01/a1_s01_seg05_boy.jpg</t>
         </is>
       </c>
+      <c r="L7" s="26" t="inlineStr">
+        <is>
+          <t>videos/T1/t1_seg_05.mp4</t>
+        </is>
+      </c>
     </row>
     <row r="8" ht="30" customHeight="1">
       <c r="A8" s="8" t="inlineStr">
@@ -19593,6 +19633,11 @@
           <t>images/track_01/a1_s01_seg06_boy.jpg</t>
         </is>
       </c>
+      <c r="L8" s="26" t="inlineStr">
+        <is>
+          <t>videos/T1/t1_seg_06.mp4</t>
+        </is>
+      </c>
     </row>
     <row r="9" ht="30" customHeight="1">
       <c r="A9" s="10" t="inlineStr">
@@ -19646,6 +19691,11 @@
           <t>images/track_01/a1_s01_seg07_boy.jpg</t>
         </is>
       </c>
+      <c r="L9" s="26" t="inlineStr">
+        <is>
+          <t>videos/T1/t1_seg_07.mp4</t>
+        </is>
+      </c>
     </row>
     <row r="10" ht="30" customHeight="1">
       <c r="A10" s="8" t="inlineStr">
@@ -19699,6 +19749,11 @@
           <t>images/track_01/a1_s01_seg08_boy.jpg</t>
         </is>
       </c>
+      <c r="L10" s="26" t="inlineStr">
+        <is>
+          <t>videos/T1/t1_seg_08.mp4</t>
+        </is>
+      </c>
     </row>
     <row r="11" ht="30" customHeight="1">
       <c r="A11" s="10" t="inlineStr">
@@ -19752,6 +19807,11 @@
           <t>images/track_01/a1_s01_seg09_boy.jpg</t>
         </is>
       </c>
+      <c r="L11" s="26" t="inlineStr">
+        <is>
+          <t>videos/T1/t1_seg_09.mp4</t>
+        </is>
+      </c>
     </row>
     <row r="12" ht="30" customHeight="1">
       <c r="A12" s="8" t="inlineStr">
@@ -19805,6 +19865,11 @@
           <t>images/track_01/a1_s01_seg10_boy.jpg</t>
         </is>
       </c>
+      <c r="L12" s="26" t="inlineStr">
+        <is>
+          <t>videos/T1/t1_seg_10.mp4</t>
+        </is>
+      </c>
     </row>
     <row r="13" ht="30" customHeight="1">
       <c r="A13" s="10" t="inlineStr">
@@ -19858,6 +19923,11 @@
           <t>images/track_01/a1_s01_seg11_boy.jpg</t>
         </is>
       </c>
+      <c r="L13" s="26" t="inlineStr">
+        <is>
+          <t>videos/T1/t1_seg_11.mp4</t>
+        </is>
+      </c>
     </row>
     <row r="14" ht="30" customHeight="1">
       <c r="A14" s="8" t="inlineStr">
@@ -19911,6 +19981,11 @@
           <t>images/track_01/a1_s01_seg12_boy.jpg</t>
         </is>
       </c>
+      <c r="L14" s="26" t="inlineStr">
+        <is>
+          <t>videos/T1/t1_seg_12.mp4</t>
+        </is>
+      </c>
     </row>
     <row r="15" ht="30" customHeight="1">
       <c r="A15" s="10" t="inlineStr">
@@ -19964,6 +20039,11 @@
           <t>images/track_01/a1_s01_seg13_boy.jpg</t>
         </is>
       </c>
+      <c r="L15" s="26" t="inlineStr">
+        <is>
+          <t>videos/T1/t1_seg_13.mp4</t>
+        </is>
+      </c>
     </row>
     <row r="16" ht="30" customHeight="1">
       <c r="A16" s="8" t="inlineStr">
@@ -20017,6 +20097,11 @@
           <t>images/track_01/a1_s01_seg14_boy.jpg</t>
         </is>
       </c>
+      <c r="L16" s="26" t="inlineStr">
+        <is>
+          <t>videos/T1/t1_seg_14.mp4</t>
+        </is>
+      </c>
     </row>
     <row r="17" ht="30" customHeight="1">
       <c r="A17" s="10" t="inlineStr">
@@ -20070,6 +20155,11 @@
           <t>images/track_01/a1_s01_seg15_boy.jpg</t>
         </is>
       </c>
+      <c r="L17" s="26" t="inlineStr">
+        <is>
+          <t>videos/T1/t1_seg_15.mp4</t>
+        </is>
+      </c>
     </row>
     <row r="18" ht="30" customHeight="1">
       <c r="A18" s="8" t="inlineStr">
@@ -20123,6 +20213,11 @@
           <t>images/track_01/a1_s01_seg16_boy.jpg</t>
         </is>
       </c>
+      <c r="L18" s="26" t="inlineStr">
+        <is>
+          <t>videos/T1/t1_seg_16.mp4</t>
+        </is>
+      </c>
     </row>
     <row r="19" ht="30" customHeight="1">
       <c r="A19" s="10" t="inlineStr">
@@ -20176,6 +20271,11 @@
           <t>images/track_01/a1_s01_seg17_boy.jpg</t>
         </is>
       </c>
+      <c r="L19" s="26" t="inlineStr">
+        <is>
+          <t>videos/T1/t1_seg_17.mp4</t>
+        </is>
+      </c>
     </row>
     <row r="20" ht="30" customHeight="1">
       <c r="A20" s="8" t="inlineStr">
@@ -20229,6 +20329,11 @@
           <t>images/track_01/a1_s01_seg18_boy.jpg</t>
         </is>
       </c>
+      <c r="L20" s="26" t="inlineStr">
+        <is>
+          <t>videos/T1/t1_seg_18.mp4</t>
+        </is>
+      </c>
     </row>
     <row r="21" ht="30" customHeight="1">
       <c r="A21" s="10" t="inlineStr">
@@ -20282,6 +20387,11 @@
           <t>images/track_01/a1_s01_seg19_boy.jpg</t>
         </is>
       </c>
+      <c r="L21" s="26" t="inlineStr">
+        <is>
+          <t>videos/T1/t1_seg_19.mp4</t>
+        </is>
+      </c>
     </row>
     <row r="22" ht="30" customHeight="1">
       <c r="A22" s="8" t="inlineStr">
@@ -20335,6 +20445,11 @@
           <t>images/track_01/a1_s01_seg20_boy.jpg</t>
         </is>
       </c>
+      <c r="L22" s="26" t="inlineStr">
+        <is>
+          <t>videos/T1/t1_seg_20.mp4</t>
+        </is>
+      </c>
     </row>
     <row r="23" ht="30" customHeight="1">
       <c r="A23" s="10" t="inlineStr">
@@ -20388,6 +20503,11 @@
           <t>images/track_01/a1_s01_seg21_boy.jpg</t>
         </is>
       </c>
+      <c r="L23" s="26" t="inlineStr">
+        <is>
+          <t>videos/T1/t1_seg_21.mp4</t>
+        </is>
+      </c>
     </row>
     <row r="24" ht="30" customHeight="1">
       <c r="A24" s="8" t="inlineStr">
@@ -20441,6 +20561,11 @@
           <t>images/track_01/a1_s01_seg22_boy.jpg</t>
         </is>
       </c>
+      <c r="L24" s="26" t="inlineStr">
+        <is>
+          <t>videos/T1/t1_seg_22.mp4</t>
+        </is>
+      </c>
     </row>
     <row r="25" ht="30" customHeight="1">
       <c r="A25" s="10" t="inlineStr">
@@ -20492,6 +20617,11 @@
       <c r="K25" s="20" t="inlineStr">
         <is>
           <t>images/track_01/a1_s01_seg23_boy.jpg</t>
+        </is>
+      </c>
+      <c r="L25" s="26" t="inlineStr">
+        <is>
+          <t>videos/T1/t1_seg_23.mp4</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
feat: integrate 20 T2 dance animation videos for Track 02 and fallback missing seg 07 & 17 to coach photos
</commit_message>
<xml_diff>
--- a/docs/Album1_Dance_Production_Spec.xlsx
+++ b/docs/Album1_Dance_Production_Spec.xlsx
@@ -29,7 +29,7 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <numFmts count="0"/>
-  <fonts count="13">
+  <fonts count="14">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
@@ -106,8 +106,14 @@
       <color rgb="004338CA"/>
       <sz val="9"/>
     </font>
+    <font>
+      <name val="Microsoft JhengHei"/>
+      <b val="1"/>
+      <color rgb="00DC2626"/>
+      <sz val="9"/>
+    </font>
   </fonts>
-  <fills count="8">
+  <fills count="9">
     <fill>
       <patternFill/>
     </fill>
@@ -148,6 +154,12 @@
       <patternFill patternType="solid">
         <fgColor rgb="000D9488"/>
         <bgColor rgb="000D9488"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00FEE2E2"/>
+        <bgColor rgb="00FEE2E2"/>
       </patternFill>
     </fill>
   </fills>
@@ -191,7 +203,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="27">
+  <cellXfs count="28">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
@@ -269,6 +281,9 @@
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="12" fillId="0" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="13" fillId="8" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
   </cellXfs>
@@ -20639,7 +20654,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:K24"/>
+  <dimension ref="A1:L24"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="18" customWidth="1" min="1" max="1"/>
@@ -20653,6 +20668,7 @@
     <col width="12" customWidth="1" min="9" max="9"/>
     <col width="55" customWidth="1" min="10" max="10"/>
     <col width="34" customWidth="1" min="11" max="11"/>
+    <col width="34" customWidth="1" min="12" max="12"/>
   </cols>
   <sheetData>
     <row r="1" ht="32" customHeight="1">
@@ -20718,6 +20734,11 @@
           <t>首張圖片路徑 (9:16 720p)</t>
         </is>
       </c>
+      <c r="L2" s="21" t="inlineStr">
+        <is>
+          <t>AI 影片動畫路徑 (T2 目錄)</t>
+        </is>
+      </c>
     </row>
     <row r="3" ht="30" customHeight="1">
       <c r="A3" s="10" t="inlineStr">
@@ -20771,6 +20792,11 @@
           <t>images/track_02/a1_s02_seg01_girl.jpg</t>
         </is>
       </c>
+      <c r="L3" s="26" t="inlineStr">
+        <is>
+          <t>videos/T2/t2_seg_01.mp4</t>
+        </is>
+      </c>
     </row>
     <row r="4" ht="30" customHeight="1">
       <c r="A4" s="8" t="inlineStr">
@@ -20824,6 +20850,11 @@
           <t>images/track_02/a1_s02_seg02_girl.jpg</t>
         </is>
       </c>
+      <c r="L4" s="26" t="inlineStr">
+        <is>
+          <t>videos/T2/t2_seg_02.mp4</t>
+        </is>
+      </c>
     </row>
     <row r="5" ht="30" customHeight="1">
       <c r="A5" s="10" t="inlineStr">
@@ -20877,6 +20908,11 @@
           <t>images/track_02/a1_s02_seg03_girl.jpg</t>
         </is>
       </c>
+      <c r="L5" s="26" t="inlineStr">
+        <is>
+          <t>videos/T2/t2_seg_03.mp4</t>
+        </is>
+      </c>
     </row>
     <row r="6" ht="30" customHeight="1">
       <c r="A6" s="8" t="inlineStr">
@@ -20930,6 +20966,11 @@
           <t>images/track_02/a1_s02_seg04_girl.jpg</t>
         </is>
       </c>
+      <c r="L6" s="26" t="inlineStr">
+        <is>
+          <t>videos/T2/t2_seg_04.mp4</t>
+        </is>
+      </c>
     </row>
     <row r="7" ht="30" customHeight="1">
       <c r="A7" s="10" t="inlineStr">
@@ -20983,6 +21024,11 @@
           <t>images/track_02/a1_s02_seg05_girl.jpg</t>
         </is>
       </c>
+      <c r="L7" s="26" t="inlineStr">
+        <is>
+          <t>videos/T2/t2_seg_05.mp4</t>
+        </is>
+      </c>
     </row>
     <row r="8" ht="30" customHeight="1">
       <c r="A8" s="8" t="inlineStr">
@@ -21036,6 +21082,11 @@
           <t>images/track_02/a1_s02_seg06_girl.jpg</t>
         </is>
       </c>
+      <c r="L8" s="26" t="inlineStr">
+        <is>
+          <t>videos/T2/t2_seg_06.mp4</t>
+        </is>
+      </c>
     </row>
     <row r="9" ht="30" customHeight="1">
       <c r="A9" s="10" t="inlineStr">
@@ -21089,6 +21140,11 @@
           <t>images/track_02/a1_s02_seg07_girl.jpg</t>
         </is>
       </c>
+      <c r="L9" s="27" t="inlineStr">
+        <is>
+          <t>❌ 缺少影片 (暫以靜態美美寫真代替)</t>
+        </is>
+      </c>
     </row>
     <row r="10" ht="30" customHeight="1">
       <c r="A10" s="8" t="inlineStr">
@@ -21142,6 +21198,11 @@
           <t>images/track_02/a1_s02_seg08_girl.jpg</t>
         </is>
       </c>
+      <c r="L10" s="26" t="inlineStr">
+        <is>
+          <t>videos/T2/t2_seg_08.mp4</t>
+        </is>
+      </c>
     </row>
     <row r="11" ht="30" customHeight="1">
       <c r="A11" s="10" t="inlineStr">
@@ -21195,6 +21256,11 @@
           <t>images/track_02/a1_s02_seg09_girl.jpg</t>
         </is>
       </c>
+      <c r="L11" s="26" t="inlineStr">
+        <is>
+          <t>videos/T2/t2_seg_09.mp4</t>
+        </is>
+      </c>
     </row>
     <row r="12" ht="30" customHeight="1">
       <c r="A12" s="8" t="inlineStr">
@@ -21248,6 +21314,11 @@
           <t>images/track_02/a1_s02_seg10_girl.jpg</t>
         </is>
       </c>
+      <c r="L12" s="26" t="inlineStr">
+        <is>
+          <t>videos/T2/t2_seg_10.mp4</t>
+        </is>
+      </c>
     </row>
     <row r="13" ht="30" customHeight="1">
       <c r="A13" s="10" t="inlineStr">
@@ -21301,6 +21372,11 @@
           <t>images/track_02/a1_s02_seg11_girl.jpg</t>
         </is>
       </c>
+      <c r="L13" s="26" t="inlineStr">
+        <is>
+          <t>videos/T2/t2_seg_11.mp4</t>
+        </is>
+      </c>
     </row>
     <row r="14" ht="30" customHeight="1">
       <c r="A14" s="8" t="inlineStr">
@@ -21354,6 +21430,11 @@
           <t>images/track_02/a1_s02_seg12_girl.jpg</t>
         </is>
       </c>
+      <c r="L14" s="26" t="inlineStr">
+        <is>
+          <t>videos/T2/t2_seg_12.mp4</t>
+        </is>
+      </c>
     </row>
     <row r="15" ht="30" customHeight="1">
       <c r="A15" s="10" t="inlineStr">
@@ -21407,6 +21488,11 @@
           <t>images/track_02/a1_s02_seg13_girl.jpg</t>
         </is>
       </c>
+      <c r="L15" s="26" t="inlineStr">
+        <is>
+          <t>videos/T2/t2_seg_13.mp4</t>
+        </is>
+      </c>
     </row>
     <row r="16" ht="30" customHeight="1">
       <c r="A16" s="8" t="inlineStr">
@@ -21460,6 +21546,11 @@
           <t>images/track_02/a1_s02_seg14_girl.jpg</t>
         </is>
       </c>
+      <c r="L16" s="26" t="inlineStr">
+        <is>
+          <t>videos/T2/t2_seg_14.mp4</t>
+        </is>
+      </c>
     </row>
     <row r="17" ht="30" customHeight="1">
       <c r="A17" s="10" t="inlineStr">
@@ -21513,6 +21604,11 @@
           <t>images/track_02/a1_s02_seg15_girl.jpg</t>
         </is>
       </c>
+      <c r="L17" s="26" t="inlineStr">
+        <is>
+          <t>videos/T2/t2_seg_15.mp4</t>
+        </is>
+      </c>
     </row>
     <row r="18" ht="30" customHeight="1">
       <c r="A18" s="8" t="inlineStr">
@@ -21566,6 +21662,11 @@
           <t>images/track_02/a1_s02_seg16_girl.jpg</t>
         </is>
       </c>
+      <c r="L18" s="26" t="inlineStr">
+        <is>
+          <t>videos/T2/t2_seg_16.mp4</t>
+        </is>
+      </c>
     </row>
     <row r="19" ht="30" customHeight="1">
       <c r="A19" s="10" t="inlineStr">
@@ -21619,6 +21720,11 @@
           <t>images/track_02/a1_s02_seg17_girl.jpg</t>
         </is>
       </c>
+      <c r="L19" s="27" t="inlineStr">
+        <is>
+          <t>❌ 缺少影片 (暫以靜態美美寫真代替)</t>
+        </is>
+      </c>
     </row>
     <row r="20" ht="30" customHeight="1">
       <c r="A20" s="8" t="inlineStr">
@@ -21672,6 +21778,11 @@
           <t>images/track_02/a1_s02_seg18_girl.jpg</t>
         </is>
       </c>
+      <c r="L20" s="26" t="inlineStr">
+        <is>
+          <t>videos/T2/t2_seg_18.mp4</t>
+        </is>
+      </c>
     </row>
     <row r="21" ht="30" customHeight="1">
       <c r="A21" s="10" t="inlineStr">
@@ -21725,6 +21836,11 @@
           <t>images/track_02/a1_s02_seg19_girl.jpg</t>
         </is>
       </c>
+      <c r="L21" s="26" t="inlineStr">
+        <is>
+          <t>videos/T2/t2_seg_19.mp4</t>
+        </is>
+      </c>
     </row>
     <row r="22" ht="30" customHeight="1">
       <c r="A22" s="8" t="inlineStr">
@@ -21778,6 +21894,11 @@
           <t>images/track_02/a1_s02_seg20_girl.jpg</t>
         </is>
       </c>
+      <c r="L22" s="26" t="inlineStr">
+        <is>
+          <t>videos/T2/t2_seg_20.mp4</t>
+        </is>
+      </c>
     </row>
     <row r="23" ht="30" customHeight="1">
       <c r="A23" s="10" t="inlineStr">
@@ -21831,6 +21952,11 @@
           <t>images/track_02/a1_s02_seg21_girl.jpg</t>
         </is>
       </c>
+      <c r="L23" s="26" t="inlineStr">
+        <is>
+          <t>videos/T2/t2_seg_21.mp4</t>
+        </is>
+      </c>
     </row>
     <row r="24" ht="30" customHeight="1">
       <c r="A24" s="8" t="inlineStr">
@@ -21882,6 +22008,11 @@
       <c r="K24" s="20" t="inlineStr">
         <is>
           <t>images/track_02/a1_s02_seg22_girl.jpg</t>
+        </is>
+      </c>
+      <c r="L24" s="26" t="inlineStr">
+        <is>
+          <t>videos/T2/t2_seg_22.mp4</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
feat: integrate all 22 T3 animation videos for Track 03 (Rainbow Color Splash)
</commit_message>
<xml_diff>
--- a/docs/Album1_Dance_Production_Spec.xlsx
+++ b/docs/Album1_Dance_Production_Spec.xlsx
@@ -29,7 +29,7 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <numFmts count="0"/>
-  <fonts count="14">
+  <fonts count="15">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
@@ -110,6 +110,12 @@
       <name val="Microsoft JhengHei"/>
       <b val="1"/>
       <color rgb="00DC2626"/>
+      <sz val="9"/>
+    </font>
+    <font>
+      <name val="Microsoft JhengHei"/>
+      <b val="1"/>
+      <color rgb="000284C7"/>
       <sz val="9"/>
     </font>
   </fonts>
@@ -203,7 +209,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="28">
+  <cellXfs count="30">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
@@ -285,6 +291,12 @@
     </xf>
     <xf numFmtId="0" fontId="13" fillId="8" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="4" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="14" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -6909,12 +6921,12 @@
       </c>
       <c r="H5" s="25" t="inlineStr">
         <is>
-          <t>images/track_03/a1_s03_seg01_girl.jpg</t>
+          <t>images/track_03/a1_s03_seg01_boy.jpg</t>
         </is>
       </c>
       <c r="I5" s="23" t="inlineStr">
         <is>
-          <t>a1_s03_seg01_girl.jpg ~ a1_s03_seg22_girl.jpg (共 22 張)</t>
+          <t>a1_s03_seg01_boy.jpg ~ a1_s03_seg22_boy.jpg (共 22 張)</t>
         </is>
       </c>
       <c r="J5" s="24" t="inlineStr">
@@ -22030,7 +22042,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:K24"/>
+  <dimension ref="A1:L24"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="18" customWidth="1" min="1" max="1"/>
@@ -22044,6 +22056,7 @@
     <col width="12" customWidth="1" min="9" max="9"/>
     <col width="55" customWidth="1" min="10" max="10"/>
     <col width="34" customWidth="1" min="11" max="11"/>
+    <col width="28" customWidth="1" min="12" max="12"/>
   </cols>
   <sheetData>
     <row r="1" ht="32" customHeight="1">
@@ -22109,6 +22122,11 @@
           <t>首張圖片路徑 (9:16 720p)</t>
         </is>
       </c>
+      <c r="L2" s="28" t="inlineStr">
+        <is>
+          <t>AI 影片動畫路徑 (T3 目錄)</t>
+        </is>
+      </c>
     </row>
     <row r="3" ht="30" customHeight="1">
       <c r="A3" s="10" t="inlineStr">
@@ -22159,7 +22177,12 @@
       </c>
       <c r="K3" s="20" t="inlineStr">
         <is>
-          <t>images/track_03/a1_s03_seg01_girl.jpg</t>
+          <t>images/track_03/a1_s03_seg01_boy.jpg</t>
+        </is>
+      </c>
+      <c r="L3" s="29" t="inlineStr">
+        <is>
+          <t>videos/T3/t3_seg_01.mp4</t>
         </is>
       </c>
     </row>
@@ -22215,6 +22238,11 @@
           <t>images/track_03/a1_s03_seg02_girl.jpg</t>
         </is>
       </c>
+      <c r="L4" s="29" t="inlineStr">
+        <is>
+          <t>videos/T3/t3_seg_02.mp4</t>
+        </is>
+      </c>
     </row>
     <row r="5" ht="30" customHeight="1">
       <c r="A5" s="10" t="inlineStr">
@@ -22268,6 +22296,11 @@
           <t>images/track_03/a1_s03_seg03_girl.jpg</t>
         </is>
       </c>
+      <c r="L5" s="29" t="inlineStr">
+        <is>
+          <t>videos/T3/t3_seg_03.mp4</t>
+        </is>
+      </c>
     </row>
     <row r="6" ht="30" customHeight="1">
       <c r="A6" s="8" t="inlineStr">
@@ -22321,6 +22354,11 @@
           <t>images/track_03/a1_s03_seg04_girl.jpg</t>
         </is>
       </c>
+      <c r="L6" s="29" t="inlineStr">
+        <is>
+          <t>videos/T3/t3_seg_04.mp4</t>
+        </is>
+      </c>
     </row>
     <row r="7" ht="30" customHeight="1">
       <c r="A7" s="10" t="inlineStr">
@@ -22374,6 +22412,11 @@
           <t>images/track_03/a1_s03_seg05_girl.jpg</t>
         </is>
       </c>
+      <c r="L7" s="29" t="inlineStr">
+        <is>
+          <t>videos/T3/t3_seg_05.mp4</t>
+        </is>
+      </c>
     </row>
     <row r="8" ht="30" customHeight="1">
       <c r="A8" s="8" t="inlineStr">
@@ -22427,6 +22470,11 @@
           <t>images/track_03/a1_s03_seg06_girl.jpg</t>
         </is>
       </c>
+      <c r="L8" s="29" t="inlineStr">
+        <is>
+          <t>videos/T3/t3_seg_06.mp4</t>
+        </is>
+      </c>
     </row>
     <row r="9" ht="30" customHeight="1">
       <c r="A9" s="10" t="inlineStr">
@@ -22480,6 +22528,11 @@
           <t>images/track_03/a1_s03_seg07_girl.jpg</t>
         </is>
       </c>
+      <c r="L9" s="29" t="inlineStr">
+        <is>
+          <t>videos/T3/t3_seg_07.mp4</t>
+        </is>
+      </c>
     </row>
     <row r="10" ht="30" customHeight="1">
       <c r="A10" s="8" t="inlineStr">
@@ -22533,6 +22586,11 @@
           <t>images/track_03/a1_s03_seg08_girl.jpg</t>
         </is>
       </c>
+      <c r="L10" s="29" t="inlineStr">
+        <is>
+          <t>videos/T3/t3_seg_08.mp4</t>
+        </is>
+      </c>
     </row>
     <row r="11" ht="30" customHeight="1">
       <c r="A11" s="10" t="inlineStr">
@@ -22586,6 +22644,11 @@
           <t>images/track_03/a1_s03_seg09_girl.jpg</t>
         </is>
       </c>
+      <c r="L11" s="29" t="inlineStr">
+        <is>
+          <t>videos/T3/t3_seg_09.mp4</t>
+        </is>
+      </c>
     </row>
     <row r="12" ht="30" customHeight="1">
       <c r="A12" s="8" t="inlineStr">
@@ -22639,6 +22702,11 @@
           <t>images/track_03/a1_s03_seg10_girl.jpg</t>
         </is>
       </c>
+      <c r="L12" s="29" t="inlineStr">
+        <is>
+          <t>videos/T3/t3_seg_10.mp4</t>
+        </is>
+      </c>
     </row>
     <row r="13" ht="30" customHeight="1">
       <c r="A13" s="10" t="inlineStr">
@@ -22692,6 +22760,11 @@
           <t>images/track_03/a1_s03_seg11_girl.jpg</t>
         </is>
       </c>
+      <c r="L13" s="29" t="inlineStr">
+        <is>
+          <t>videos/T3/t3_seg_11.mp4</t>
+        </is>
+      </c>
     </row>
     <row r="14" ht="30" customHeight="1">
       <c r="A14" s="8" t="inlineStr">
@@ -22745,6 +22818,11 @@
           <t>images/track_03/a1_s03_seg12_girl.jpg</t>
         </is>
       </c>
+      <c r="L14" s="29" t="inlineStr">
+        <is>
+          <t>videos/T3/t3_seg_12.mp4</t>
+        </is>
+      </c>
     </row>
     <row r="15" ht="30" customHeight="1">
       <c r="A15" s="10" t="inlineStr">
@@ -22798,6 +22876,11 @@
           <t>images/track_03/a1_s03_seg13_girl.jpg</t>
         </is>
       </c>
+      <c r="L15" s="29" t="inlineStr">
+        <is>
+          <t>videos/T3/t3_seg_13.mp4</t>
+        </is>
+      </c>
     </row>
     <row r="16" ht="30" customHeight="1">
       <c r="A16" s="8" t="inlineStr">
@@ -22851,6 +22934,11 @@
           <t>images/track_03/a1_s03_seg14_girl.jpg</t>
         </is>
       </c>
+      <c r="L16" s="29" t="inlineStr">
+        <is>
+          <t>videos/T3/t3_seg_14.mp4</t>
+        </is>
+      </c>
     </row>
     <row r="17" ht="30" customHeight="1">
       <c r="A17" s="10" t="inlineStr">
@@ -22904,6 +22992,11 @@
           <t>images/track_03/a1_s03_seg15_girl.jpg</t>
         </is>
       </c>
+      <c r="L17" s="29" t="inlineStr">
+        <is>
+          <t>videos/T3/t3_seg_15.mp4</t>
+        </is>
+      </c>
     </row>
     <row r="18" ht="30" customHeight="1">
       <c r="A18" s="8" t="inlineStr">
@@ -22957,6 +23050,11 @@
           <t>images/track_03/a1_s03_seg16_girl.jpg</t>
         </is>
       </c>
+      <c r="L18" s="29" t="inlineStr">
+        <is>
+          <t>videos/T3/t3_seg_16.mp4</t>
+        </is>
+      </c>
     </row>
     <row r="19" ht="30" customHeight="1">
       <c r="A19" s="10" t="inlineStr">
@@ -23010,6 +23108,11 @@
           <t>images/track_03/a1_s03_seg17_girl.jpg</t>
         </is>
       </c>
+      <c r="L19" s="29" t="inlineStr">
+        <is>
+          <t>videos/T3/t3_seg_17.mp4</t>
+        </is>
+      </c>
     </row>
     <row r="20" ht="30" customHeight="1">
       <c r="A20" s="8" t="inlineStr">
@@ -23063,6 +23166,11 @@
           <t>images/track_03/a1_s03_seg18_girl.jpg</t>
         </is>
       </c>
+      <c r="L20" s="29" t="inlineStr">
+        <is>
+          <t>videos/T3/t3_seg_18.mp4</t>
+        </is>
+      </c>
     </row>
     <row r="21" ht="30" customHeight="1">
       <c r="A21" s="10" t="inlineStr">
@@ -23116,6 +23224,11 @@
           <t>images/track_03/a1_s03_seg19_girl.jpg</t>
         </is>
       </c>
+      <c r="L21" s="29" t="inlineStr">
+        <is>
+          <t>videos/T3/t3_seg_19.mp4</t>
+        </is>
+      </c>
     </row>
     <row r="22" ht="30" customHeight="1">
       <c r="A22" s="8" t="inlineStr">
@@ -23169,6 +23282,11 @@
           <t>images/track_03/a1_s03_seg20_girl.jpg</t>
         </is>
       </c>
+      <c r="L22" s="29" t="inlineStr">
+        <is>
+          <t>videos/T3/t3_seg_20.mp4</t>
+        </is>
+      </c>
     </row>
     <row r="23" ht="30" customHeight="1">
       <c r="A23" s="10" t="inlineStr">
@@ -23222,6 +23340,11 @@
           <t>images/track_03/a1_s03_seg21_girl.jpg</t>
         </is>
       </c>
+      <c r="L23" s="29" t="inlineStr">
+        <is>
+          <t>videos/T3/t3_seg_21.mp4</t>
+        </is>
+      </c>
     </row>
     <row r="24" ht="30" customHeight="1">
       <c r="A24" s="8" t="inlineStr">
@@ -23273,6 +23396,11 @@
       <c r="K24" s="20" t="inlineStr">
         <is>
           <t>images/track_03/a1_s03_seg22_girl.jpg</t>
+        </is>
+      </c>
+      <c r="L24" s="29" t="inlineStr">
+        <is>
+          <t>videos/T3/t3_seg_22.mp4</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
feat: customize Track 04 lead dance coach character based on photo with Pixar styling
</commit_message>
<xml_diff>
--- a/docs/Album1_Dance_Production_Spec.xlsx
+++ b/docs/Album1_Dance_Production_Spec.xlsx
@@ -6983,12 +6983,12 @@
       </c>
       <c r="H6" s="25" t="inlineStr">
         <is>
-          <t>images/track_04/a1_s04_seg01_boy.jpg</t>
+          <t>images/track_04/a1_s04_seg01_girl.jpg</t>
         </is>
       </c>
       <c r="I6" s="23" t="inlineStr">
         <is>
-          <t>a1_s04_seg01_boy.jpg ~ a1_s04_seg26_boy.jpg (共 26 張)</t>
+          <t>a1_s04_seg01_girl.jpg ~ a1_s04_seg26_girl.jpg (共 26 張)</t>
         </is>
       </c>
       <c r="J6" s="24" t="inlineStr">
@@ -23547,7 +23547,7 @@
       </c>
       <c r="K3" s="20" t="inlineStr">
         <is>
-          <t>images/track_04/a1_s04_seg01_boy.jpg</t>
+          <t>images/track_04/a1_s04_seg01_girl.jpg</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
feat: integrate all 26 T4 animation videos for Track 04 (Animal Safari March)
</commit_message>
<xml_diff>
--- a/docs/Album1_Dance_Production_Spec.xlsx
+++ b/docs/Album1_Dance_Production_Spec.xlsx
@@ -23418,7 +23418,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:K28"/>
+  <dimension ref="A1:L28"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="18" customWidth="1" min="1" max="1"/>
@@ -23432,6 +23432,7 @@
     <col width="12" customWidth="1" min="9" max="9"/>
     <col width="55" customWidth="1" min="10" max="10"/>
     <col width="34" customWidth="1" min="11" max="11"/>
+    <col width="28" customWidth="1" min="12" max="12"/>
   </cols>
   <sheetData>
     <row r="1" ht="32" customHeight="1">
@@ -23497,6 +23498,11 @@
           <t>首張圖片路徑 (9:16 720p)</t>
         </is>
       </c>
+      <c r="L2" s="28" t="inlineStr">
+        <is>
+          <t>AI 影片動畫路徑 (T4 目錄)</t>
+        </is>
+      </c>
     </row>
     <row r="3" ht="30" customHeight="1">
       <c r="A3" s="10" t="inlineStr">
@@ -23550,6 +23556,11 @@
           <t>images/track_04/a1_s04_seg01_girl.jpg</t>
         </is>
       </c>
+      <c r="L3" s="29" t="inlineStr">
+        <is>
+          <t>videos/T4/t4_seg_01.mp4</t>
+        </is>
+      </c>
     </row>
     <row r="4" ht="30" customHeight="1">
       <c r="A4" s="8" t="inlineStr">
@@ -23603,6 +23614,11 @@
           <t>images/track_04/a1_s04_seg02_boy.jpg</t>
         </is>
       </c>
+      <c r="L4" s="29" t="inlineStr">
+        <is>
+          <t>videos/T4/t4_seg_02.mp4</t>
+        </is>
+      </c>
     </row>
     <row r="5" ht="30" customHeight="1">
       <c r="A5" s="10" t="inlineStr">
@@ -23656,6 +23672,11 @@
           <t>images/track_04/a1_s04_seg03_boy.jpg</t>
         </is>
       </c>
+      <c r="L5" s="29" t="inlineStr">
+        <is>
+          <t>videos/T4/t4_seg_03.mp4</t>
+        </is>
+      </c>
     </row>
     <row r="6" ht="30" customHeight="1">
       <c r="A6" s="8" t="inlineStr">
@@ -23709,6 +23730,11 @@
           <t>images/track_04/a1_s04_seg04_boy.jpg</t>
         </is>
       </c>
+      <c r="L6" s="29" t="inlineStr">
+        <is>
+          <t>videos/T4/t4_seg_04.mp4</t>
+        </is>
+      </c>
     </row>
     <row r="7" ht="30" customHeight="1">
       <c r="A7" s="10" t="inlineStr">
@@ -23762,6 +23788,11 @@
           <t>images/track_04/a1_s04_seg05_boy.jpg</t>
         </is>
       </c>
+      <c r="L7" s="29" t="inlineStr">
+        <is>
+          <t>videos/T4/t4_seg_05.mp4</t>
+        </is>
+      </c>
     </row>
     <row r="8" ht="30" customHeight="1">
       <c r="A8" s="8" t="inlineStr">
@@ -23815,6 +23846,11 @@
           <t>images/track_04/a1_s04_seg06_boy.jpg</t>
         </is>
       </c>
+      <c r="L8" s="29" t="inlineStr">
+        <is>
+          <t>videos/T4/t4_seg_06.mp4</t>
+        </is>
+      </c>
     </row>
     <row r="9" ht="30" customHeight="1">
       <c r="A9" s="10" t="inlineStr">
@@ -23868,6 +23904,11 @@
           <t>images/track_04/a1_s04_seg07_boy.jpg</t>
         </is>
       </c>
+      <c r="L9" s="29" t="inlineStr">
+        <is>
+          <t>videos/T4/t4_seg_07.mp4</t>
+        </is>
+      </c>
     </row>
     <row r="10" ht="30" customHeight="1">
       <c r="A10" s="8" t="inlineStr">
@@ -23921,6 +23962,11 @@
           <t>images/track_04/a1_s04_seg08_boy.jpg</t>
         </is>
       </c>
+      <c r="L10" s="29" t="inlineStr">
+        <is>
+          <t>videos/T4/t4_seg_08.mp4</t>
+        </is>
+      </c>
     </row>
     <row r="11" ht="30" customHeight="1">
       <c r="A11" s="10" t="inlineStr">
@@ -23974,6 +24020,11 @@
           <t>images/track_04/a1_s04_seg09_boy.jpg</t>
         </is>
       </c>
+      <c r="L11" s="29" t="inlineStr">
+        <is>
+          <t>videos/T4/t4_seg_09.mp4</t>
+        </is>
+      </c>
     </row>
     <row r="12" ht="30" customHeight="1">
       <c r="A12" s="8" t="inlineStr">
@@ -24027,6 +24078,11 @@
           <t>images/track_04/a1_s04_seg10_boy.jpg</t>
         </is>
       </c>
+      <c r="L12" s="29" t="inlineStr">
+        <is>
+          <t>videos/T4/t4_seg_10.mp4</t>
+        </is>
+      </c>
     </row>
     <row r="13" ht="30" customHeight="1">
       <c r="A13" s="10" t="inlineStr">
@@ -24080,6 +24136,11 @@
           <t>images/track_04/a1_s04_seg11_boy.jpg</t>
         </is>
       </c>
+      <c r="L13" s="29" t="inlineStr">
+        <is>
+          <t>videos/T4/t4_seg_11.mp4</t>
+        </is>
+      </c>
     </row>
     <row r="14" ht="30" customHeight="1">
       <c r="A14" s="8" t="inlineStr">
@@ -24133,6 +24194,11 @@
           <t>images/track_04/a1_s04_seg12_boy.jpg</t>
         </is>
       </c>
+      <c r="L14" s="29" t="inlineStr">
+        <is>
+          <t>videos/T4/t4_seg_12.mp4</t>
+        </is>
+      </c>
     </row>
     <row r="15" ht="30" customHeight="1">
       <c r="A15" s="10" t="inlineStr">
@@ -24186,6 +24252,11 @@
           <t>images/track_04/a1_s04_seg13_boy.jpg</t>
         </is>
       </c>
+      <c r="L15" s="29" t="inlineStr">
+        <is>
+          <t>videos/T4/t4_seg_13.mp4</t>
+        </is>
+      </c>
     </row>
     <row r="16" ht="30" customHeight="1">
       <c r="A16" s="8" t="inlineStr">
@@ -24239,6 +24310,11 @@
           <t>images/track_04/a1_s04_seg14_boy.jpg</t>
         </is>
       </c>
+      <c r="L16" s="29" t="inlineStr">
+        <is>
+          <t>videos/T4/t4_seg_14.mp4</t>
+        </is>
+      </c>
     </row>
     <row r="17" ht="30" customHeight="1">
       <c r="A17" s="10" t="inlineStr">
@@ -24292,6 +24368,11 @@
           <t>images/track_04/a1_s04_seg15_boy.jpg</t>
         </is>
       </c>
+      <c r="L17" s="29" t="inlineStr">
+        <is>
+          <t>videos/T4/t4_seg_15.mp4</t>
+        </is>
+      </c>
     </row>
     <row r="18" ht="30" customHeight="1">
       <c r="A18" s="8" t="inlineStr">
@@ -24345,6 +24426,11 @@
           <t>images/track_04/a1_s04_seg16_boy.jpg</t>
         </is>
       </c>
+      <c r="L18" s="29" t="inlineStr">
+        <is>
+          <t>videos/T4/t4_seg_16.mp4</t>
+        </is>
+      </c>
     </row>
     <row r="19" ht="30" customHeight="1">
       <c r="A19" s="10" t="inlineStr">
@@ -24398,6 +24484,11 @@
           <t>images/track_04/a1_s04_seg17_boy.jpg</t>
         </is>
       </c>
+      <c r="L19" s="29" t="inlineStr">
+        <is>
+          <t>videos/T4/t4_seg_17.mp4</t>
+        </is>
+      </c>
     </row>
     <row r="20" ht="30" customHeight="1">
       <c r="A20" s="8" t="inlineStr">
@@ -24451,6 +24542,11 @@
           <t>images/track_04/a1_s04_seg18_boy.jpg</t>
         </is>
       </c>
+      <c r="L20" s="29" t="inlineStr">
+        <is>
+          <t>videos/T4/t4_seg_18.mp4</t>
+        </is>
+      </c>
     </row>
     <row r="21" ht="30" customHeight="1">
       <c r="A21" s="10" t="inlineStr">
@@ -24504,6 +24600,11 @@
           <t>images/track_04/a1_s04_seg19_boy.jpg</t>
         </is>
       </c>
+      <c r="L21" s="29" t="inlineStr">
+        <is>
+          <t>videos/T4/t4_seg_19.mp4</t>
+        </is>
+      </c>
     </row>
     <row r="22" ht="30" customHeight="1">
       <c r="A22" s="8" t="inlineStr">
@@ -24557,6 +24658,11 @@
           <t>images/track_04/a1_s04_seg20_boy.jpg</t>
         </is>
       </c>
+      <c r="L22" s="29" t="inlineStr">
+        <is>
+          <t>videos/T4/t4_seg_20.mp4</t>
+        </is>
+      </c>
     </row>
     <row r="23" ht="30" customHeight="1">
       <c r="A23" s="10" t="inlineStr">
@@ -24610,6 +24716,11 @@
           <t>images/track_04/a1_s04_seg21_boy.jpg</t>
         </is>
       </c>
+      <c r="L23" s="29" t="inlineStr">
+        <is>
+          <t>videos/T4/t4_seg_21.mp4</t>
+        </is>
+      </c>
     </row>
     <row r="24" ht="30" customHeight="1">
       <c r="A24" s="8" t="inlineStr">
@@ -24663,6 +24774,11 @@
           <t>images/track_04/a1_s04_seg22_boy.jpg</t>
         </is>
       </c>
+      <c r="L24" s="29" t="inlineStr">
+        <is>
+          <t>videos/T4/t4_seg_22.mp4</t>
+        </is>
+      </c>
     </row>
     <row r="25" ht="30" customHeight="1">
       <c r="A25" s="10" t="inlineStr">
@@ -24716,6 +24832,11 @@
           <t>images/track_04/a1_s04_seg23_boy.jpg</t>
         </is>
       </c>
+      <c r="L25" s="29" t="inlineStr">
+        <is>
+          <t>videos/T4/t4_seg_23.mp4</t>
+        </is>
+      </c>
     </row>
     <row r="26" ht="30" customHeight="1">
       <c r="A26" s="8" t="inlineStr">
@@ -24769,6 +24890,11 @@
           <t>images/track_04/a1_s04_seg24_boy.jpg</t>
         </is>
       </c>
+      <c r="L26" s="29" t="inlineStr">
+        <is>
+          <t>videos/T4/t4_seg_24.mp4</t>
+        </is>
+      </c>
     </row>
     <row r="27" ht="30" customHeight="1">
       <c r="A27" s="10" t="inlineStr">
@@ -24822,6 +24948,11 @@
           <t>images/track_04/a1_s04_seg25_boy.jpg</t>
         </is>
       </c>
+      <c r="L27" s="29" t="inlineStr">
+        <is>
+          <t>videos/T4/t4_seg_25.mp4</t>
+        </is>
+      </c>
     </row>
     <row r="28" ht="30" customHeight="1">
       <c r="A28" s="8" t="inlineStr">
@@ -24873,6 +25004,11 @@
       <c r="K28" s="20" t="inlineStr">
         <is>
           <t>images/track_04/a1_s04_seg26_boy.jpg</t>
+        </is>
+      </c>
+      <c r="L28" s="29" t="inlineStr">
+        <is>
+          <t>videos/T4/t4_seg_26.mp4</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
feat: integrate all 26 T5 animation videos for Track 05 (Clean Up Little Helpers)
</commit_message>
<xml_diff>
--- a/docs/Album1_Dance_Production_Spec.xlsx
+++ b/docs/Album1_Dance_Production_Spec.xlsx
@@ -25026,7 +25026,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:K28"/>
+  <dimension ref="A1:L28"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="18" customWidth="1" min="1" max="1"/>
@@ -25040,6 +25040,7 @@
     <col width="12" customWidth="1" min="9" max="9"/>
     <col width="55" customWidth="1" min="10" max="10"/>
     <col width="34" customWidth="1" min="11" max="11"/>
+    <col width="28" customWidth="1" min="12" max="12"/>
   </cols>
   <sheetData>
     <row r="1" ht="32" customHeight="1">
@@ -25105,6 +25106,11 @@
           <t>首張圖片路徑 (9:16 720p)</t>
         </is>
       </c>
+      <c r="L2" s="28" t="inlineStr">
+        <is>
+          <t>AI 影片動畫路徑 (T5 目錄)</t>
+        </is>
+      </c>
     </row>
     <row r="3" ht="30" customHeight="1">
       <c r="A3" s="10" t="inlineStr">
@@ -25158,6 +25164,11 @@
           <t>images/track_05/a1_s05_seg01_girl.jpg</t>
         </is>
       </c>
+      <c r="L3" s="29" t="inlineStr">
+        <is>
+          <t>videos/T5/t5_seg_01.mp4</t>
+        </is>
+      </c>
     </row>
     <row r="4" ht="30" customHeight="1">
       <c r="A4" s="8" t="inlineStr">
@@ -25211,6 +25222,11 @@
           <t>images/track_05/a1_s05_seg02_girl.jpg</t>
         </is>
       </c>
+      <c r="L4" s="29" t="inlineStr">
+        <is>
+          <t>videos/T5/t5_seg_02.mp4</t>
+        </is>
+      </c>
     </row>
     <row r="5" ht="30" customHeight="1">
       <c r="A5" s="10" t="inlineStr">
@@ -25264,6 +25280,11 @@
           <t>images/track_05/a1_s05_seg03_girl.jpg</t>
         </is>
       </c>
+      <c r="L5" s="29" t="inlineStr">
+        <is>
+          <t>videos/T5/t5_seg_03.mp4</t>
+        </is>
+      </c>
     </row>
     <row r="6" ht="30" customHeight="1">
       <c r="A6" s="8" t="inlineStr">
@@ -25317,6 +25338,11 @@
           <t>images/track_05/a1_s05_seg04_girl.jpg</t>
         </is>
       </c>
+      <c r="L6" s="29" t="inlineStr">
+        <is>
+          <t>videos/T5/t5_seg_04.mp4</t>
+        </is>
+      </c>
     </row>
     <row r="7" ht="30" customHeight="1">
       <c r="A7" s="10" t="inlineStr">
@@ -25370,6 +25396,11 @@
           <t>images/track_05/a1_s05_seg05_girl.jpg</t>
         </is>
       </c>
+      <c r="L7" s="29" t="inlineStr">
+        <is>
+          <t>videos/T5/t5_seg_05.mp4</t>
+        </is>
+      </c>
     </row>
     <row r="8" ht="30" customHeight="1">
       <c r="A8" s="8" t="inlineStr">
@@ -25423,6 +25454,11 @@
           <t>images/track_05/a1_s05_seg06_girl.jpg</t>
         </is>
       </c>
+      <c r="L8" s="29" t="inlineStr">
+        <is>
+          <t>videos/T5/t5_seg_06.mp4</t>
+        </is>
+      </c>
     </row>
     <row r="9" ht="30" customHeight="1">
       <c r="A9" s="10" t="inlineStr">
@@ -25476,6 +25512,11 @@
           <t>images/track_05/a1_s05_seg07_girl.jpg</t>
         </is>
       </c>
+      <c r="L9" s="29" t="inlineStr">
+        <is>
+          <t>videos/T5/t5_seg_07.mp4</t>
+        </is>
+      </c>
     </row>
     <row r="10" ht="30" customHeight="1">
       <c r="A10" s="8" t="inlineStr">
@@ -25529,6 +25570,11 @@
           <t>images/track_05/a1_s05_seg08_girl.jpg</t>
         </is>
       </c>
+      <c r="L10" s="29" t="inlineStr">
+        <is>
+          <t>videos/T5/t5_seg_08.mp4</t>
+        </is>
+      </c>
     </row>
     <row r="11" ht="30" customHeight="1">
       <c r="A11" s="10" t="inlineStr">
@@ -25582,6 +25628,11 @@
           <t>images/track_05/a1_s05_seg09_girl.jpg</t>
         </is>
       </c>
+      <c r="L11" s="29" t="inlineStr">
+        <is>
+          <t>videos/T5/t5_seg_09.mp4</t>
+        </is>
+      </c>
     </row>
     <row r="12" ht="30" customHeight="1">
       <c r="A12" s="8" t="inlineStr">
@@ -25635,6 +25686,11 @@
           <t>images/track_05/a1_s05_seg10_girl.jpg</t>
         </is>
       </c>
+      <c r="L12" s="29" t="inlineStr">
+        <is>
+          <t>videos/T5/t5_seg_10.mp4</t>
+        </is>
+      </c>
     </row>
     <row r="13" ht="30" customHeight="1">
       <c r="A13" s="10" t="inlineStr">
@@ -25688,6 +25744,11 @@
           <t>images/track_05/a1_s05_seg11_girl.jpg</t>
         </is>
       </c>
+      <c r="L13" s="29" t="inlineStr">
+        <is>
+          <t>videos/T5/t5_seg_11.mp4</t>
+        </is>
+      </c>
     </row>
     <row r="14" ht="30" customHeight="1">
       <c r="A14" s="8" t="inlineStr">
@@ -25741,6 +25802,11 @@
           <t>images/track_05/a1_s05_seg12_girl.jpg</t>
         </is>
       </c>
+      <c r="L14" s="29" t="inlineStr">
+        <is>
+          <t>videos/T5/t5_seg_12.mp4</t>
+        </is>
+      </c>
     </row>
     <row r="15" ht="30" customHeight="1">
       <c r="A15" s="10" t="inlineStr">
@@ -25794,6 +25860,11 @@
           <t>images/track_05/a1_s05_seg13_girl.jpg</t>
         </is>
       </c>
+      <c r="L15" s="29" t="inlineStr">
+        <is>
+          <t>videos/T5/t5_seg_13.mp4</t>
+        </is>
+      </c>
     </row>
     <row r="16" ht="30" customHeight="1">
       <c r="A16" s="8" t="inlineStr">
@@ -25847,6 +25918,11 @@
           <t>images/track_05/a1_s05_seg14_girl.jpg</t>
         </is>
       </c>
+      <c r="L16" s="29" t="inlineStr">
+        <is>
+          <t>videos/T5/t5_seg_14.mp4</t>
+        </is>
+      </c>
     </row>
     <row r="17" ht="30" customHeight="1">
       <c r="A17" s="10" t="inlineStr">
@@ -25900,6 +25976,11 @@
           <t>images/track_05/a1_s05_seg15_girl.jpg</t>
         </is>
       </c>
+      <c r="L17" s="29" t="inlineStr">
+        <is>
+          <t>videos/T5/t5_seg_15.mp4</t>
+        </is>
+      </c>
     </row>
     <row r="18" ht="30" customHeight="1">
       <c r="A18" s="8" t="inlineStr">
@@ -25953,6 +26034,11 @@
           <t>images/track_05/a1_s05_seg16_girl.jpg</t>
         </is>
       </c>
+      <c r="L18" s="29" t="inlineStr">
+        <is>
+          <t>videos/T5/t5_seg_16.mp4</t>
+        </is>
+      </c>
     </row>
     <row r="19" ht="30" customHeight="1">
       <c r="A19" s="10" t="inlineStr">
@@ -26006,6 +26092,11 @@
           <t>images/track_05/a1_s05_seg17_girl.jpg</t>
         </is>
       </c>
+      <c r="L19" s="29" t="inlineStr">
+        <is>
+          <t>videos/T5/t5_seg_17.mp4</t>
+        </is>
+      </c>
     </row>
     <row r="20" ht="30" customHeight="1">
       <c r="A20" s="8" t="inlineStr">
@@ -26059,6 +26150,11 @@
           <t>images/track_05/a1_s05_seg18_girl.jpg</t>
         </is>
       </c>
+      <c r="L20" s="29" t="inlineStr">
+        <is>
+          <t>videos/T5/t5_seg_18.mp4</t>
+        </is>
+      </c>
     </row>
     <row r="21" ht="30" customHeight="1">
       <c r="A21" s="10" t="inlineStr">
@@ -26112,6 +26208,11 @@
           <t>images/track_05/a1_s05_seg19_girl.jpg</t>
         </is>
       </c>
+      <c r="L21" s="29" t="inlineStr">
+        <is>
+          <t>videos/T5/t5_seg_19.mp4</t>
+        </is>
+      </c>
     </row>
     <row r="22" ht="30" customHeight="1">
       <c r="A22" s="8" t="inlineStr">
@@ -26165,6 +26266,11 @@
           <t>images/track_05/a1_s05_seg20_girl.jpg</t>
         </is>
       </c>
+      <c r="L22" s="29" t="inlineStr">
+        <is>
+          <t>videos/T5/t5_seg_20.mp4</t>
+        </is>
+      </c>
     </row>
     <row r="23" ht="30" customHeight="1">
       <c r="A23" s="10" t="inlineStr">
@@ -26218,6 +26324,11 @@
           <t>images/track_05/a1_s05_seg21_girl.jpg</t>
         </is>
       </c>
+      <c r="L23" s="29" t="inlineStr">
+        <is>
+          <t>videos/T5/t5_seg_21.mp4</t>
+        </is>
+      </c>
     </row>
     <row r="24" ht="30" customHeight="1">
       <c r="A24" s="8" t="inlineStr">
@@ -26271,6 +26382,11 @@
           <t>images/track_05/a1_s05_seg22_girl.jpg</t>
         </is>
       </c>
+      <c r="L24" s="29" t="inlineStr">
+        <is>
+          <t>videos/T5/t5_seg_22.mp4</t>
+        </is>
+      </c>
     </row>
     <row r="25" ht="30" customHeight="1">
       <c r="A25" s="10" t="inlineStr">
@@ -26324,6 +26440,11 @@
           <t>images/track_05/a1_s05_seg23_girl.jpg</t>
         </is>
       </c>
+      <c r="L25" s="29" t="inlineStr">
+        <is>
+          <t>videos/T5/t5_seg_23.mp4</t>
+        </is>
+      </c>
     </row>
     <row r="26" ht="30" customHeight="1">
       <c r="A26" s="8" t="inlineStr">
@@ -26377,6 +26498,11 @@
           <t>images/track_05/a1_s05_seg24_girl.jpg</t>
         </is>
       </c>
+      <c r="L26" s="29" t="inlineStr">
+        <is>
+          <t>videos/T5/t5_seg_24.mp4</t>
+        </is>
+      </c>
     </row>
     <row r="27" ht="30" customHeight="1">
       <c r="A27" s="10" t="inlineStr">
@@ -26430,6 +26556,11 @@
           <t>images/track_05/a1_s05_seg25_girl.jpg</t>
         </is>
       </c>
+      <c r="L27" s="29" t="inlineStr">
+        <is>
+          <t>videos/T5/t5_seg_25.mp4</t>
+        </is>
+      </c>
     </row>
     <row r="28" ht="30" customHeight="1">
       <c r="A28" s="8" t="inlineStr">
@@ -26481,6 +26612,11 @@
       <c r="K28" s="20" t="inlineStr">
         <is>
           <t>images/track_05/a1_s05_seg26_girl.jpg</t>
+        </is>
+      </c>
+      <c r="L28" s="29" t="inlineStr">
+        <is>
+          <t>videos/T5/t5_seg_26.mp4</t>
         </is>
       </c>
     </row>

</xml_diff>